<commit_message>
update data 14 okt
update data 14 okt
</commit_message>
<xml_diff>
--- a/Database/DAFTAR SP2D SATKER.xlsx
+++ b/Database/DAFTAR SP2D SATKER.xlsx
@@ -725,28 +725,37 @@
     <t>00363T/403829/2025</t>
   </si>
   <si>
+    <t xml:space="preserve"> 259991530041993</t>
+  </si>
+  <si>
+    <t>19-08-2025</t>
+  </si>
+  <si>
+    <t>00335T/403829/2025</t>
+  </si>
+  <si>
+    <t>11-08-2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan September 2025 untuk 50 Pegawai/125 Jiwa</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 259991530041992</t>
   </si>
   <si>
-    <t>19-08-2025</t>
-  </si>
-  <si>
     <t>00340T/403829/2025</t>
   </si>
   <si>
-    <t>11-08-2025</t>
-  </si>
-  <si>
     <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan September 2025 untuk 131 Pegawai/384 Jiwa</t>
   </si>
   <si>
-    <t xml:space="preserve"> 259991530041993</t>
-  </si>
-  <si>
-    <t>00335T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan September 2025 untuk 50 Pegawai/125 Jiwa</t>
+    <t xml:space="preserve"> 259991530041994</t>
+  </si>
+  <si>
+    <t>00337T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan September 2025 untuk 35 Pegawai/101 Jiwa</t>
   </si>
   <si>
     <t xml:space="preserve"> 259991530041991</t>
@@ -761,15 +770,6 @@
     <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan September 2025 untuk 37 Pegawai/103 Jiwa</t>
   </si>
   <si>
-    <t xml:space="preserve"> 259991530041994</t>
-  </si>
-  <si>
-    <t>00337T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan September 2025 untuk 35 Pegawai/101 Jiwa</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 259991525018157</t>
   </si>
   <si>
@@ -779,6 +779,24 @@
     <t>Pembayaran Belanja Pegawai berupa Gaji Induk bulan September 2025 untuk 4 Pegawai/16 Jiwa</t>
   </si>
   <si>
+    <t xml:space="preserve"> 259991531008984</t>
+  </si>
+  <si>
+    <t>00339T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan September 2025 untuk 170 Pegawai /532 Jiwa</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 259991531008986</t>
+  </si>
+  <si>
+    <t>00338T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan September 2025 untuk 23 Pegawai/52 jiwa</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 259991531008985</t>
   </si>
   <si>
@@ -788,22 +806,13 @@
     <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan September 2025  untuk 63 Pegawai/181 jiwa</t>
   </si>
   <si>
-    <t xml:space="preserve"> 259991531008984</t>
-  </si>
-  <si>
-    <t>00339T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan September 2025 untuk 170 Pegawai /532 Jiwa</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 259991531008986</t>
-  </si>
-  <si>
-    <t>00338T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan September 2025 untuk 23 Pegawai/52 jiwa</t>
+    <t xml:space="preserve"> 259991310471405</t>
+  </si>
+  <si>
+    <t>00359T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran tunjangan kinerja bulan Juli tahun 2025 untuk 50 Pegawai</t>
   </si>
   <si>
     <t xml:space="preserve"> 259991310471406</t>
@@ -824,15 +833,6 @@
     <t>Pembayaran tunjangan kinerja bulan JULI tahun 2025 untuk 134 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 259991310471405</t>
-  </si>
-  <si>
-    <t>00359T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran tunjangan kinerja bulan Juli tahun 2025 untuk 50 Pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 259991330150985</t>
   </si>
   <si>
@@ -1121,48 +1121,48 @@
     <t>Pembayaran Belanja Barang Berupa Honor PPNPN Bulan Juli Tahun 2025 untuk 91 Pegawai.Sesuai Sk No 9 Tahun 2025 Tanggal 6 Januari 2025</t>
   </si>
   <si>
+    <t xml:space="preserve"> 259991530020754</t>
+  </si>
+  <si>
+    <t>17-07-2025</t>
+  </si>
+  <si>
+    <t>00309T/403829/2025</t>
+  </si>
+  <si>
+    <t>09-07-2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan Agustus 2025 untuk 132 Pegawai/388 Jiwa</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 259991530020753</t>
+  </si>
+  <si>
+    <t>00308T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji induk Bulan Agustus 2025 untuk 38 Pegawai/107 Jiwa</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 259991530020756</t>
+  </si>
+  <si>
+    <t>00301T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK bulan Agustus 2025 untuk 35 Pegawai/101 Jiwa</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 259991530020755</t>
   </si>
   <si>
-    <t>17-07-2025</t>
-  </si>
-  <si>
     <t>00299T/403829/2025</t>
   </si>
   <si>
-    <t>09-07-2025</t>
-  </si>
-  <si>
     <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan Agustus 2025 untuk 50 Pegawai/124 jiwa</t>
   </si>
   <si>
-    <t xml:space="preserve"> 259991530020754</t>
-  </si>
-  <si>
-    <t>00309T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan Agustus 2025 untuk 132 Pegawai/388 Jiwa</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 259991530020756</t>
-  </si>
-  <si>
-    <t>00301T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK bulan Agustus 2025 untuk 35 Pegawai/101 Jiwa</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 259991530020753</t>
-  </si>
-  <si>
-    <t>00308T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji induk Bulan Agustus 2025 untuk 38 Pegawai/107 Jiwa</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 259991531004439</t>
   </si>
   <si>
@@ -1205,25 +1205,43 @@
     <t>Pembayaran Belanja Barang sesuai SPD No. 0023-0037/BRPBATPP/KP.440/VII/2025 Tanggal 19 April 2025 sd 07 Juli 2025</t>
   </si>
   <si>
+    <t xml:space="preserve"> 259991310239039</t>
+  </si>
+  <si>
+    <t>11-07-2025</t>
+  </si>
+  <si>
+    <t>00318T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran tunjangan kinerja bulan Juni tahun 2025 untuk 35 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 259991310239038</t>
   </si>
   <si>
-    <t>11-07-2025</t>
-  </si>
-  <si>
     <t>00315T/403829/2025</t>
   </si>
   <si>
     <t>Pembayaran tunjangan kinerja bulan Juni tahun 2025 untuk 134 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 259991310239039</t>
-  </si>
-  <si>
-    <t>00318T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran tunjangan kinerja bulan Juni tahun 2025 untuk 35 Pegawai</t>
+    <t xml:space="preserve"> 259991330071755</t>
+  </si>
+  <si>
+    <t>00319T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran tunjangan kinerja bulan Juni tahun 2025 untuk 23 Pegawai</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 259991330071754</t>
+  </si>
+  <si>
+    <t>00317T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran tunjangan kinerja bulan Juni tahun 2025 untuk 63 Pegawai</t>
   </si>
   <si>
     <t xml:space="preserve"> 259991330071753</t>
@@ -1235,24 +1253,6 @@
     <t>Pembayaran tunjangan kinerja bulan Juni tahun 2025 untuk 174 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 259991330071754</t>
-  </si>
-  <si>
-    <t>00317T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran tunjangan kinerja bulan Juni tahun 2025 untuk 63 Pegawai</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 259991330071755</t>
-  </si>
-  <si>
-    <t>00319T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran tunjangan kinerja bulan Juni tahun 2025 untuk 23 Pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 259991310238647</t>
   </si>
   <si>
@@ -1262,18 +1262,36 @@
     <t>Pembayaran tunjangan kinerja bulan Juni tahun 2025 untuk 50 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 259991310222993</t>
+  </si>
+  <si>
+    <t>10-07-2025</t>
+  </si>
+  <si>
+    <t>00305T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Uang Makan PPPK Bulan Juni 2025 untuk 34 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 259991310222991</t>
   </si>
   <si>
-    <t>10-07-2025</t>
-  </si>
-  <si>
     <t>00314T/403829/2025</t>
   </si>
   <si>
     <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Juni 2025 untuk 37 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 259991310222992</t>
+  </si>
+  <si>
+    <t>00304T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Uang Makan PPPK Bulan Juni 2025 untuk 50 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 259991310222990</t>
   </si>
   <si>
@@ -1283,24 +1301,6 @@
     <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Juni 2025 untuk 132 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 259991310222992</t>
-  </si>
-  <si>
-    <t>00304T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Uang Makan PPPK Bulan Juni 2025 untuk 50 Pegawai</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 259991310222993</t>
-  </si>
-  <si>
-    <t>00305T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Uang Makan PPPK Bulan Juni 2025 untuk 34 Pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 259991305050216</t>
   </si>
   <si>
@@ -1310,6 +1310,15 @@
     <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Juni 2025 untuk 2 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 259991330066248</t>
+  </si>
+  <si>
+    <t>00307T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Uang Makan PPPK Bulan Juni 2025  untuk 22 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 259991330066246</t>
   </si>
   <si>
@@ -1328,15 +1337,6 @@
     <t>Pembayaran Belanja Pegawai berupa Uang Makan PPPK Bulan Juni 2025  untuk 62 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 259991330066248</t>
-  </si>
-  <si>
-    <t>00307T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Uang Makan PPPK Bulan Juni 2025  untuk 22 Pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 259991310213072</t>
   </si>
   <si>
@@ -1403,27 +1403,27 @@
     <t>Pembayaran Tukin ke-13 Tahun 2025 Untuk 1 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 259991330045564</t>
+  </si>
+  <si>
+    <t>00291T/403829/2025</t>
+  </si>
+  <si>
+    <t>01-07-2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Mei 2025 untuk 1 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 259991330045565</t>
   </si>
   <si>
     <t>00292T/403829/2025</t>
   </si>
   <si>
-    <t>01-07-2025</t>
-  </si>
-  <si>
     <t>Pembayaran tunjangan kinerja  bulan Mei tahun 2025 untuk 1 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 259991330045564</t>
-  </si>
-  <si>
-    <t>00291T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Mei 2025 untuk 1 Pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 259991310150031</t>
   </si>
   <si>
@@ -1454,21 +1454,39 @@
     <t>00288T/403829/2025</t>
   </si>
   <si>
+    <t xml:space="preserve"> 259991530018166</t>
+  </si>
+  <si>
+    <t>25-06-2025</t>
+  </si>
+  <si>
+    <t>00270T/403829/2025</t>
+  </si>
+  <si>
+    <t>11-06-2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan Juli 2025 untuk 39 Pegawai/111 Jiwa</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 259991530018167</t>
   </si>
   <si>
-    <t>25-06-2025</t>
-  </si>
-  <si>
     <t>00271T/403829/2025</t>
   </si>
   <si>
-    <t>11-06-2025</t>
-  </si>
-  <si>
     <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan Juli 2025 untuk 135 Pegawai/396 jiwa</t>
   </si>
   <si>
+    <t xml:space="preserve"> 259991530018169</t>
+  </si>
+  <si>
+    <t>00267T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan Juli 2025 untuk 35 Pegawai/101 Jiwa</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 259991530018168</t>
   </si>
   <si>
@@ -1478,24 +1496,6 @@
     <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan Juli 2025 untuk 50 Pegawai/124 Jiwa</t>
   </si>
   <si>
-    <t xml:space="preserve"> 259991530018169</t>
-  </si>
-  <si>
-    <t>00267T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan Juli 2025 untuk 35 Pegawai/101 Jiwa</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 259991530018166</t>
-  </si>
-  <si>
-    <t>00270T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan Juli 2025 untuk 39 Pegawai/111 Jiwa</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 259991310116799</t>
   </si>
   <si>
@@ -1520,6 +1520,15 @@
     <t>Pembayaran tunjangan kinerja bulan Juli tahun 2025 untuk 2 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 259991530011368</t>
+  </si>
+  <si>
+    <t>00286T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Barang Berupa Honor PPNPN Bulan Juni Tahun 2025 untuk 103 Pegawai.Sesuai Sk No.9 Tahun 2025 Tanggal 6 Januari 2025</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 259991530011369</t>
   </si>
   <si>
@@ -1529,13 +1538,34 @@
     <t>Pembayaran Belanja Barang Berupa Honor PPNPN Bulan Juni Tahun 2025 untuk 16 Pegawai.Sesuai Sk No. B.4/BRPBATPP/KP.340/I/2025 Tanggal 2 Januari 2025</t>
   </si>
   <si>
-    <t xml:space="preserve"> 259991530011368</t>
-  </si>
-  <si>
-    <t>00286T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Barang Berupa Honor PPNPN Bulan Juni Tahun 2025 untuk 103 Pegawai.Sesuai Sk No.9 Tahun 2025 Tanggal 6 Januari 2025</t>
+    <t xml:space="preserve"> 259991531001948</t>
+  </si>
+  <si>
+    <t>00266T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan Juli 2025 untuk 63 Pegawai/181 Jiwa</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 259991531001947</t>
+  </si>
+  <si>
+    <t>00282T/403829/2025</t>
+  </si>
+  <si>
+    <t>19-06-2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan Juli 2025 untuk 173 Pegawai/538 Jiwa</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 259991531001949</t>
+  </si>
+  <si>
+    <t>00268T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan Juli 2025 untuk 23 Pegawai/52 Jiwa</t>
   </si>
   <si>
     <t xml:space="preserve"> 259991531001971</t>
@@ -1547,36 +1577,6 @@
     <t>Pembayaran Belanja Barang Berupa Honor PPNPN Bulan Juni Tahun 2025 untuk 91 Pegawai.Sesuai Sk No.9 Tahun 2025 Tanggal 6 Januari 2025</t>
   </si>
   <si>
-    <t xml:space="preserve"> 259991531001949</t>
-  </si>
-  <si>
-    <t>00268T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan Juli 2025 untuk 23 Pegawai/52 Jiwa</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 259991531001947</t>
-  </si>
-  <si>
-    <t>00282T/403829/2025</t>
-  </si>
-  <si>
-    <t>19-06-2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan Juli 2025 untuk 173 Pegawai/538 Jiwa</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 259991531001948</t>
-  </si>
-  <si>
-    <t>00266T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan Juli 2025 untuk 63 Pegawai/181 Jiwa</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 259991525004591</t>
   </si>
   <si>
@@ -1598,15 +1598,24 @@
     <t>Penjualan Belanja Pegawai berupa Kekurangan Gaji Bulan Januari 2025 untuk 1 Pegawai/3 Jiwa</t>
   </si>
   <si>
+    <t xml:space="preserve"> 259991310059124</t>
+  </si>
+  <si>
+    <t>13-06-2025</t>
+  </si>
+  <si>
+    <t>16-06-2025</t>
+  </si>
+  <si>
+    <t>00275T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran tunjangan kinerja  bulan Mei tahun 2025 untuk 137 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 259991310059125</t>
   </si>
   <si>
-    <t>13-06-2025</t>
-  </si>
-  <si>
-    <t>16-06-2025</t>
-  </si>
-  <si>
     <t>00277T/403829/2025</t>
   </si>
   <si>
@@ -1622,13 +1631,22 @@
     <t>Pembayaran tunjangan kinerja bulan Mei tahun 2025 untuk 35 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 259991310059124</t>
-  </si>
-  <si>
-    <t>00275T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran tunjangan kinerja  bulan Mei tahun 2025 untuk 137 Pegawai</t>
+    <t xml:space="preserve"> 259991330013160</t>
+  </si>
+  <si>
+    <t>00276T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran tunjangan kinerja bulan Mei tahun 2025 untuk 173 Pegawai</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 259991330013162</t>
+  </si>
+  <si>
+    <t>00279T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran tunjangan kinerja bulan Mei tahun 2025 untuk 23 Pegawai</t>
   </si>
   <si>
     <t xml:space="preserve"> 259991330013161</t>
@@ -1640,24 +1658,6 @@
     <t>Pembayaran tunjangan kinerja bulan Mei tahun 2025 untuk 63 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 259991330013162</t>
-  </si>
-  <si>
-    <t>00279T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran tunjangan kinerja bulan Mei tahun 2025 untuk 23 Pegawai</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 259991330013160</t>
-  </si>
-  <si>
-    <t>00276T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran tunjangan kinerja bulan Mei tahun 2025 untuk 173 Pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 259991320016562</t>
   </si>
   <si>
@@ -1670,18 +1670,18 @@
     <t>Pembayaran Belanja Barang berupa Tagihan Internet Bulan Mei 2025 idpel No.GO18A106 An Balai Riset Perikanan Budidaya Air Tawar dan Penyuluhan Perikanan</t>
   </si>
   <si>
+    <t xml:space="preserve"> 259991310050294</t>
+  </si>
+  <si>
+    <t>00273T/403829/2025</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 259991310050295</t>
   </si>
   <si>
     <t>00274T/403829/2025</t>
   </si>
   <si>
-    <t xml:space="preserve"> 259991310050294</t>
-  </si>
-  <si>
-    <t>00273T/403829/2025</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 259991310039873</t>
   </si>
   <si>
@@ -1721,43 +1721,52 @@
     <t>Pembayaran Belanja Pegawai berupa Kekurangan Gaji Bulan April 2025 sd Mei 2025 untuk 11 Pegawai/41 Jiwa</t>
   </si>
   <si>
+    <t xml:space="preserve"> 259991310036822</t>
+  </si>
+  <si>
+    <t>00256T/403829/2025</t>
+  </si>
+  <si>
+    <t>05-06-2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Mei 2025 untuk 38 Jiwa</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 259991310036825</t>
+  </si>
+  <si>
+    <t>00257T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Mei 2025 untuk 136 jiwa</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 259991310036824</t>
+  </si>
+  <si>
+    <t>00254T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Kekurangan Gaji bulan Mei 2025 untuk 2 pegawai/ 4 Jiwa</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 259991310036823</t>
   </si>
   <si>
     <t>00252T/403829/2025</t>
   </si>
   <si>
-    <t>05-06-2025</t>
-  </si>
-  <si>
     <t>Pembayaran Belanja Pegawai berupa Kekurangan Gaji Bulan April 2025 sd Mei 2025 untuk 2 Pegawai/5 Jiwa</t>
   </si>
   <si>
-    <t xml:space="preserve"> 259991310036822</t>
-  </si>
-  <si>
-    <t>00256T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Mei 2025 untuk 38 Jiwa</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 259991310036825</t>
-  </si>
-  <si>
-    <t>00257T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Mei 2025 untuk 136 jiwa</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 259991310036824</t>
-  </si>
-  <si>
-    <t>00254T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Kekurangan Gaji bulan Mei 2025 untuk 2 pegawai/ 4 Jiwa</t>
+    <t xml:space="preserve"> 259991330008176</t>
+  </si>
+  <si>
+    <t>00259T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Mei 2025 untuk 171 Pegawai</t>
   </si>
   <si>
     <t xml:space="preserve"> 259991330008175</t>
@@ -1769,15 +1778,6 @@
     <t>Pembayaran Belanja Pegawai berupa Kekurangan Gaji Bulan Juni 2025 untuk 1 Pegawai/1 Jiwa</t>
   </si>
   <si>
-    <t xml:space="preserve"> 259991330008176</t>
-  </si>
-  <si>
-    <t>00259T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Mei 2025 untuk 171 Pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 259991330008177</t>
   </si>
   <si>
@@ -1796,6 +1796,15 @@
     <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Mei 2025 untuk 2 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 259991310033061</t>
+  </si>
+  <si>
+    <t>00250T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Uang Makan PPPK Bulan Mei 2025 untuk 34 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 259991310033060</t>
   </si>
   <si>
@@ -1805,15 +1814,6 @@
     <t>Pembayaran Belanja Pegawai berupa Uang Makan PPPK Bulan Mei 2025 untuk 50 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 259991310033061</t>
-  </si>
-  <si>
-    <t>00250T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Uang Makan PPPK Bulan Mei 2025 untuk 34 Pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 259991330007277</t>
   </si>
   <si>
@@ -1913,6 +1913,24 @@
     <t>Pembayaran Tukin ke-13 Tahun 2025 Untuk 35 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231303002007</t>
+  </si>
+  <si>
+    <t>00240T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Tukin ke-13 Tahun 2025 Untuk 63 Pegawai</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 250231303002006</t>
+  </si>
+  <si>
+    <t>00238T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Tukin ke-13 Tahun 2025 Untuk 173 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231303002008</t>
   </si>
   <si>
@@ -1922,24 +1940,6 @@
     <t>Pembayaran Tukin ke-13 Tahun 2025 Untuk 23 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231303002007</t>
-  </si>
-  <si>
-    <t>00240T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Tukin ke-13 Tahun 2025 Untuk 63 Pegawai</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 250231303002006</t>
-  </si>
-  <si>
-    <t>00238T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Tukin ke-13 Tahun 2025 Untuk 173 Pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231305000975</t>
   </si>
   <si>
@@ -1952,12 +1952,24 @@
     <t>Pembayaran Tukin ke-13 Tahun 2025 Untuk 2 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231501001413</t>
+  </si>
+  <si>
+    <t>26-05-2025</t>
+  </si>
+  <si>
+    <t>00232T/403829/2025</t>
+  </si>
+  <si>
+    <t>SPM Gaji 13 PPPK</t>
+  </si>
+  <si>
+    <t>Pembayaran Gaji ke-13 Tahun 2025 Untuk 50 PPPK.</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231501001439</t>
   </si>
   <si>
-    <t>26-05-2025</t>
-  </si>
-  <si>
     <t>00228T/403829/2025</t>
   </si>
   <si>
@@ -1970,21 +1982,9 @@
     <t>00234T/403829/2025</t>
   </si>
   <si>
-    <t>SPM Gaji 13 PPPK</t>
-  </si>
-  <si>
     <t>Pembayaran Gaji ke-13 Tahun 2025 Untuk 35 PPPK.</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231501001413</t>
-  </si>
-  <si>
-    <t>00232T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Gaji ke-13 Tahun 2025 Untuk 50 PPPK.</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231507000406</t>
   </si>
   <si>
@@ -1994,6 +1994,24 @@
     <t>Pembayaran Gaji ke-13 Tahun 2025 Untuk 2 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231503000383</t>
+  </si>
+  <si>
+    <t>00233T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Gaji ke-13 Tahun 2025 Untuk 63 PPPK.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 250231503000382</t>
+  </si>
+  <si>
+    <t>00229T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Gaji ke-13 Tahun 2025 Untuk 173 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231503000384</t>
   </si>
   <si>
@@ -2003,24 +2021,6 @@
     <t>Pembayaran Gaji ke-13 Tahun 2025 Untuk 23 PPPK.</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231503000382</t>
-  </si>
-  <si>
-    <t>00229T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Gaji ke-13 Tahun 2025 Untuk 173 Pegawai</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 250231503000383</t>
-  </si>
-  <si>
-    <t>00233T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Gaji ke-13 Tahun 2025 Untuk 63 PPPK.</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231305000959</t>
   </si>
   <si>
@@ -2072,30 +2072,30 @@
     <t>Pembayaran Belanja Barang Berupa Honor PPNPN Bulan Mei Tahun 2025 untuk 91 Pegawai.sesuai Sk No.9 Tahun 2025 Tanggal 6 Januari 2025</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231503000351</t>
+  </si>
+  <si>
+    <t>21-05-2025</t>
+  </si>
+  <si>
+    <t>00202T/403829/2025</t>
+  </si>
+  <si>
+    <t>08-05-2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji induk PPPK Bulan Juni 2025 untuk 63 Pegawai/181 Jiwa</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231503000352</t>
   </si>
   <si>
-    <t>21-05-2025</t>
-  </si>
-  <si>
     <t>00204T/403829/2025</t>
   </si>
   <si>
-    <t>08-05-2025</t>
-  </si>
-  <si>
     <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan Juni 2025 untuk 23 Pegawai/52 Jiwa</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231503000351</t>
-  </si>
-  <si>
-    <t>00202T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji induk PPPK Bulan Juni 2025 untuk 63 Pegawai/181 Jiwa</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231503000350</t>
   </si>
   <si>
@@ -2117,6 +2117,33 @@
     <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan Juni 2025 untuk 2 Pegawai/8 jiwa</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231501001202</t>
+  </si>
+  <si>
+    <t>00206T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan Juni 2025 untuk 135 Pegawai/ 396 Jiwa</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 250231501001208</t>
+  </si>
+  <si>
+    <t>00201T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan Juni 2025 untuk 50 Pegawai/124 Jiwa</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 250231501001201</t>
+  </si>
+  <si>
+    <t>00205T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa  Gaji Induk Bulan Juni 2025 untuk 39 Pegawai/111 Jiwa</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231501001209</t>
   </si>
   <si>
@@ -2126,54 +2153,27 @@
     <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan Juni 2025 untuk 35 Pegawai/101 Jiwa</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231501001201</t>
-  </si>
-  <si>
-    <t>00205T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa  Gaji Induk Bulan Juni 2025 untuk 39 Pegawai/111 Jiwa</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 250231501001208</t>
-  </si>
-  <si>
-    <t>00201T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan Juni 2025 untuk 50 Pegawai/124 Jiwa</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 250231501001202</t>
-  </si>
-  <si>
-    <t>00206T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan Juni 2025 untuk 135 Pegawai/ 396 Jiwa</t>
+    <t xml:space="preserve"> 250231303001771</t>
+  </si>
+  <si>
+    <t>20-05-2025</t>
+  </si>
+  <si>
+    <t>00222T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran tunjangan kinerja bulan April tahun 2025 untuk 63 Pegawai</t>
   </si>
   <si>
     <t xml:space="preserve"> 250231303001770</t>
   </si>
   <si>
-    <t>20-05-2025</t>
-  </si>
-  <si>
     <t>00219T/403829/2025</t>
   </si>
   <si>
     <t>Pembayaran Belanja Pegawai Berupa Uang Makan PPPK Bulan April 2025 untuk 63 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231303001771</t>
-  </si>
-  <si>
-    <t>00222T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran tunjangan kinerja bulan April tahun 2025 untuk 63 Pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231303001766</t>
   </si>
   <si>
@@ -2246,6 +2246,24 @@
     <t>Pembayaran tunjangan kinerja bulan April tahun 2025 untuk 173 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231301005718</t>
+  </si>
+  <si>
+    <t>00213T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran tunjangan kinerja bulan April tahun 2025 untuk 36 Pegawai</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 250231301005716</t>
+  </si>
+  <si>
+    <t>00211T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan April 2025  untuk 135 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231301005717</t>
   </si>
   <si>
@@ -2255,39 +2273,21 @@
     <t>Pembayaran tunjangan kinerja bulan April tahun 2025 untuk 50 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231301005718</t>
-  </si>
-  <si>
-    <t>00213T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran tunjangan kinerja bulan April tahun 2025 untuk 36 Pegawai</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 250231301005716</t>
-  </si>
-  <si>
-    <t>00211T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan April 2025  untuk 135 Pegawai</t>
+    <t xml:space="preserve"> 250231301005582</t>
+  </si>
+  <si>
+    <t>14-05-2025</t>
+  </si>
+  <si>
+    <t>00210T/403829/2025</t>
   </si>
   <si>
     <t xml:space="preserve"> 250231301005583</t>
   </si>
   <si>
-    <t>14-05-2025</t>
-  </si>
-  <si>
     <t>00209T/403829/2025</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231301005582</t>
-  </si>
-  <si>
-    <t>00210T/403829/2025</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231302005378</t>
   </si>
   <si>
@@ -2345,27 +2345,27 @@
     <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan April 2025 untuk 38 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231302005132</t>
+  </si>
+  <si>
+    <t>06-05-2025</t>
+  </si>
+  <si>
+    <t>00189T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Barang berupa Tagihan PDAM Bulan April 2025 Idpel No. 1249-1046 An. Lemb Perikanan Darat</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231302005131</t>
   </si>
   <si>
-    <t>06-05-2025</t>
-  </si>
-  <si>
     <t>00194T/403829/2025</t>
   </si>
   <si>
     <t>Pembayaran Belanja Barang sesuai Kwitansi No.02/SAj/KW/IV/2025 Tanggal 8 April 2025 berupa pemeliharaan CCTV Instalasi depok</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231302005132</t>
-  </si>
-  <si>
-    <t>00189T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Barang berupa Tagihan PDAM Bulan April 2025 Idpel No. 1249-1046 An. Lemb Perikanan Darat</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231301005196</t>
   </si>
   <si>
@@ -2498,27 +2498,36 @@
     <t>Pembayaran Belanja Barang Berupa Honor PPNPN Bulan April Tahun 2025 untuk 91 Pegawai.sesuai Sk No.9 Tahun 2025 tanggal 6 januari 2025</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231501001051</t>
+  </si>
+  <si>
+    <t>00158T/403829/2025</t>
+  </si>
+  <si>
+    <t>10-04-2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan Mei 2025 untuk 39 Pegawai/111 Jiwa</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 250231501001059</t>
+  </si>
+  <si>
+    <t>00153T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan Mei 2025 untuk 36 Pegawai/105 Jiwa</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231501001057</t>
   </si>
   <si>
     <t>00156T/403829/2025</t>
   </si>
   <si>
-    <t>10-04-2025</t>
-  </si>
-  <si>
     <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan Mei 2025 untuk 50 Pegawai/124 Jiwa</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231501001059</t>
-  </si>
-  <si>
-    <t>00153T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan Mei 2025 untuk 36 Pegawai/105 Jiwa</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231501001058</t>
   </si>
   <si>
@@ -2528,15 +2537,6 @@
     <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan Mei 2025 untuk 137 Pegawai/401 Jiwa</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231501001051</t>
-  </si>
-  <si>
-    <t>00158T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan Mei 2025 untuk 39 Pegawai/111 Jiwa</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231507000303</t>
   </si>
   <si>
@@ -2585,6 +2585,15 @@
     <t>Pembayaran tunjangan kinerja bulan Maret tahun 2025 untuk 63 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231301004024</t>
+  </si>
+  <si>
+    <t>00176T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran tunjangan kinerja bulan Maret tahun 2025 untuk 138 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231301004026</t>
   </si>
   <si>
@@ -2594,15 +2603,6 @@
     <t>Pembayaran tunjangan kinerja bulan Maret tahun 2025 untuk 36 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231301004024</t>
-  </si>
-  <si>
-    <t>00176T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran tunjangan kinerja bulan Maret tahun 2025 untuk 138 Pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231301004025</t>
   </si>
   <si>
@@ -2612,6 +2612,15 @@
     <t>Pembayaran tunjangan kinerja bulan Maret tahun 2025 untuk 50 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231303001235</t>
+  </si>
+  <si>
+    <t>00177T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran tunjangan kinerja bulan Maret tahun 2025 untuk 175 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231303001236</t>
   </si>
   <si>
@@ -2621,15 +2630,6 @@
     <t>Pembayaran tunjangan kinerja bulan Maret tahun 2025 untuk 23 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231303001235</t>
-  </si>
-  <si>
-    <t>00177T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran tunjangan kinerja bulan Maret tahun 2025 untuk 175 Pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231302003921</t>
   </si>
   <si>
@@ -2699,6 +2699,33 @@
     <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Maret 2025 untuk 2 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231301003745</t>
+  </si>
+  <si>
+    <t>00168T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Maret 2025 untuk 136 Pegawai</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 250231301003744</t>
+  </si>
+  <si>
+    <t>00163T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Uang Makan PPPK Bulan Maret 2025 untuk 49 Pegawai</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 250231301003746</t>
+  </si>
+  <si>
+    <t>00162T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Uang Makan PPPK Bulan Maret 2025 untuk 36 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231301003743</t>
   </si>
   <si>
@@ -2708,33 +2735,6 @@
     <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Maret 2025 untuk 38 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231301003744</t>
-  </si>
-  <si>
-    <t>00163T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Uang Makan PPPK Bulan Maret 2025 untuk 49 Pegawai</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 250231301003746</t>
-  </si>
-  <si>
-    <t>00162T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Uang Makan PPPK Bulan Maret 2025 untuk 36 Pegawai</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 250231301003745</t>
-  </si>
-  <si>
-    <t>00168T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Maret 2025 untuk 136 Pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231303001158</t>
   </si>
   <si>
@@ -2846,6 +2846,24 @@
     <t>Pembayaran tunjangan kinerja bulan April tahun 2025 untuk 39 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231501000906</t>
+  </si>
+  <si>
+    <t>00146T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Barang Berupa Honor PPNPN Bulan Maret Tahun 2025 untuk 1 Pegawai.sesuai SK No. 9 Tahun 2025 tanggal 6 Januari 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 250231501000908</t>
+  </si>
+  <si>
+    <t>00135T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Barang Berupa Honor PPNPN Bulan Maret Tahun 2025 untuk 16 Pegawai.sesuai Sk No.B.4/BRPBATPP/KP.340/I/2025 Tanggal 2 Januari 2025</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231501000907</t>
   </si>
   <si>
@@ -2855,24 +2873,6 @@
     <t>Pembayaran Belanja Barang Berupa Honor PPNPN Bulan Maret Tahun 2025 untuk 102 Pegawai.Sesuai SK No. 9 Tahun 2025 Tanggal 6 Januari 2025</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231501000908</t>
-  </si>
-  <si>
-    <t>00135T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Barang Berupa Honor PPNPN Bulan Maret Tahun 2025 untuk 16 Pegawai.sesuai Sk No.B.4/BRPBATPP/KP.340/I/2025 Tanggal 2 Januari 2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 250231501000906</t>
-  </si>
-  <si>
-    <t>00146T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Barang Berupa Honor PPNPN Bulan Maret Tahun 2025 untuk 1 Pegawai.sesuai SK No. 9 Tahun 2025 tanggal 6 Januari 2025</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231503000261</t>
   </si>
   <si>
@@ -2882,45 +2882,45 @@
     <t>Pembayaran Belanja Barang Berupa Honor PPNPN Bulan Maret Tahun 2025 untuk 91 Pegawai.Sesuai Sk No.9 tahun 2025 Tanggal 6 Januari 2025</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231501000781</t>
+  </si>
+  <si>
+    <t>00092T/403829/2025</t>
+  </si>
+  <si>
+    <t>11-03-2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan April 2025 untuk 50 Pegawai/124 Jiwa</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 250231501000767</t>
+  </si>
+  <si>
+    <t>00094T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan April 2025 untuk 36 Pegawai/106 Jiwa</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 250231501000766</t>
+  </si>
+  <si>
+    <t>00089T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan April 2025 untuk 137 Pegawai/403 Jiwa</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231501000765</t>
   </si>
   <si>
     <t>00090T/403829/2025</t>
   </si>
   <si>
-    <t>11-03-2025</t>
-  </si>
-  <si>
     <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan April 2025 untuk 39 Pegawai/ 111 Jiwa</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231501000766</t>
-  </si>
-  <si>
-    <t>00089T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan April 2025 untuk 137 Pegawai/403 Jiwa</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 250231501000781</t>
-  </si>
-  <si>
-    <t>00092T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan April 2025 untuk 50 Pegawai/124 Jiwa</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 250231501000767</t>
-  </si>
-  <si>
-    <t>00094T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan April 2025 untuk 36 Pegawai/106 Jiwa</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231507000254</t>
   </si>
   <si>
@@ -3086,6 +3086,15 @@
     <t>Pembayaran THR Tunkin Tahun 2025 Untuk 2 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231303000889</t>
+  </si>
+  <si>
+    <t>00129T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Uang Makan februari 2025 untuk 1 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231303000888</t>
   </si>
   <si>
@@ -3104,15 +3113,6 @@
     <t>Pembayaran THR Tunkin Tahun 2025 Untuk 63 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231303000889</t>
-  </si>
-  <si>
-    <t>00129T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Uang Makan februari 2025 untuk 1 Pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231301002724</t>
   </si>
   <si>
@@ -3158,6 +3158,15 @@
     <t>Pembayaran THR Tahun 2025 Untuk 2 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231503000156</t>
+  </si>
+  <si>
+    <t>00117T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran THR Tahun 2025 Untuk 177 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231503000157</t>
   </si>
   <si>
@@ -3167,13 +3176,22 @@
     <t>Pembayaran THR Tahun 2025 Untuk 63 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231503000156</t>
-  </si>
-  <si>
-    <t>00117T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran THR Tahun 2025 Untuk 177 Pegawai</t>
+    <t xml:space="preserve"> 250231501000527</t>
+  </si>
+  <si>
+    <t>00114T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran THR Tahun 2025 Untuk 1 Pegawai</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 250231501000526</t>
+  </si>
+  <si>
+    <t>00113T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran THR Tahun 2025 Untuk 39 Pegawai</t>
   </si>
   <si>
     <t xml:space="preserve"> 250231501000528</t>
@@ -3185,15 +3203,6 @@
     <t>Pembayaran THR Tahun 2025 Untuk 139 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231501000527</t>
-  </si>
-  <si>
-    <t>00114T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran THR Tahun 2025 Untuk 1 Pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231501000545</t>
   </si>
   <si>
@@ -3203,6 +3212,15 @@
     <t>Pembayaran THR Keagamaan Tahun 2025 Untuk 16 Pegawai.</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231501000529</t>
+  </si>
+  <si>
+    <t>00118T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran THR Tahun 2025 Untuk 50 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231501000530</t>
   </si>
   <si>
@@ -3212,24 +3230,6 @@
     <t>Pembayaran THR Tahun 2025 Untuk 36 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231501000526</t>
-  </si>
-  <si>
-    <t>00113T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran THR Tahun 2025 Untuk 39 Pegawai</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 250231501000529</t>
-  </si>
-  <si>
-    <t>00118T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran THR Tahun 2025 Untuk 50 Pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231302002452</t>
   </si>
   <si>
@@ -3278,6 +3278,15 @@
     <t>Pembayaran tunjangan kinerja bulan Januari tahun 2025 untuk 1 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231303000778</t>
+  </si>
+  <si>
+    <t>00110T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran tunjangan kinerja bulan Februari tahun 2025 untuk 177 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231303000777</t>
   </si>
   <si>
@@ -3290,13 +3299,22 @@
     <t>Pembayaran Belanja Pegawai berupa Gaji Susulan Bulan Maret 2025 untuk 1 Pegawai/4 jiwa</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231303000778</t>
-  </si>
-  <si>
-    <t>00110T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran tunjangan kinerja bulan Februari tahun 2025 untuk 177 Pegawai</t>
+    <t xml:space="preserve"> 250231301002370</t>
+  </si>
+  <si>
+    <t>00100T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Februari 2025 untuk 37 pegawai</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 250231301002372</t>
+  </si>
+  <si>
+    <t>00106T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran tunjangan kinerja bulan Februari tahun 2025 untuk 36 Pegawai</t>
   </si>
   <si>
     <t xml:space="preserve"> 250231301002369</t>
@@ -3308,24 +3326,6 @@
     <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan februari 2025 untuk 136 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231301002372</t>
-  </si>
-  <si>
-    <t>00106T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran tunjangan kinerja bulan Februari tahun 2025 untuk 36 Pegawai</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 250231301002370</t>
-  </si>
-  <si>
-    <t>00100T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Februari 2025 untuk 37 pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231301002371</t>
   </si>
   <si>
@@ -3344,6 +3344,15 @@
     <t>Pembayaran Belanja Pegawai berupa Uang Makan bulan Februari 2025 untuk 36 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231303000774</t>
+  </si>
+  <si>
+    <t>00105T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran tunjangan kinerja bulan Februari tahun 2025 untuk 63 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231303000773</t>
   </si>
   <si>
@@ -3353,15 +3362,6 @@
     <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan februari 2025 untuk 63 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231303000774</t>
-  </si>
-  <si>
-    <t>00105T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran tunjangan kinerja bulan Februari tahun 2025 untuk 63 Pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231303000772</t>
   </si>
   <si>
@@ -3473,48 +3473,48 @@
     <t>Pembayaran Belanja Barang Berupa Honor PPNPN Bulan Januari Tahun 2025 untuk 90 Pegawai.sesuai Sk no.9 tahun 2025 tanggal 6 januari 2025</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231303000475</t>
+  </si>
+  <si>
+    <t>25-02-2025</t>
+  </si>
+  <si>
+    <t>26-02-2025</t>
+  </si>
+  <si>
+    <t>00076T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran tunjangan kinerja bulan Januari tahun 2025 untuk 63 Pegawai</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 250231303000476</t>
+  </si>
+  <si>
+    <t>00075T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran tunjangan kinerja bulan Januari tahun 2025 untuk 177 Pegawai</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 250231303000474</t>
+  </si>
+  <si>
+    <t>00074T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Uang Makan PPPK bulan Januari 2025 untuk 63 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231303000473</t>
   </si>
   <si>
-    <t>25-02-2025</t>
-  </si>
-  <si>
-    <t>26-02-2025</t>
-  </si>
-  <si>
     <t>00073T/403829/2025</t>
   </si>
   <si>
     <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Januari 2025 untuk 175 pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231303000476</t>
-  </si>
-  <si>
-    <t>00075T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran tunjangan kinerja bulan Januari tahun 2025 untuk 177 Pegawai</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 250231303000475</t>
-  </si>
-  <si>
-    <t>00076T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran tunjangan kinerja bulan Januari tahun 2025 untuk 63 Pegawai</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 250231303000474</t>
-  </si>
-  <si>
-    <t>00074T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Uang Makan PPPK bulan Januari 2025 untuk 63 Pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231305000180</t>
   </si>
   <si>
@@ -3563,6 +3563,36 @@
     <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan Maret 2025 untuk 2 Pegawai /8 Jiwa</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231501000434</t>
+  </si>
+  <si>
+    <t>00067T/403829/2025</t>
+  </si>
+  <si>
+    <t>18-02-2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan Maret 2025 untuk 36 Pegawai/106 Jiwa</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 250231501000432</t>
+  </si>
+  <si>
+    <t>00064T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai Berupa Gaji Induk bulan Maret 2025 untuk 137 Pegawai/403 Jiwa</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 250231501000433</t>
+  </si>
+  <si>
+    <t>00065T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai Berupa Gaji Induk Maret 2025 untuk 50 Pegawai/123 Jiwa</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231501000431</t>
   </si>
   <si>
@@ -3572,27 +3602,6 @@
     <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan Maret 2025 untuk 39 Pegawai/112 Jiwa</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231501000434</t>
-  </si>
-  <si>
-    <t>00067T/403829/2025</t>
-  </si>
-  <si>
-    <t>18-02-2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan Maret 2025 untuk 36 Pegawai/106 Jiwa</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 250231501000433</t>
-  </si>
-  <si>
-    <t>00065T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai Berupa Gaji Induk Maret 2025 untuk 50 Pegawai/123 Jiwa</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231501000339</t>
   </si>
   <si>
@@ -3605,15 +3614,6 @@
     <t>Pembayaran Belanja Barang Berupa Honor PPNPN Bulan Februari Tahun 2025 untuk 16 Pegawai.sesuai SK No.04/BRPBATPP/KP.340/I/2025 Tanggal 2 Januari 2025</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231501000432</t>
-  </si>
-  <si>
-    <t>00064T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai Berupa Gaji Induk bulan Maret 2025 untuk 137 Pegawai/403 Jiwa</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231503000118</t>
   </si>
   <si>
@@ -3644,6 +3644,15 @@
     <t>Pembayaran tunjangan kinerja bulan Januari tahun 2025 untuk 138 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231301001113</t>
+  </si>
+  <si>
+    <t>00061T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran tunjangan kinerja bulan Januari tahun 2025 untuk 36 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231301001112</t>
   </si>
   <si>
@@ -3653,39 +3662,30 @@
     <t>Pembayaran tunjangan kinerja  bulan Januari tahun 2025 untuk 50 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231301001113</t>
-  </si>
-  <si>
-    <t>00061T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran tunjangan kinerja bulan Januari tahun 2025 untuk 36 Pegawai</t>
+    <t xml:space="preserve"> 250231301001062</t>
+  </si>
+  <si>
+    <t>16-02-2025</t>
+  </si>
+  <si>
+    <t>00051T/403829/2025</t>
+  </si>
+  <si>
+    <t>13-02-2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Uang Makan bulan Januari 2025 untuk 36 Pegawai</t>
   </si>
   <si>
     <t xml:space="preserve"> 250231301001061</t>
   </si>
   <si>
-    <t>16-02-2025</t>
-  </si>
-  <si>
     <t>00052T/403829/2025</t>
   </si>
   <si>
-    <t>13-02-2025</t>
-  </si>
-  <si>
     <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Januari 2025 untuk 37 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231301001062</t>
-  </si>
-  <si>
-    <t>00051T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Uang Makan bulan Januari 2025 untuk 36 Pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231305000122</t>
   </si>
   <si>
@@ -3698,6 +3698,15 @@
     <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Januari 2025 untuk 2 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231301000961</t>
+  </si>
+  <si>
+    <t>00050T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Januari 2025 untuk 50 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231301000960</t>
   </si>
   <si>
@@ -3707,15 +3716,6 @@
     <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Januari 2025 untuk 136 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231301000961</t>
-  </si>
-  <si>
-    <t>00050T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Januari 2025 untuk 50 Pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231305000116</t>
   </si>
   <si>
@@ -3764,6 +3764,15 @@
     <t>Pembayaran belanja barang berupa tagihan telepon bulan Februari 2025 untuk 12 invoice</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231302000796</t>
+  </si>
+  <si>
+    <t>00048T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Barang sesuai Kwitansi No. 02/SAJ/KW/II/2025 Tanggal 3 Februari 2025 berupa Pemeliharaan Halaman Kantor Instalasi Riset Pengendalian Penyakit Ikan Depok</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231302000795</t>
   </si>
   <si>
@@ -3773,15 +3782,6 @@
     <t>Pembayaran Belanja Barang sesuai Kwitansi No.001/KW-PNA/II/2025 Tanggal 6 Februari 2025 berupa Pemelliharaan Talud Cijeruk</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231302000796</t>
-  </si>
-  <si>
-    <t>00048T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Barang sesuai Kwitansi No. 02/SAJ/KW/II/2025 Tanggal 3 Februari 2025 berupa Pemeliharaan Halaman Kantor Instalasi Riset Pengendalian Penyakit Ikan Depok</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231301000882</t>
   </si>
   <si>
@@ -3893,6 +3893,15 @@
     <t>Pembayaran tunjangan kinerja bulan Februari tahun 2025 untuk 2 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231301000432</t>
+  </si>
+  <si>
+    <t>00030T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran tunjangan kinerja bulan Februari tahun 2025 untuk 38 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231301000433</t>
   </si>
   <si>
@@ -3902,15 +3911,6 @@
     <t>Pembayaran tunjangan kinerja bulan Februari tahun 2025 untuk 1 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231301000432</t>
-  </si>
-  <si>
-    <t>00030T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran tunjangan kinerja bulan Februari tahun 2025 untuk 38 Pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231303000130</t>
   </si>
   <si>
@@ -3920,6 +3920,15 @@
     <t>Pembayaran Belanja Barang sesuai Kwitansi No. 02/MSP/KW/I/2025 Tanggal 20 Januari 2025 berupa Perbaikan Kamar Mandi dan Sanitasi</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231301000416</t>
+  </si>
+  <si>
+    <t>00028T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran tunjangan kinerja susulan bulan Desember tahun 2024 untuk 1 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231301000417</t>
   </si>
   <si>
@@ -3929,15 +3938,6 @@
     <t>Pembayaran kekurangan tunjangan kinerja bulan Desember tahun 2024 untuk 1 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231301000416</t>
-  </si>
-  <si>
-    <t>00028T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran tunjangan kinerja susulan bulan Desember tahun 2024 untuk 1 Pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231501000261</t>
   </si>
   <si>
@@ -3950,27 +3950,27 @@
     <t>Pembayaran Belanja Barang Berupa Honor PPNPN Bulan Januari Tahun 2025 untuk 17 Pegawai.sesuai SK No.B.4/BRPBATPP/KP.340/I/2025 tanggal 2 Januari 2025</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231301000385</t>
+  </si>
+  <si>
+    <t>23-01-2025</t>
+  </si>
+  <si>
+    <t>00025T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji Susulan Bulan Desember 2024 untuk 1 Pegawai/4 Jiwa</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231301000386</t>
   </si>
   <si>
-    <t>23-01-2025</t>
-  </si>
-  <si>
     <t>00026T/403829/2025</t>
   </si>
   <si>
     <t>Pembayaran Belanja Pegawai berupa Kekurangan Gaji Bulan Desember 2024 untuk 1 Pegawai/4 Jiwa</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231301000385</t>
-  </si>
-  <si>
-    <t>00025T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji Susulan Bulan Desember 2024 untuk 1 Pegawai/4 Jiwa</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231302000370</t>
   </si>
   <si>
@@ -3995,6 +3995,27 @@
     <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan Februari 2025 untuk 36 Pegawai/105 Jiwa</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231501000228</t>
+  </si>
+  <si>
+    <t>00021T/403829/2025</t>
+  </si>
+  <si>
+    <t>14-01-2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan februari 2025 untuk 138 Pegawai/406 Jiwa</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 250231501000227</t>
+  </si>
+  <si>
+    <t>00019T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan februari 2025 untuk 39 Pegawai/112 jiwa</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231501000229</t>
   </si>
   <si>
@@ -4004,27 +4025,6 @@
     <t>Pembayaran Belanja Pegawai Berupa Gaji Induk PPPK Bulan Februari 2025 untuk 50 Pegawai/123 Jiwa</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231501000227</t>
-  </si>
-  <si>
-    <t>00019T/403829/2025</t>
-  </si>
-  <si>
-    <t>14-01-2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan februari 2025 untuk 39 Pegawai/112 jiwa</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 250231501000228</t>
-  </si>
-  <si>
-    <t>00021T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan februari 2025 untuk 138 Pegawai/406 Jiwa</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231507000048</t>
   </si>
   <si>
@@ -4067,15 +4067,24 @@
     <t>Pembayaran Belanja Barang berupa Tagihan Internet Bulan Januari 2025 Idpel No.GO18A106 An Balai Riset Perikanan Budidaya Air Tawar dan Penyuluhan Perikanan</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231301000152</t>
+  </si>
+  <si>
+    <t>10-01-2025</t>
+  </si>
+  <si>
+    <t>13-01-2025</t>
+  </si>
+  <si>
+    <t>00016T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gai Susulan Bulan Desember 2024 sd Januari 2025 untuk 1 Pegawai/4 Jiwa</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231301000153</t>
   </si>
   <si>
-    <t>10-01-2025</t>
-  </si>
-  <si>
-    <t>13-01-2025</t>
-  </si>
-  <si>
     <t>00017T/403829/2025</t>
   </si>
   <si>
@@ -4083,15 +4092,6 @@
   </si>
   <si>
     <t>Penyediaan Uang Persediaan BALAI RISET PERIKANAN BUDIDAYA AIR TAWAR DAN PENYULUHAN PERIKANAN Tahun Anggaran 2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 250231301000152</t>
-  </si>
-  <si>
-    <t>00016T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gai Susulan Bulan Desember 2024 sd Januari 2025 untuk 1 Pegawai/4 Jiwa</t>
   </si>
   <si>
     <t xml:space="preserve"> 250231303000044</t>
@@ -6830,7 +6830,7 @@
         <v>211</v>
       </c>
       <c r="E65" s="1">
-        <v>655816000</v>
+        <v>200500400</v>
       </c>
       <c r="F65" s="1" t="s">
         <v>238</v>
@@ -6839,7 +6839,7 @@
         <v>239</v>
       </c>
       <c r="H65" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I65" s="1" t="s">
         <v>78</v>
@@ -6866,7 +6866,7 @@
         <v>211</v>
       </c>
       <c r="E66" s="1">
-        <v>200500400</v>
+        <v>655816000</v>
       </c>
       <c r="F66" s="1" t="s">
         <v>242</v>
@@ -6875,7 +6875,7 @@
         <v>239</v>
       </c>
       <c r="H66" s="1" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="I66" s="1" t="s">
         <v>78</v>
@@ -6902,22 +6902,22 @@
         <v>211</v>
       </c>
       <c r="E67" s="1">
-        <v>168310100</v>
+        <v>144846400</v>
       </c>
       <c r="F67" s="1" t="s">
         <v>245</v>
       </c>
       <c r="G67" s="1" t="s">
-        <v>246</v>
+        <v>239</v>
       </c>
       <c r="H67" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I67" s="1" t="s">
         <v>78</v>
       </c>
       <c r="J67" s="1" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="K67" s="1" t="s">
         <v>19</v>
@@ -6929,7 +6929,7 @@
         <v>65</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C68" s="1" t="s">
         <v>237</v>
@@ -6938,16 +6938,16 @@
         <v>211</v>
       </c>
       <c r="E68" s="1">
-        <v>144846400</v>
+        <v>168310100</v>
       </c>
       <c r="F68" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="G68" s="1" t="s">
         <v>249</v>
       </c>
-      <c r="G68" s="1" t="s">
-        <v>239</v>
-      </c>
       <c r="H68" s="1" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="I68" s="1" t="s">
         <v>78</v>
@@ -7010,7 +7010,7 @@
         <v>211</v>
       </c>
       <c r="E70" s="1">
-        <v>268443100</v>
+        <v>844985400</v>
       </c>
       <c r="F70" s="1" t="s">
         <v>255</v>
@@ -7019,7 +7019,7 @@
         <v>239</v>
       </c>
       <c r="H70" s="1" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="I70" s="1" t="s">
         <v>78</v>
@@ -7046,7 +7046,7 @@
         <v>211</v>
       </c>
       <c r="E71" s="1">
-        <v>844985400</v>
+        <v>91372600</v>
       </c>
       <c r="F71" s="1" t="s">
         <v>258</v>
@@ -7055,7 +7055,7 @@
         <v>239</v>
       </c>
       <c r="H71" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I71" s="1" t="s">
         <v>78</v>
@@ -7082,7 +7082,7 @@
         <v>211</v>
       </c>
       <c r="E72" s="1">
-        <v>91372600</v>
+        <v>268443100</v>
       </c>
       <c r="F72" s="1" t="s">
         <v>261</v>
@@ -7112,19 +7112,19 @@
         <v>263</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="D73" s="1" t="s">
         <v>237</v>
       </c>
       <c r="E73" s="1">
-        <v>153763873</v>
+        <v>213199358</v>
       </c>
       <c r="F73" s="1" t="s">
         <v>264</v>
       </c>
       <c r="G73" s="1" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="H73" s="1" t="s">
         <v>135</v>
@@ -7148,19 +7148,19 @@
         <v>266</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="D74" s="1" t="s">
         <v>237</v>
       </c>
       <c r="E74" s="1">
-        <v>823139642</v>
+        <v>153763873</v>
       </c>
       <c r="F74" s="1" t="s">
         <v>267</v>
       </c>
       <c r="G74" s="1" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="H74" s="1" t="s">
         <v>135</v>
@@ -7184,19 +7184,19 @@
         <v>269</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="D75" s="1" t="s">
         <v>237</v>
       </c>
       <c r="E75" s="1">
-        <v>213199358</v>
+        <v>823139642</v>
       </c>
       <c r="F75" s="1" t="s">
         <v>270</v>
       </c>
       <c r="G75" s="1" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="H75" s="1" t="s">
         <v>135</v>
@@ -7220,7 +7220,7 @@
         <v>272</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="D76" s="1" t="s">
         <v>237</v>
@@ -7232,7 +7232,7 @@
         <v>273</v>
       </c>
       <c r="G76" s="1" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="H76" s="1" t="s">
         <v>135</v>
@@ -7256,7 +7256,7 @@
         <v>275</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="D77" s="1" t="s">
         <v>237</v>
@@ -7268,7 +7268,7 @@
         <v>276</v>
       </c>
       <c r="G77" s="1" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="H77" s="1" t="s">
         <v>135</v>
@@ -7292,10 +7292,10 @@
         <v>278</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="D78" s="1" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="E78" s="1">
         <v>455600</v>
@@ -7304,7 +7304,7 @@
         <v>279</v>
       </c>
       <c r="G78" s="1" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="H78" s="1" t="s">
         <v>42</v>
@@ -7328,10 +7328,10 @@
         <v>281</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="D79" s="1" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="E79" s="1">
         <v>698200</v>
@@ -7340,7 +7340,7 @@
         <v>282</v>
       </c>
       <c r="G79" s="1" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="H79" s="1" t="s">
         <v>42</v>
@@ -7727,7 +7727,7 @@
         <v>239</v>
       </c>
       <c r="D90" s="1" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="E90" s="1">
         <v>41758847</v>
@@ -7763,7 +7763,7 @@
         <v>239</v>
       </c>
       <c r="D91" s="1" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="E91" s="1">
         <v>2844264</v>
@@ -8270,7 +8270,7 @@
         <v>336</v>
       </c>
       <c r="E105" s="1">
-        <v>200371400</v>
+        <v>661725600</v>
       </c>
       <c r="F105" s="1" t="s">
         <v>370</v>
@@ -8279,7 +8279,7 @@
         <v>371</v>
       </c>
       <c r="H105" s="1" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="I105" s="1" t="s">
         <v>78</v>
@@ -8306,7 +8306,7 @@
         <v>336</v>
       </c>
       <c r="E106" s="1">
-        <v>661725600</v>
+        <v>171835300</v>
       </c>
       <c r="F106" s="1" t="s">
         <v>374</v>
@@ -8378,7 +8378,7 @@
         <v>336</v>
       </c>
       <c r="E108" s="1">
-        <v>171835300</v>
+        <v>200371400</v>
       </c>
       <c r="F108" s="1" t="s">
         <v>380</v>
@@ -8387,7 +8387,7 @@
         <v>371</v>
       </c>
       <c r="H108" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I108" s="1" t="s">
         <v>78</v>
@@ -8558,7 +8558,7 @@
         <v>397</v>
       </c>
       <c r="E113" s="1">
-        <v>822658451</v>
+        <v>154096751</v>
       </c>
       <c r="F113" s="1" t="s">
         <v>398</v>
@@ -8594,7 +8594,7 @@
         <v>397</v>
       </c>
       <c r="E114" s="1">
-        <v>154096751</v>
+        <v>822658451</v>
       </c>
       <c r="F114" s="1" t="s">
         <v>401</v>
@@ -8630,7 +8630,7 @@
         <v>397</v>
       </c>
       <c r="E115" s="1">
-        <v>1040244280</v>
+        <v>99668220</v>
       </c>
       <c r="F115" s="1" t="s">
         <v>404</v>
@@ -8702,7 +8702,7 @@
         <v>397</v>
       </c>
       <c r="E117" s="1">
-        <v>99668220</v>
+        <v>1040244280</v>
       </c>
       <c r="F117" s="1" t="s">
         <v>410</v>
@@ -8774,7 +8774,7 @@
         <v>416</v>
       </c>
       <c r="E119" s="1">
-        <v>22399900</v>
+        <v>21398250</v>
       </c>
       <c r="F119" s="1" t="s">
         <v>417</v>
@@ -8783,7 +8783,7 @@
         <v>371</v>
       </c>
       <c r="H119" s="1" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="I119" s="1" t="s">
         <v>17</v>
@@ -8810,7 +8810,7 @@
         <v>416</v>
       </c>
       <c r="E120" s="1">
-        <v>82033000</v>
+        <v>22399900</v>
       </c>
       <c r="F120" s="1" t="s">
         <v>420</v>
@@ -8882,7 +8882,7 @@
         <v>416</v>
       </c>
       <c r="E122" s="1">
-        <v>21398250</v>
+        <v>82033000</v>
       </c>
       <c r="F122" s="1" t="s">
         <v>426</v>
@@ -8891,7 +8891,7 @@
         <v>371</v>
       </c>
       <c r="H122" s="1" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="I122" s="1" t="s">
         <v>17</v>
@@ -8954,7 +8954,7 @@
         <v>416</v>
       </c>
       <c r="E124" s="1">
-        <v>106926550</v>
+        <v>13597650</v>
       </c>
       <c r="F124" s="1" t="s">
         <v>432</v>
@@ -8963,7 +8963,7 @@
         <v>371</v>
       </c>
       <c r="H124" s="1" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="I124" s="1" t="s">
         <v>17</v>
@@ -8990,7 +8990,7 @@
         <v>416</v>
       </c>
       <c r="E125" s="1">
-        <v>38519000</v>
+        <v>106926550</v>
       </c>
       <c r="F125" s="1" t="s">
         <v>435</v>
@@ -8999,7 +8999,7 @@
         <v>371</v>
       </c>
       <c r="H125" s="1" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="I125" s="1" t="s">
         <v>17</v>
@@ -9026,7 +9026,7 @@
         <v>416</v>
       </c>
       <c r="E126" s="1">
-        <v>13597650</v>
+        <v>38519000</v>
       </c>
       <c r="F126" s="1" t="s">
         <v>438</v>
@@ -9242,7 +9242,7 @@
         <v>456</v>
       </c>
       <c r="E132" s="1">
-        <v>4595150</v>
+        <v>597550</v>
       </c>
       <c r="F132" s="1" t="s">
         <v>463</v>
@@ -9251,7 +9251,7 @@
         <v>464</v>
       </c>
       <c r="H132" s="1" t="s">
-        <v>135</v>
+        <v>16</v>
       </c>
       <c r="I132" s="1" t="s">
         <v>17</v>
@@ -9278,7 +9278,7 @@
         <v>456</v>
       </c>
       <c r="E133" s="1">
-        <v>597550</v>
+        <v>4595150</v>
       </c>
       <c r="F133" s="1" t="s">
         <v>467</v>
@@ -9287,7 +9287,7 @@
         <v>464</v>
       </c>
       <c r="H133" s="1" t="s">
-        <v>16</v>
+        <v>135</v>
       </c>
       <c r="I133" s="1" t="s">
         <v>17</v>
@@ -9422,7 +9422,7 @@
         <v>464</v>
       </c>
       <c r="E137" s="1">
-        <v>679180900</v>
+        <v>177279700</v>
       </c>
       <c r="F137" s="1" t="s">
         <v>481</v>
@@ -9458,7 +9458,7 @@
         <v>464</v>
       </c>
       <c r="E138" s="1">
-        <v>200371400</v>
+        <v>679180900</v>
       </c>
       <c r="F138" s="1" t="s">
         <v>485</v>
@@ -9467,7 +9467,7 @@
         <v>482</v>
       </c>
       <c r="H138" s="1" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="I138" s="1" t="s">
         <v>78</v>
@@ -9530,7 +9530,7 @@
         <v>464</v>
       </c>
       <c r="E140" s="1">
-        <v>177279700</v>
+        <v>200371400</v>
       </c>
       <c r="F140" s="1" t="s">
         <v>491</v>
@@ -9539,7 +9539,7 @@
         <v>482</v>
       </c>
       <c r="H140" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I140" s="1" t="s">
         <v>78</v>
@@ -9638,7 +9638,7 @@
         <v>464</v>
       </c>
       <c r="E143" s="1">
-        <v>62679696</v>
+        <v>261119293</v>
       </c>
       <c r="F143" s="1" t="s">
         <v>502</v>
@@ -9674,7 +9674,7 @@
         <v>464</v>
       </c>
       <c r="E144" s="1">
-        <v>261119293</v>
+        <v>62679696</v>
       </c>
       <c r="F144" s="1" t="s">
         <v>505</v>
@@ -9710,16 +9710,16 @@
         <v>464</v>
       </c>
       <c r="E145" s="1">
-        <v>230734521</v>
+        <v>261772500</v>
       </c>
       <c r="F145" s="1" t="s">
         <v>508</v>
       </c>
       <c r="G145" s="1" t="s">
-        <v>496</v>
+        <v>482</v>
       </c>
       <c r="H145" s="1" t="s">
-        <v>77</v>
+        <v>101</v>
       </c>
       <c r="I145" s="1" t="s">
         <v>78</v>
@@ -9746,22 +9746,22 @@
         <v>464</v>
       </c>
       <c r="E146" s="1">
-        <v>91372600</v>
+        <v>865011300</v>
       </c>
       <c r="F146" s="1" t="s">
         <v>511</v>
       </c>
       <c r="G146" s="1" t="s">
-        <v>482</v>
+        <v>512</v>
       </c>
       <c r="H146" s="1" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="I146" s="1" t="s">
         <v>78</v>
       </c>
       <c r="J146" s="1" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="K146" s="1" t="s">
         <v>19</v>
@@ -9773,7 +9773,7 @@
         <v>144</v>
       </c>
       <c r="B147" s="1" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="C147" s="1" t="s">
         <v>494</v>
@@ -9782,16 +9782,16 @@
         <v>464</v>
       </c>
       <c r="E147" s="1">
-        <v>865011300</v>
+        <v>91372600</v>
       </c>
       <c r="F147" s="1" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="G147" s="1" t="s">
-        <v>515</v>
+        <v>482</v>
       </c>
       <c r="H147" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I147" s="1" t="s">
         <v>78</v>
@@ -9818,16 +9818,16 @@
         <v>464</v>
       </c>
       <c r="E148" s="1">
-        <v>261772500</v>
+        <v>230734521</v>
       </c>
       <c r="F148" s="1" t="s">
         <v>518</v>
       </c>
       <c r="G148" s="1" t="s">
-        <v>482</v>
+        <v>496</v>
       </c>
       <c r="H148" s="1" t="s">
-        <v>101</v>
+        <v>77</v>
       </c>
       <c r="I148" s="1" t="s">
         <v>78</v>
@@ -9884,10 +9884,10 @@
         <v>523</v>
       </c>
       <c r="C150" s="1" t="s">
-        <v>515</v>
+        <v>512</v>
       </c>
       <c r="D150" s="1" t="s">
-        <v>515</v>
+        <v>512</v>
       </c>
       <c r="E150" s="1">
         <v>150900</v>
@@ -9926,7 +9926,7 @@
         <v>529</v>
       </c>
       <c r="E151" s="1">
-        <v>213272917</v>
+        <v>846201196</v>
       </c>
       <c r="F151" s="1" t="s">
         <v>530</v>
@@ -9962,7 +9962,7 @@
         <v>529</v>
       </c>
       <c r="E152" s="1">
-        <v>153824056</v>
+        <v>213272917</v>
       </c>
       <c r="F152" s="1" t="s">
         <v>533</v>
@@ -9998,7 +9998,7 @@
         <v>529</v>
       </c>
       <c r="E153" s="1">
-        <v>846201196</v>
+        <v>153824056</v>
       </c>
       <c r="F153" s="1" t="s">
         <v>536</v>
@@ -10034,7 +10034,7 @@
         <v>529</v>
       </c>
       <c r="E154" s="1">
-        <v>279620735</v>
+        <v>1035489776</v>
       </c>
       <c r="F154" s="1" t="s">
         <v>539</v>
@@ -10106,7 +10106,7 @@
         <v>529</v>
       </c>
       <c r="E156" s="1">
-        <v>1035489776</v>
+        <v>279620735</v>
       </c>
       <c r="F156" s="1" t="s">
         <v>545</v>
@@ -10178,7 +10178,7 @@
         <v>548</v>
       </c>
       <c r="E158" s="1">
-        <v>15407872</v>
+        <v>119845265</v>
       </c>
       <c r="F158" s="1" t="s">
         <v>552</v>
@@ -10187,13 +10187,13 @@
         <v>548</v>
       </c>
       <c r="H158" s="1" t="s">
-        <v>129</v>
+        <v>53</v>
       </c>
       <c r="I158" s="1" t="s">
         <v>17</v>
       </c>
       <c r="J158" s="1" t="s">
-        <v>130</v>
+        <v>54</v>
       </c>
       <c r="K158" s="1" t="s">
         <v>19</v>
@@ -10214,7 +10214,7 @@
         <v>548</v>
       </c>
       <c r="E159" s="1">
-        <v>119845265</v>
+        <v>15407872</v>
       </c>
       <c r="F159" s="1" t="s">
         <v>554</v>
@@ -10223,13 +10223,13 @@
         <v>548</v>
       </c>
       <c r="H159" s="1" t="s">
-        <v>53</v>
+        <v>129</v>
       </c>
       <c r="I159" s="1" t="s">
         <v>17</v>
       </c>
       <c r="J159" s="1" t="s">
-        <v>54</v>
+        <v>130</v>
       </c>
       <c r="K159" s="1" t="s">
         <v>19</v>
@@ -10394,7 +10394,7 @@
         <v>556</v>
       </c>
       <c r="E164" s="1">
-        <v>933200</v>
+        <v>22220250</v>
       </c>
       <c r="F164" s="1" t="s">
         <v>569</v>
@@ -10403,7 +10403,7 @@
         <v>570</v>
       </c>
       <c r="H164" s="1" t="s">
-        <v>42</v>
+        <v>16</v>
       </c>
       <c r="I164" s="1" t="s">
         <v>17</v>
@@ -10430,7 +10430,7 @@
         <v>556</v>
       </c>
       <c r="E165" s="1">
-        <v>22220250</v>
+        <v>79464800</v>
       </c>
       <c r="F165" s="1" t="s">
         <v>573</v>
@@ -10466,7 +10466,7 @@
         <v>556</v>
       </c>
       <c r="E166" s="1">
-        <v>79464800</v>
+        <v>441700</v>
       </c>
       <c r="F166" s="1" t="s">
         <v>576</v>
@@ -10475,7 +10475,7 @@
         <v>570</v>
       </c>
       <c r="H166" s="1" t="s">
-        <v>16</v>
+        <v>42</v>
       </c>
       <c r="I166" s="1" t="s">
         <v>17</v>
@@ -10502,7 +10502,7 @@
         <v>556</v>
       </c>
       <c r="E167" s="1">
-        <v>441700</v>
+        <v>933200</v>
       </c>
       <c r="F167" s="1" t="s">
         <v>579</v>
@@ -10538,7 +10538,7 @@
         <v>556</v>
       </c>
       <c r="E168" s="1">
-        <v>219100</v>
+        <v>100681700</v>
       </c>
       <c r="F168" s="1" t="s">
         <v>582</v>
@@ -10547,7 +10547,7 @@
         <v>570</v>
       </c>
       <c r="H168" s="1" t="s">
-        <v>42</v>
+        <v>16</v>
       </c>
       <c r="I168" s="1" t="s">
         <v>17</v>
@@ -10574,7 +10574,7 @@
         <v>556</v>
       </c>
       <c r="E169" s="1">
-        <v>100681700</v>
+        <v>219100</v>
       </c>
       <c r="F169" s="1" t="s">
         <v>585</v>
@@ -10583,7 +10583,7 @@
         <v>570</v>
       </c>
       <c r="H169" s="1" t="s">
-        <v>16</v>
+        <v>42</v>
       </c>
       <c r="I169" s="1" t="s">
         <v>17</v>
@@ -10682,7 +10682,7 @@
         <v>570</v>
       </c>
       <c r="E172" s="1">
-        <v>29781850</v>
+        <v>20168600</v>
       </c>
       <c r="F172" s="1" t="s">
         <v>594</v>
@@ -10718,7 +10718,7 @@
         <v>570</v>
       </c>
       <c r="E173" s="1">
-        <v>20168600</v>
+        <v>29781850</v>
       </c>
       <c r="F173" s="1" t="s">
         <v>597</v>
@@ -11114,7 +11114,7 @@
         <v>613</v>
       </c>
       <c r="E184" s="1">
-        <v>102434200</v>
+        <v>287324950</v>
       </c>
       <c r="F184" s="1" t="s">
         <v>633</v>
@@ -11150,7 +11150,7 @@
         <v>613</v>
       </c>
       <c r="E185" s="1">
-        <v>287324950</v>
+        <v>1037129350</v>
       </c>
       <c r="F185" s="1" t="s">
         <v>636</v>
@@ -11186,7 +11186,7 @@
         <v>613</v>
       </c>
       <c r="E186" s="1">
-        <v>1037129350</v>
+        <v>102434200</v>
       </c>
       <c r="F186" s="1" t="s">
         <v>639</v>
@@ -11258,7 +11258,7 @@
         <v>613</v>
       </c>
       <c r="E188" s="1">
-        <v>751528800</v>
+        <v>204525900</v>
       </c>
       <c r="F188" s="1" t="s">
         <v>647</v>
@@ -11267,13 +11267,13 @@
         <v>646</v>
       </c>
       <c r="H188" s="1" t="s">
-        <v>474</v>
+        <v>648</v>
       </c>
       <c r="I188" s="1" t="s">
         <v>78</v>
       </c>
       <c r="J188" s="1" t="s">
-        <v>648</v>
+        <v>649</v>
       </c>
       <c r="K188" s="1" t="s">
         <v>19</v>
@@ -11285,7 +11285,7 @@
         <v>186</v>
       </c>
       <c r="B189" s="1" t="s">
-        <v>649</v>
+        <v>650</v>
       </c>
       <c r="C189" s="1" t="s">
         <v>646</v>
@@ -11294,16 +11294,16 @@
         <v>613</v>
       </c>
       <c r="E189" s="1">
-        <v>147826000</v>
+        <v>751528800</v>
       </c>
       <c r="F189" s="1" t="s">
-        <v>650</v>
+        <v>651</v>
       </c>
       <c r="G189" s="1" t="s">
         <v>646</v>
       </c>
       <c r="H189" s="1" t="s">
-        <v>651</v>
+        <v>474</v>
       </c>
       <c r="I189" s="1" t="s">
         <v>78</v>
@@ -11330,7 +11330,7 @@
         <v>613</v>
       </c>
       <c r="E190" s="1">
-        <v>204525900</v>
+        <v>147826000</v>
       </c>
       <c r="F190" s="1" t="s">
         <v>654</v>
@@ -11339,7 +11339,7 @@
         <v>646</v>
       </c>
       <c r="H190" s="1" t="s">
-        <v>651</v>
+        <v>648</v>
       </c>
       <c r="I190" s="1" t="s">
         <v>78</v>
@@ -11402,7 +11402,7 @@
         <v>613</v>
       </c>
       <c r="E192" s="1">
-        <v>93291700</v>
+        <v>267194900</v>
       </c>
       <c r="F192" s="1" t="s">
         <v>660</v>
@@ -11411,7 +11411,7 @@
         <v>646</v>
       </c>
       <c r="H192" s="1" t="s">
-        <v>651</v>
+        <v>648</v>
       </c>
       <c r="I192" s="1" t="s">
         <v>78</v>
@@ -11474,7 +11474,7 @@
         <v>613</v>
       </c>
       <c r="E194" s="1">
-        <v>267194900</v>
+        <v>93291700</v>
       </c>
       <c r="F194" s="1" t="s">
         <v>666</v>
@@ -11483,7 +11483,7 @@
         <v>646</v>
       </c>
       <c r="H194" s="1" t="s">
-        <v>651</v>
+        <v>648</v>
       </c>
       <c r="I194" s="1" t="s">
         <v>78</v>
@@ -11690,7 +11690,7 @@
         <v>669</v>
       </c>
       <c r="E200" s="1">
-        <v>91372600</v>
+        <v>261772500</v>
       </c>
       <c r="F200" s="1" t="s">
         <v>687</v>
@@ -11726,7 +11726,7 @@
         <v>669</v>
       </c>
       <c r="E201" s="1">
-        <v>261772500</v>
+        <v>91372600</v>
       </c>
       <c r="F201" s="1" t="s">
         <v>691</v>
@@ -11834,16 +11834,16 @@
         <v>669</v>
       </c>
       <c r="E204" s="1">
-        <v>144846400</v>
+        <v>679180900</v>
       </c>
       <c r="F204" s="1" t="s">
         <v>701</v>
       </c>
       <c r="G204" s="1" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
       <c r="H204" s="1" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="I204" s="1" t="s">
         <v>78</v>
@@ -11870,16 +11870,16 @@
         <v>669</v>
       </c>
       <c r="E205" s="1">
-        <v>177279700</v>
+        <v>200371400</v>
       </c>
       <c r="F205" s="1" t="s">
         <v>704</v>
       </c>
       <c r="G205" s="1" t="s">
-        <v>695</v>
+        <v>688</v>
       </c>
       <c r="H205" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I205" s="1" t="s">
         <v>78</v>
@@ -11906,16 +11906,16 @@
         <v>669</v>
       </c>
       <c r="E206" s="1">
-        <v>200371400</v>
+        <v>177279700</v>
       </c>
       <c r="F206" s="1" t="s">
         <v>707</v>
       </c>
       <c r="G206" s="1" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
       <c r="H206" s="1" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="I206" s="1" t="s">
         <v>78</v>
@@ -11942,16 +11942,16 @@
         <v>669</v>
       </c>
       <c r="E207" s="1">
-        <v>679180900</v>
+        <v>144846400</v>
       </c>
       <c r="F207" s="1" t="s">
         <v>710</v>
       </c>
       <c r="G207" s="1" t="s">
-        <v>695</v>
+        <v>688</v>
       </c>
       <c r="H207" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I207" s="1" t="s">
         <v>78</v>
@@ -11978,7 +11978,7 @@
         <v>713</v>
       </c>
       <c r="E208" s="1">
-        <v>34899150</v>
+        <v>279581387</v>
       </c>
       <c r="F208" s="1" t="s">
         <v>714</v>
@@ -11987,7 +11987,7 @@
         <v>713</v>
       </c>
       <c r="H208" s="1" t="s">
-        <v>25</v>
+        <v>135</v>
       </c>
       <c r="I208" s="1" t="s">
         <v>17</v>
@@ -12014,7 +12014,7 @@
         <v>713</v>
       </c>
       <c r="E209" s="1">
-        <v>279581387</v>
+        <v>34899150</v>
       </c>
       <c r="F209" s="1" t="s">
         <v>717</v>
@@ -12023,7 +12023,7 @@
         <v>713</v>
       </c>
       <c r="H209" s="1" t="s">
-        <v>135</v>
+        <v>25</v>
       </c>
       <c r="I209" s="1" t="s">
         <v>17</v>
@@ -12302,7 +12302,7 @@
         <v>730</v>
       </c>
       <c r="E217" s="1">
-        <v>212914412</v>
+        <v>158091056</v>
       </c>
       <c r="F217" s="1" t="s">
         <v>744</v>
@@ -12338,7 +12338,7 @@
         <v>730</v>
       </c>
       <c r="E218" s="1">
-        <v>158091056</v>
+        <v>74276700</v>
       </c>
       <c r="F218" s="1" t="s">
         <v>747</v>
@@ -12347,7 +12347,7 @@
         <v>730</v>
       </c>
       <c r="H218" s="1" t="s">
-        <v>135</v>
+        <v>16</v>
       </c>
       <c r="I218" s="1" t="s">
         <v>17</v>
@@ -12374,7 +12374,7 @@
         <v>730</v>
       </c>
       <c r="E219" s="1">
-        <v>74276700</v>
+        <v>212914412</v>
       </c>
       <c r="F219" s="1" t="s">
         <v>750</v>
@@ -12383,7 +12383,7 @@
         <v>730</v>
       </c>
       <c r="H219" s="1" t="s">
-        <v>16</v>
+        <v>135</v>
       </c>
       <c r="I219" s="1" t="s">
         <v>17</v>
@@ -12410,7 +12410,7 @@
         <v>730</v>
       </c>
       <c r="E220" s="1">
-        <v>100933077</v>
+        <v>1912000</v>
       </c>
       <c r="F220" s="1" t="s">
         <v>754</v>
@@ -12419,13 +12419,13 @@
         <v>753</v>
       </c>
       <c r="H220" s="1" t="s">
-        <v>53</v>
+        <v>129</v>
       </c>
       <c r="I220" s="1" t="s">
         <v>17</v>
       </c>
       <c r="J220" s="1" t="s">
-        <v>54</v>
+        <v>130</v>
       </c>
       <c r="K220" s="1" t="s">
         <v>19</v>
@@ -12446,7 +12446,7 @@
         <v>730</v>
       </c>
       <c r="E221" s="1">
-        <v>1912000</v>
+        <v>100933077</v>
       </c>
       <c r="F221" s="1" t="s">
         <v>756</v>
@@ -12455,13 +12455,13 @@
         <v>753</v>
       </c>
       <c r="H221" s="1" t="s">
-        <v>129</v>
+        <v>53</v>
       </c>
       <c r="I221" s="1" t="s">
         <v>17</v>
       </c>
       <c r="J221" s="1" t="s">
-        <v>130</v>
+        <v>54</v>
       </c>
       <c r="K221" s="1" t="s">
         <v>19</v>
@@ -12698,7 +12698,7 @@
         <v>688</v>
       </c>
       <c r="E228" s="1">
-        <v>3160500</v>
+        <v>337800</v>
       </c>
       <c r="F228" s="1" t="s">
         <v>778</v>
@@ -12734,7 +12734,7 @@
         <v>688</v>
       </c>
       <c r="E229" s="1">
-        <v>337800</v>
+        <v>3160500</v>
       </c>
       <c r="F229" s="1" t="s">
         <v>781</v>
@@ -13202,7 +13202,7 @@
         <v>811</v>
       </c>
       <c r="E242" s="1">
-        <v>200371400</v>
+        <v>177618600</v>
       </c>
       <c r="F242" s="1" t="s">
         <v>828</v>
@@ -13211,7 +13211,7 @@
         <v>829</v>
       </c>
       <c r="H242" s="1" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="I242" s="1" t="s">
         <v>78</v>
@@ -13274,7 +13274,7 @@
         <v>811</v>
       </c>
       <c r="E244" s="1">
-        <v>688714100</v>
+        <v>200371400</v>
       </c>
       <c r="F244" s="1" t="s">
         <v>835</v>
@@ -13283,7 +13283,7 @@
         <v>829</v>
       </c>
       <c r="H244" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I244" s="1" t="s">
         <v>78</v>
@@ -13310,7 +13310,7 @@
         <v>811</v>
       </c>
       <c r="E245" s="1">
-        <v>177618600</v>
+        <v>688714100</v>
       </c>
       <c r="F245" s="1" t="s">
         <v>838</v>
@@ -13526,7 +13526,7 @@
         <v>853</v>
       </c>
       <c r="E251" s="1">
-        <v>158436845</v>
+        <v>845082696</v>
       </c>
       <c r="F251" s="1" t="s">
         <v>857</v>
@@ -13562,7 +13562,7 @@
         <v>853</v>
       </c>
       <c r="E252" s="1">
-        <v>845082696</v>
+        <v>158436845</v>
       </c>
       <c r="F252" s="1" t="s">
         <v>860</v>
@@ -13634,7 +13634,7 @@
         <v>853</v>
       </c>
       <c r="E254" s="1">
-        <v>99929015</v>
+        <v>1055833082</v>
       </c>
       <c r="F254" s="1" t="s">
         <v>866</v>
@@ -13670,7 +13670,7 @@
         <v>853</v>
       </c>
       <c r="E255" s="1">
-        <v>1055833082</v>
+        <v>99929015</v>
       </c>
       <c r="F255" s="1" t="s">
         <v>869</v>
@@ -13958,7 +13958,7 @@
         <v>885</v>
       </c>
       <c r="E263" s="1">
-        <v>24294250</v>
+        <v>90092300</v>
       </c>
       <c r="F263" s="1" t="s">
         <v>895</v>
@@ -14066,7 +14066,7 @@
         <v>885</v>
       </c>
       <c r="E266" s="1">
-        <v>90092300</v>
+        <v>24294250</v>
       </c>
       <c r="F266" s="1" t="s">
         <v>904</v>
@@ -14462,7 +14462,7 @@
         <v>937</v>
       </c>
       <c r="E277" s="1">
-        <v>258570562</v>
+        <v>2548731</v>
       </c>
       <c r="F277" s="1" t="s">
         <v>944</v>
@@ -14534,7 +14534,7 @@
         <v>937</v>
       </c>
       <c r="E279" s="1">
-        <v>2548731</v>
+        <v>258570562</v>
       </c>
       <c r="F279" s="1" t="s">
         <v>950</v>
@@ -14606,7 +14606,7 @@
         <v>937</v>
       </c>
       <c r="E281" s="1">
-        <v>177359200</v>
+        <v>200371400</v>
       </c>
       <c r="F281" s="1" t="s">
         <v>956</v>
@@ -14615,7 +14615,7 @@
         <v>957</v>
       </c>
       <c r="H281" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I281" s="1" t="s">
         <v>78</v>
@@ -14642,7 +14642,7 @@
         <v>937</v>
       </c>
       <c r="E282" s="1">
-        <v>689018800</v>
+        <v>149250700</v>
       </c>
       <c r="F282" s="1" t="s">
         <v>960</v>
@@ -14651,7 +14651,7 @@
         <v>957</v>
       </c>
       <c r="H282" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I282" s="1" t="s">
         <v>78</v>
@@ -14678,7 +14678,7 @@
         <v>937</v>
       </c>
       <c r="E283" s="1">
-        <v>200371400</v>
+        <v>689018800</v>
       </c>
       <c r="F283" s="1" t="s">
         <v>963</v>
@@ -14687,7 +14687,7 @@
         <v>957</v>
       </c>
       <c r="H283" s="1" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="I283" s="1" t="s">
         <v>78</v>
@@ -14714,7 +14714,7 @@
         <v>937</v>
       </c>
       <c r="E284" s="1">
-        <v>149250700</v>
+        <v>177359200</v>
       </c>
       <c r="F284" s="1" t="s">
         <v>966</v>
@@ -14723,7 +14723,7 @@
         <v>957</v>
       </c>
       <c r="H284" s="1" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="I284" s="1" t="s">
         <v>78</v>
@@ -15326,7 +15326,7 @@
         <v>1010</v>
       </c>
       <c r="E301" s="1">
-        <v>667850</v>
+        <v>703000</v>
       </c>
       <c r="F301" s="1" t="s">
         <v>1024</v>
@@ -15362,7 +15362,7 @@
         <v>1010</v>
       </c>
       <c r="E302" s="1">
-        <v>287324950</v>
+        <v>667850</v>
       </c>
       <c r="F302" s="1" t="s">
         <v>1027</v>
@@ -15371,7 +15371,7 @@
         <v>1015</v>
       </c>
       <c r="H302" s="1" t="s">
-        <v>929</v>
+        <v>16</v>
       </c>
       <c r="I302" s="1" t="s">
         <v>17</v>
@@ -15398,7 +15398,7 @@
         <v>1010</v>
       </c>
       <c r="E303" s="1">
-        <v>703000</v>
+        <v>287324950</v>
       </c>
       <c r="F303" s="1" t="s">
         <v>1030</v>
@@ -15407,7 +15407,7 @@
         <v>1015</v>
       </c>
       <c r="H303" s="1" t="s">
-        <v>16</v>
+        <v>929</v>
       </c>
       <c r="I303" s="1" t="s">
         <v>17</v>
@@ -15578,7 +15578,7 @@
         <v>1015</v>
       </c>
       <c r="E308" s="1">
-        <v>267194900</v>
+        <v>960197300</v>
       </c>
       <c r="F308" s="1" t="s">
         <v>1048</v>
@@ -15587,7 +15587,7 @@
         <v>1044</v>
       </c>
       <c r="H308" s="1" t="s">
-        <v>933</v>
+        <v>1045</v>
       </c>
       <c r="I308" s="1" t="s">
         <v>78</v>
@@ -15614,7 +15614,7 @@
         <v>1015</v>
       </c>
       <c r="E309" s="1">
-        <v>960197300</v>
+        <v>267194900</v>
       </c>
       <c r="F309" s="1" t="s">
         <v>1051</v>
@@ -15623,7 +15623,7 @@
         <v>1044</v>
       </c>
       <c r="H309" s="1" t="s">
-        <v>1045</v>
+        <v>933</v>
       </c>
       <c r="I309" s="1" t="s">
         <v>78</v>
@@ -15650,7 +15650,7 @@
         <v>1015</v>
       </c>
       <c r="E310" s="1">
-        <v>762330900</v>
+        <v>4313300</v>
       </c>
       <c r="F310" s="1" t="s">
         <v>1054</v>
@@ -15686,7 +15686,7 @@
         <v>1015</v>
       </c>
       <c r="E311" s="1">
-        <v>4313300</v>
+        <v>193894600</v>
       </c>
       <c r="F311" s="1" t="s">
         <v>1057</v>
@@ -15722,7 +15722,7 @@
         <v>1015</v>
       </c>
       <c r="E312" s="1">
-        <v>63500000</v>
+        <v>762330900</v>
       </c>
       <c r="F312" s="1" t="s">
         <v>1060</v>
@@ -15731,7 +15731,7 @@
         <v>1044</v>
       </c>
       <c r="H312" s="1" t="s">
-        <v>995</v>
+        <v>1045</v>
       </c>
       <c r="I312" s="1" t="s">
         <v>78</v>
@@ -15758,7 +15758,7 @@
         <v>1015</v>
       </c>
       <c r="E313" s="1">
-        <v>151924700</v>
+        <v>63500000</v>
       </c>
       <c r="F313" s="1" t="s">
         <v>1063</v>
@@ -15767,7 +15767,7 @@
         <v>1044</v>
       </c>
       <c r="H313" s="1" t="s">
-        <v>933</v>
+        <v>995</v>
       </c>
       <c r="I313" s="1" t="s">
         <v>78</v>
@@ -15794,7 +15794,7 @@
         <v>1015</v>
       </c>
       <c r="E314" s="1">
-        <v>193894600</v>
+        <v>204133200</v>
       </c>
       <c r="F314" s="1" t="s">
         <v>1066</v>
@@ -15803,7 +15803,7 @@
         <v>1044</v>
       </c>
       <c r="H314" s="1" t="s">
-        <v>1045</v>
+        <v>933</v>
       </c>
       <c r="I314" s="1" t="s">
         <v>78</v>
@@ -15830,7 +15830,7 @@
         <v>1015</v>
       </c>
       <c r="E315" s="1">
-        <v>204133200</v>
+        <v>151924700</v>
       </c>
       <c r="F315" s="1" t="s">
         <v>1069</v>
@@ -16046,7 +16046,7 @@
         <v>1072</v>
       </c>
       <c r="E321" s="1">
-        <v>5246000</v>
+        <v>1067934069</v>
       </c>
       <c r="F321" s="1" t="s">
         <v>1088</v>
@@ -16055,13 +16055,13 @@
         <v>957</v>
       </c>
       <c r="H321" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="I321" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="J321" s="1" t="s">
         <v>1089</v>
-      </c>
-      <c r="I321" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="J321" s="1" t="s">
-        <v>1090</v>
       </c>
       <c r="K321" s="1" t="s">
         <v>19</v>
@@ -16073,7 +16073,7 @@
         <v>319</v>
       </c>
       <c r="B322" s="1" t="s">
-        <v>1091</v>
+        <v>1090</v>
       </c>
       <c r="C322" s="1" t="s">
         <v>1072</v>
@@ -16082,16 +16082,16 @@
         <v>1072</v>
       </c>
       <c r="E322" s="1">
-        <v>1067934069</v>
+        <v>5246000</v>
       </c>
       <c r="F322" s="1" t="s">
-        <v>1092</v>
+        <v>1091</v>
       </c>
       <c r="G322" s="1" t="s">
         <v>957</v>
       </c>
       <c r="H322" s="1" t="s">
-        <v>135</v>
+        <v>1092</v>
       </c>
       <c r="I322" s="1" t="s">
         <v>17</v>
@@ -16118,7 +16118,7 @@
         <v>1072</v>
       </c>
       <c r="E323" s="1">
-        <v>94750900</v>
+        <v>25170300</v>
       </c>
       <c r="F323" s="1" t="s">
         <v>1095</v>
@@ -16190,7 +16190,7 @@
         <v>1072</v>
       </c>
       <c r="E325" s="1">
-        <v>25170300</v>
+        <v>94750900</v>
       </c>
       <c r="F325" s="1" t="s">
         <v>1101</v>
@@ -16298,7 +16298,7 @@
         <v>1072</v>
       </c>
       <c r="E328" s="1">
-        <v>44072100</v>
+        <v>279548291</v>
       </c>
       <c r="F328" s="1" t="s">
         <v>1110</v>
@@ -16307,7 +16307,7 @@
         <v>957</v>
       </c>
       <c r="H328" s="1" t="s">
-        <v>25</v>
+        <v>135</v>
       </c>
       <c r="I328" s="1" t="s">
         <v>17</v>
@@ -16334,7 +16334,7 @@
         <v>1072</v>
       </c>
       <c r="E329" s="1">
-        <v>279548291</v>
+        <v>44072100</v>
       </c>
       <c r="F329" s="1" t="s">
         <v>1113</v>
@@ -16343,7 +16343,7 @@
         <v>957</v>
       </c>
       <c r="H329" s="1" t="s">
-        <v>135</v>
+        <v>25</v>
       </c>
       <c r="I329" s="1" t="s">
         <v>17</v>
@@ -16523,7 +16523,7 @@
         <v>1121</v>
       </c>
       <c r="H334" s="1" t="s">
-        <v>1089</v>
+        <v>1092</v>
       </c>
       <c r="I334" s="1" t="s">
         <v>17</v>
@@ -16766,7 +16766,7 @@
         <v>1154</v>
       </c>
       <c r="E341" s="1">
-        <v>116066650</v>
+        <v>279584469</v>
       </c>
       <c r="F341" s="1" t="s">
         <v>1155</v>
@@ -16775,7 +16775,7 @@
         <v>1153</v>
       </c>
       <c r="H341" s="1" t="s">
-        <v>16</v>
+        <v>135</v>
       </c>
       <c r="I341" s="1" t="s">
         <v>17</v>
@@ -16838,7 +16838,7 @@
         <v>1154</v>
       </c>
       <c r="E343" s="1">
-        <v>279584469</v>
+        <v>41365850</v>
       </c>
       <c r="F343" s="1" t="s">
         <v>1161</v>
@@ -16847,7 +16847,7 @@
         <v>1153</v>
       </c>
       <c r="H343" s="1" t="s">
-        <v>135</v>
+        <v>25</v>
       </c>
       <c r="I343" s="1" t="s">
         <v>17</v>
@@ -16874,7 +16874,7 @@
         <v>1154</v>
       </c>
       <c r="E344" s="1">
-        <v>41365850</v>
+        <v>116066650</v>
       </c>
       <c r="F344" s="1" t="s">
         <v>1164</v>
@@ -16883,7 +16883,7 @@
         <v>1153</v>
       </c>
       <c r="H344" s="1" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="I344" s="1" t="s">
         <v>17</v>
@@ -17054,22 +17054,22 @@
         <v>1168</v>
       </c>
       <c r="E349" s="1">
-        <v>177151200</v>
+        <v>149250700</v>
       </c>
       <c r="F349" s="1" t="s">
         <v>1183</v>
       </c>
       <c r="G349" s="1" t="s">
-        <v>1180</v>
+        <v>1184</v>
       </c>
       <c r="H349" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I349" s="1" t="s">
         <v>78</v>
       </c>
       <c r="J349" s="1" t="s">
-        <v>1184</v>
+        <v>1185</v>
       </c>
       <c r="K349" s="1" t="s">
         <v>19</v>
@@ -17081,7 +17081,7 @@
         <v>347</v>
       </c>
       <c r="B350" s="1" t="s">
-        <v>1185</v>
+        <v>1186</v>
       </c>
       <c r="C350" s="1" t="s">
         <v>1170</v>
@@ -17090,16 +17090,16 @@
         <v>1168</v>
       </c>
       <c r="E350" s="1">
-        <v>149250700</v>
+        <v>689692300</v>
       </c>
       <c r="F350" s="1" t="s">
-        <v>1186</v>
+        <v>1187</v>
       </c>
       <c r="G350" s="1" t="s">
-        <v>1187</v>
+        <v>1180</v>
       </c>
       <c r="H350" s="1" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="I350" s="1" t="s">
         <v>78</v>
@@ -17162,22 +17162,22 @@
         <v>1168</v>
       </c>
       <c r="E352" s="1">
-        <v>62679696</v>
+        <v>177151200</v>
       </c>
       <c r="F352" s="1" t="s">
         <v>1193</v>
       </c>
       <c r="G352" s="1" t="s">
-        <v>1194</v>
+        <v>1180</v>
       </c>
       <c r="H352" s="1" t="s">
-        <v>77</v>
+        <v>97</v>
       </c>
       <c r="I352" s="1" t="s">
         <v>78</v>
       </c>
       <c r="J352" s="1" t="s">
-        <v>1195</v>
+        <v>1194</v>
       </c>
       <c r="K352" s="1" t="s">
         <v>19</v>
@@ -17189,7 +17189,7 @@
         <v>350</v>
       </c>
       <c r="B353" s="1" t="s">
-        <v>1196</v>
+        <v>1195</v>
       </c>
       <c r="C353" s="1" t="s">
         <v>1170</v>
@@ -17198,16 +17198,16 @@
         <v>1168</v>
       </c>
       <c r="E353" s="1">
-        <v>689692300</v>
+        <v>62679696</v>
       </c>
       <c r="F353" s="1" t="s">
+        <v>1196</v>
+      </c>
+      <c r="G353" s="1" t="s">
         <v>1197</v>
       </c>
-      <c r="G353" s="1" t="s">
-        <v>1180</v>
-      </c>
       <c r="H353" s="1" t="s">
-        <v>97</v>
+        <v>77</v>
       </c>
       <c r="I353" s="1" t="s">
         <v>78</v>
@@ -17240,7 +17240,7 @@
         <v>1200</v>
       </c>
       <c r="G354" s="1" t="s">
-        <v>1187</v>
+        <v>1184</v>
       </c>
       <c r="H354" s="1" t="s">
         <v>101</v>
@@ -17267,7 +17267,7 @@
         <v>1203</v>
       </c>
       <c r="D355" s="1" t="s">
-        <v>1194</v>
+        <v>1197</v>
       </c>
       <c r="E355" s="1">
         <v>258570562</v>
@@ -17303,7 +17303,7 @@
         <v>1180</v>
       </c>
       <c r="D356" s="1" t="s">
-        <v>1187</v>
+        <v>1184</v>
       </c>
       <c r="E356" s="1">
         <v>837896759</v>
@@ -17339,10 +17339,10 @@
         <v>1180</v>
       </c>
       <c r="D357" s="1" t="s">
-        <v>1187</v>
+        <v>1184</v>
       </c>
       <c r="E357" s="1">
-        <v>213243288</v>
+        <v>158575478</v>
       </c>
       <c r="F357" s="1" t="s">
         <v>1210</v>
@@ -17375,10 +17375,10 @@
         <v>1180</v>
       </c>
       <c r="D358" s="1" t="s">
-        <v>1187</v>
+        <v>1184</v>
       </c>
       <c r="E358" s="1">
-        <v>158575478</v>
+        <v>213243288</v>
       </c>
       <c r="F358" s="1" t="s">
         <v>1213</v>
@@ -17414,7 +17414,7 @@
         <v>1180</v>
       </c>
       <c r="E359" s="1">
-        <v>22608400</v>
+        <v>24034050</v>
       </c>
       <c r="F359" s="1" t="s">
         <v>1217</v>
@@ -17423,7 +17423,7 @@
         <v>1218</v>
       </c>
       <c r="H359" s="1" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="I359" s="1" t="s">
         <v>17</v>
@@ -17450,7 +17450,7 @@
         <v>1180</v>
       </c>
       <c r="E360" s="1">
-        <v>24034050</v>
+        <v>22608400</v>
       </c>
       <c r="F360" s="1" t="s">
         <v>1221</v>
@@ -17459,7 +17459,7 @@
         <v>1218</v>
       </c>
       <c r="H360" s="1" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="I360" s="1" t="s">
         <v>17</v>
@@ -17522,16 +17522,16 @@
         <v>1180</v>
       </c>
       <c r="E362" s="1">
-        <v>89459600</v>
+        <v>33188550</v>
       </c>
       <c r="F362" s="1" t="s">
         <v>1228</v>
       </c>
       <c r="G362" s="1" t="s">
-        <v>1224</v>
+        <v>1218</v>
       </c>
       <c r="H362" s="1" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="I362" s="1" t="s">
         <v>17</v>
@@ -17558,16 +17558,16 @@
         <v>1180</v>
       </c>
       <c r="E363" s="1">
-        <v>33188550</v>
+        <v>89459600</v>
       </c>
       <c r="F363" s="1" t="s">
         <v>1231</v>
       </c>
       <c r="G363" s="1" t="s">
-        <v>1218</v>
+        <v>1224</v>
       </c>
       <c r="H363" s="1" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="I363" s="1" t="s">
         <v>17</v>
@@ -17699,7 +17699,7 @@
         <v>1242</v>
       </c>
       <c r="D367" s="1" t="s">
-        <v>1187</v>
+        <v>1184</v>
       </c>
       <c r="E367" s="1">
         <v>60825925</v>
@@ -17735,7 +17735,7 @@
         <v>1242</v>
       </c>
       <c r="D368" s="1" t="s">
-        <v>1187</v>
+        <v>1184</v>
       </c>
       <c r="E368" s="1">
         <v>2844264</v>
@@ -17774,7 +17774,7 @@
         <v>1242</v>
       </c>
       <c r="E369" s="1">
-        <v>34511892</v>
+        <v>12740000</v>
       </c>
       <c r="F369" s="1" t="s">
         <v>1250</v>
@@ -17810,7 +17810,7 @@
         <v>1242</v>
       </c>
       <c r="E370" s="1">
-        <v>12740000</v>
+        <v>34511892</v>
       </c>
       <c r="F370" s="1" t="s">
         <v>1253</v>
@@ -18206,7 +18206,7 @@
         <v>1289</v>
       </c>
       <c r="E381" s="1">
-        <v>3915950</v>
+        <v>161741108</v>
       </c>
       <c r="F381" s="1" t="s">
         <v>1293</v>
@@ -18242,7 +18242,7 @@
         <v>1289</v>
       </c>
       <c r="E382" s="1">
-        <v>161741108</v>
+        <v>3915950</v>
       </c>
       <c r="F382" s="1" t="s">
         <v>1296</v>
@@ -18314,7 +18314,7 @@
         <v>1284</v>
       </c>
       <c r="E384" s="1">
-        <v>679200</v>
+        <v>3915950</v>
       </c>
       <c r="F384" s="1" t="s">
         <v>1302</v>
@@ -18323,7 +18323,7 @@
         <v>1288</v>
       </c>
       <c r="H384" s="1" t="s">
-        <v>803</v>
+        <v>135</v>
       </c>
       <c r="I384" s="1" t="s">
         <v>17</v>
@@ -18350,7 +18350,7 @@
         <v>1284</v>
       </c>
       <c r="E385" s="1">
-        <v>3915950</v>
+        <v>679200</v>
       </c>
       <c r="F385" s="1" t="s">
         <v>1305</v>
@@ -18359,7 +18359,7 @@
         <v>1288</v>
       </c>
       <c r="H385" s="1" t="s">
-        <v>135</v>
+        <v>803</v>
       </c>
       <c r="I385" s="1" t="s">
         <v>17</v>
@@ -18422,7 +18422,7 @@
         <v>1312</v>
       </c>
       <c r="E387" s="1">
-        <v>346500</v>
+        <v>4759600</v>
       </c>
       <c r="F387" s="1" t="s">
         <v>1313</v>
@@ -18431,7 +18431,7 @@
         <v>1308</v>
       </c>
       <c r="H387" s="1" t="s">
-        <v>42</v>
+        <v>1092</v>
       </c>
       <c r="I387" s="1" t="s">
         <v>17</v>
@@ -18458,7 +18458,7 @@
         <v>1312</v>
       </c>
       <c r="E388" s="1">
-        <v>4759600</v>
+        <v>346500</v>
       </c>
       <c r="F388" s="1" t="s">
         <v>1316</v>
@@ -18467,7 +18467,7 @@
         <v>1308</v>
       </c>
       <c r="H388" s="1" t="s">
-        <v>1089</v>
+        <v>42</v>
       </c>
       <c r="I388" s="1" t="s">
         <v>17</v>
@@ -18566,22 +18566,22 @@
         <v>1289</v>
       </c>
       <c r="E391" s="1">
-        <v>199981800</v>
+        <v>694524200</v>
       </c>
       <c r="F391" s="1" t="s">
         <v>1327</v>
       </c>
       <c r="G391" s="1" t="s">
-        <v>1324</v>
+        <v>1328</v>
       </c>
       <c r="H391" s="1" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="I391" s="1" t="s">
         <v>78</v>
       </c>
       <c r="J391" s="1" t="s">
-        <v>1328</v>
+        <v>1329</v>
       </c>
       <c r="K391" s="1" t="s">
         <v>19</v>
@@ -18593,7 +18593,7 @@
         <v>389</v>
       </c>
       <c r="B392" s="1" t="s">
-        <v>1329</v>
+        <v>1330</v>
       </c>
       <c r="C392" s="1" t="s">
         <v>1322</v>
@@ -18605,10 +18605,10 @@
         <v>176866300</v>
       </c>
       <c r="F392" s="1" t="s">
-        <v>1330</v>
+        <v>1331</v>
       </c>
       <c r="G392" s="1" t="s">
-        <v>1331</v>
+        <v>1328</v>
       </c>
       <c r="H392" s="1" t="s">
         <v>97</v>
@@ -18638,16 +18638,16 @@
         <v>1289</v>
       </c>
       <c r="E393" s="1">
-        <v>694524200</v>
+        <v>199981800</v>
       </c>
       <c r="F393" s="1" t="s">
         <v>1334</v>
       </c>
       <c r="G393" s="1" t="s">
-        <v>1331</v>
+        <v>1324</v>
       </c>
       <c r="H393" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I393" s="1" t="s">
         <v>78</v>
@@ -18680,7 +18680,7 @@
         <v>1337</v>
       </c>
       <c r="G394" s="1" t="s">
-        <v>1331</v>
+        <v>1328</v>
       </c>
       <c r="H394" s="1" t="s">
         <v>97</v>
@@ -18752,7 +18752,7 @@
         <v>1343</v>
       </c>
       <c r="G396" s="1" t="s">
-        <v>1331</v>
+        <v>1328</v>
       </c>
       <c r="H396" s="1" t="s">
         <v>97</v>
@@ -18788,7 +18788,7 @@
         <v>1348</v>
       </c>
       <c r="G397" s="1" t="s">
-        <v>1331</v>
+        <v>1328</v>
       </c>
       <c r="H397" s="1" t="s">
         <v>17</v>
@@ -18818,7 +18818,7 @@
         <v>1352</v>
       </c>
       <c r="E398" s="1">
-        <v>120000000</v>
+        <v>4759600</v>
       </c>
       <c r="F398" s="1" t="s">
         <v>1353</v>
@@ -18827,13 +18827,13 @@
         <v>1351</v>
       </c>
       <c r="H398" s="1" t="s">
+        <v>1092</v>
+      </c>
+      <c r="I398" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="J398" s="1" t="s">
         <v>1354</v>
-      </c>
-      <c r="I398" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="J398" s="1" t="s">
-        <v>1355</v>
       </c>
       <c r="K398" s="1" t="s">
         <v>19</v>
@@ -18845,7 +18845,7 @@
         <v>396</v>
       </c>
       <c r="B399" s="1" t="s">
-        <v>1356</v>
+        <v>1355</v>
       </c>
       <c r="C399" s="1" t="s">
         <v>1351</v>
@@ -18854,16 +18854,16 @@
         <v>1352</v>
       </c>
       <c r="E399" s="1">
-        <v>4759600</v>
+        <v>120000000</v>
       </c>
       <c r="F399" s="1" t="s">
-        <v>1357</v>
+        <v>1356</v>
       </c>
       <c r="G399" s="1" t="s">
         <v>1351</v>
       </c>
       <c r="H399" s="1" t="s">
-        <v>1089</v>
+        <v>1357</v>
       </c>
       <c r="I399" s="1" t="s">
         <v>17</v>

</xml_diff>

<commit_message>
perbaikan akrual 14 okt
perbaikan akrual 14 okt
</commit_message>
<xml_diff>
--- a/Database/DAFTAR SP2D SATKER.xlsx
+++ b/Database/DAFTAR SP2D SATKER.xlsx
@@ -725,28 +725,40 @@
     <t>00363T/403829/2025</t>
   </si>
   <si>
+    <t xml:space="preserve"> 259991530041992</t>
+  </si>
+  <si>
+    <t>19-08-2025</t>
+  </si>
+  <si>
+    <t>00340T/403829/2025</t>
+  </si>
+  <si>
+    <t>11-08-2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan September 2025 untuk 131 Pegawai/384 Jiwa</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 259991530041993</t>
   </si>
   <si>
-    <t>19-08-2025</t>
-  </si>
-  <si>
     <t>00335T/403829/2025</t>
   </si>
   <si>
-    <t>11-08-2025</t>
-  </si>
-  <si>
     <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan September 2025 untuk 50 Pegawai/125 Jiwa</t>
   </si>
   <si>
-    <t xml:space="preserve"> 259991530041992</t>
-  </si>
-  <si>
-    <t>00340T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan September 2025 untuk 131 Pegawai/384 Jiwa</t>
+    <t xml:space="preserve"> 259991530041991</t>
+  </si>
+  <si>
+    <t>00354T/403829/2025</t>
+  </si>
+  <si>
+    <t>15-08-2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan September 2025 untuk 37 Pegawai/103 Jiwa</t>
   </si>
   <si>
     <t xml:space="preserve"> 259991530041994</t>
@@ -758,18 +770,6 @@
     <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan September 2025 untuk 35 Pegawai/101 Jiwa</t>
   </si>
   <si>
-    <t xml:space="preserve"> 259991530041991</t>
-  </si>
-  <si>
-    <t>00354T/403829/2025</t>
-  </si>
-  <si>
-    <t>15-08-2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan September 2025 untuk 37 Pegawai/103 Jiwa</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 259991525018157</t>
   </si>
   <si>
@@ -779,6 +779,15 @@
     <t>Pembayaran Belanja Pegawai berupa Gaji Induk bulan September 2025 untuk 4 Pegawai/16 Jiwa</t>
   </si>
   <si>
+    <t xml:space="preserve"> 259991531008985</t>
+  </si>
+  <si>
+    <t>00336T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan September 2025  untuk 63 Pegawai/181 jiwa</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 259991531008984</t>
   </si>
   <si>
@@ -797,13 +806,22 @@
     <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan September 2025 untuk 23 Pegawai/52 jiwa</t>
   </si>
   <si>
-    <t xml:space="preserve"> 259991531008985</t>
-  </si>
-  <si>
-    <t>00336T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan September 2025  untuk 63 Pegawai/181 jiwa</t>
+    <t xml:space="preserve"> 259991310471406</t>
+  </si>
+  <si>
+    <t>00361T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran tunjangan kinerja bulan Juli tahun 2025 untuk 35 Pegawai</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 259991310471404</t>
+  </si>
+  <si>
+    <t>00357T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran tunjangan kinerja bulan JULI tahun 2025 untuk 134 Pegawai</t>
   </si>
   <si>
     <t xml:space="preserve"> 259991310471405</t>
@@ -815,24 +833,6 @@
     <t>Pembayaran tunjangan kinerja bulan Juli tahun 2025 untuk 50 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 259991310471406</t>
-  </si>
-  <si>
-    <t>00361T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran tunjangan kinerja bulan Juli tahun 2025 untuk 35 Pegawai</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 259991310471404</t>
-  </si>
-  <si>
-    <t>00357T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran tunjangan kinerja bulan JULI tahun 2025 untuk 134 Pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 259991330150985</t>
   </si>
   <si>
@@ -1121,21 +1121,39 @@
     <t>Pembayaran Belanja Barang Berupa Honor PPNPN Bulan Juli Tahun 2025 untuk 91 Pegawai.Sesuai Sk No 9 Tahun 2025 Tanggal 6 Januari 2025</t>
   </si>
   <si>
+    <t xml:space="preserve"> 259991530020755</t>
+  </si>
+  <si>
+    <t>17-07-2025</t>
+  </si>
+  <si>
+    <t>00299T/403829/2025</t>
+  </si>
+  <si>
+    <t>09-07-2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan Agustus 2025 untuk 50 Pegawai/124 jiwa</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 259991530020754</t>
   </si>
   <si>
-    <t>17-07-2025</t>
-  </si>
-  <si>
     <t>00309T/403829/2025</t>
   </si>
   <si>
-    <t>09-07-2025</t>
-  </si>
-  <si>
     <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan Agustus 2025 untuk 132 Pegawai/388 Jiwa</t>
   </si>
   <si>
+    <t xml:space="preserve"> 259991530020756</t>
+  </si>
+  <si>
+    <t>00301T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK bulan Agustus 2025 untuk 35 Pegawai/101 Jiwa</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 259991530020753</t>
   </si>
   <si>
@@ -1145,24 +1163,6 @@
     <t>Pembayaran Belanja Pegawai berupa Gaji induk Bulan Agustus 2025 untuk 38 Pegawai/107 Jiwa</t>
   </si>
   <si>
-    <t xml:space="preserve"> 259991530020756</t>
-  </si>
-  <si>
-    <t>00301T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK bulan Agustus 2025 untuk 35 Pegawai/101 Jiwa</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 259991530020755</t>
-  </si>
-  <si>
-    <t>00299T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan Agustus 2025 untuk 50 Pegawai/124 jiwa</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 259991531004439</t>
   </si>
   <si>
@@ -1205,25 +1205,43 @@
     <t>Pembayaran Belanja Barang sesuai SPD No. 0023-0037/BRPBATPP/KP.440/VII/2025 Tanggal 19 April 2025 sd 07 Juli 2025</t>
   </si>
   <si>
+    <t xml:space="preserve"> 259991310239038</t>
+  </si>
+  <si>
+    <t>11-07-2025</t>
+  </si>
+  <si>
+    <t>00315T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran tunjangan kinerja bulan Juni tahun 2025 untuk 134 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 259991310239039</t>
   </si>
   <si>
-    <t>11-07-2025</t>
-  </si>
-  <si>
     <t>00318T/403829/2025</t>
   </si>
   <si>
     <t>Pembayaran tunjangan kinerja bulan Juni tahun 2025 untuk 35 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 259991310239038</t>
-  </si>
-  <si>
-    <t>00315T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran tunjangan kinerja bulan Juni tahun 2025 untuk 134 Pegawai</t>
+    <t xml:space="preserve"> 259991330071753</t>
+  </si>
+  <si>
+    <t>00316T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran tunjangan kinerja bulan Juni tahun 2025 untuk 174 Pegawai</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 259991330071754</t>
+  </si>
+  <si>
+    <t>00317T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran tunjangan kinerja bulan Juni tahun 2025 untuk 63 Pegawai</t>
   </si>
   <si>
     <t xml:space="preserve"> 259991330071755</t>
@@ -1235,24 +1253,6 @@
     <t>Pembayaran tunjangan kinerja bulan Juni tahun 2025 untuk 23 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 259991330071754</t>
-  </si>
-  <si>
-    <t>00317T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran tunjangan kinerja bulan Juni tahun 2025 untuk 63 Pegawai</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 259991330071753</t>
-  </si>
-  <si>
-    <t>00316T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran tunjangan kinerja bulan Juni tahun 2025 untuk 174 Pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 259991310238647</t>
   </si>
   <si>
@@ -1262,45 +1262,45 @@
     <t>Pembayaran tunjangan kinerja bulan Juni tahun 2025 untuk 50 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 259991310222991</t>
+  </si>
+  <si>
+    <t>10-07-2025</t>
+  </si>
+  <si>
+    <t>00314T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Juni 2025 untuk 37 Pegawai</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 259991310222990</t>
+  </si>
+  <si>
+    <t>00313T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Juni 2025 untuk 132 Pegawai</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 259991310222992</t>
+  </si>
+  <si>
+    <t>00304T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Uang Makan PPPK Bulan Juni 2025 untuk 50 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 259991310222993</t>
   </si>
   <si>
-    <t>10-07-2025</t>
-  </si>
-  <si>
     <t>00305T/403829/2025</t>
   </si>
   <si>
     <t>Pembayaran Belanja Pegawai berupa Uang Makan PPPK Bulan Juni 2025 untuk 34 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 259991310222991</t>
-  </si>
-  <si>
-    <t>00314T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Juni 2025 untuk 37 Pegawai</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 259991310222992</t>
-  </si>
-  <si>
-    <t>00304T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Uang Makan PPPK Bulan Juni 2025 untuk 50 Pegawai</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 259991310222990</t>
-  </si>
-  <si>
-    <t>00313T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Juni 2025 untuk 132 Pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 259991305050216</t>
   </si>
   <si>
@@ -1310,6 +1310,24 @@
     <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Juni 2025 untuk 2 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 259991330066246</t>
+  </si>
+  <si>
+    <t>00312T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Juni 2025 untuk 172 Pegawai</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 259991330066247</t>
+  </si>
+  <si>
+    <t>00306T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Uang Makan PPPK Bulan Juni 2025  untuk 62 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 259991330066248</t>
   </si>
   <si>
@@ -1319,24 +1337,6 @@
     <t>Pembayaran Belanja Pegawai berupa Uang Makan PPPK Bulan Juni 2025  untuk 22 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 259991330066246</t>
-  </si>
-  <si>
-    <t>00312T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Juni 2025 untuk 172 Pegawai</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 259991330066247</t>
-  </si>
-  <si>
-    <t>00306T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Uang Makan PPPK Bulan Juni 2025  untuk 62 Pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 259991310213072</t>
   </si>
   <si>
@@ -1403,27 +1403,27 @@
     <t>Pembayaran Tukin ke-13 Tahun 2025 Untuk 1 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 259991330045565</t>
+  </si>
+  <si>
+    <t>00292T/403829/2025</t>
+  </si>
+  <si>
+    <t>01-07-2025</t>
+  </si>
+  <si>
+    <t>Pembayaran tunjangan kinerja  bulan Mei tahun 2025 untuk 1 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 259991330045564</t>
   </si>
   <si>
     <t>00291T/403829/2025</t>
   </si>
   <si>
-    <t>01-07-2025</t>
-  </si>
-  <si>
     <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Mei 2025 untuk 1 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 259991330045565</t>
-  </si>
-  <si>
-    <t>00292T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran tunjangan kinerja  bulan Mei tahun 2025 untuk 1 Pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 259991310150031</t>
   </si>
   <si>
@@ -1454,48 +1454,48 @@
     <t>00288T/403829/2025</t>
   </si>
   <si>
+    <t xml:space="preserve"> 259991530018167</t>
+  </si>
+  <si>
+    <t>25-06-2025</t>
+  </si>
+  <si>
+    <t>00271T/403829/2025</t>
+  </si>
+  <si>
+    <t>11-06-2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan Juli 2025 untuk 135 Pegawai/396 jiwa</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 259991530018168</t>
+  </si>
+  <si>
+    <t>00265T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan Juli 2025 untuk 50 Pegawai/124 Jiwa</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 259991530018169</t>
+  </si>
+  <si>
+    <t>00267T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan Juli 2025 untuk 35 Pegawai/101 Jiwa</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 259991530018166</t>
   </si>
   <si>
-    <t>25-06-2025</t>
-  </si>
-  <si>
     <t>00270T/403829/2025</t>
   </si>
   <si>
-    <t>11-06-2025</t>
-  </si>
-  <si>
     <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan Juli 2025 untuk 39 Pegawai/111 Jiwa</t>
   </si>
   <si>
-    <t xml:space="preserve"> 259991530018167</t>
-  </si>
-  <si>
-    <t>00271T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan Juli 2025 untuk 135 Pegawai/396 jiwa</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 259991530018169</t>
-  </si>
-  <si>
-    <t>00267T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan Juli 2025 untuk 35 Pegawai/101 Jiwa</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 259991530018168</t>
-  </si>
-  <si>
-    <t>00265T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan Juli 2025 untuk 50 Pegawai/124 Jiwa</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 259991310116799</t>
   </si>
   <si>
@@ -1520,6 +1520,15 @@
     <t>Pembayaran tunjangan kinerja bulan Juli tahun 2025 untuk 2 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 259991530011369</t>
+  </si>
+  <si>
+    <t>00285T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Barang Berupa Honor PPNPN Bulan Juni Tahun 2025 untuk 16 Pegawai.Sesuai Sk No. B.4/BRPBATPP/KP.340/I/2025 Tanggal 2 Januari 2025</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 259991530011368</t>
   </si>
   <si>
@@ -1529,13 +1538,34 @@
     <t>Pembayaran Belanja Barang Berupa Honor PPNPN Bulan Juni Tahun 2025 untuk 103 Pegawai.Sesuai Sk No.9 Tahun 2025 Tanggal 6 Januari 2025</t>
   </si>
   <si>
-    <t xml:space="preserve"> 259991530011369</t>
-  </si>
-  <si>
-    <t>00285T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Barang Berupa Honor PPNPN Bulan Juni Tahun 2025 untuk 16 Pegawai.Sesuai Sk No. B.4/BRPBATPP/KP.340/I/2025 Tanggal 2 Januari 2025</t>
+    <t xml:space="preserve"> 259991531001971</t>
+  </si>
+  <si>
+    <t>00287T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Barang Berupa Honor PPNPN Bulan Juni Tahun 2025 untuk 91 Pegawai.Sesuai Sk No.9 Tahun 2025 Tanggal 6 Januari 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 259991531001949</t>
+  </si>
+  <si>
+    <t>00268T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan Juli 2025 untuk 23 Pegawai/52 Jiwa</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 259991531001947</t>
+  </si>
+  <si>
+    <t>00282T/403829/2025</t>
+  </si>
+  <si>
+    <t>19-06-2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan Juli 2025 untuk 173 Pegawai/538 Jiwa</t>
   </si>
   <si>
     <t xml:space="preserve"> 259991531001948</t>
@@ -1547,36 +1577,6 @@
     <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan Juli 2025 untuk 63 Pegawai/181 Jiwa</t>
   </si>
   <si>
-    <t xml:space="preserve"> 259991531001947</t>
-  </si>
-  <si>
-    <t>00282T/403829/2025</t>
-  </si>
-  <si>
-    <t>19-06-2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan Juli 2025 untuk 173 Pegawai/538 Jiwa</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 259991531001949</t>
-  </si>
-  <si>
-    <t>00268T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan Juli 2025 untuk 23 Pegawai/52 Jiwa</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 259991531001971</t>
-  </si>
-  <si>
-    <t>00287T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Barang Berupa Honor PPNPN Bulan Juni Tahun 2025 untuk 91 Pegawai.Sesuai Sk No.9 Tahun 2025 Tanggal 6 Januari 2025</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 259991525004591</t>
   </si>
   <si>
@@ -1598,37 +1598,55 @@
     <t>Penjualan Belanja Pegawai berupa Kekurangan Gaji Bulan Januari 2025 untuk 1 Pegawai/3 Jiwa</t>
   </si>
   <si>
+    <t xml:space="preserve"> 259991310059125</t>
+  </si>
+  <si>
+    <t>13-06-2025</t>
+  </si>
+  <si>
+    <t>16-06-2025</t>
+  </si>
+  <si>
+    <t>00277T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran tunjangan kinerja bulan Mei tahun 2025 untuk 50 Pegawai</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 259991310059126</t>
+  </si>
+  <si>
+    <t>00280T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran tunjangan kinerja bulan Mei tahun 2025 untuk 35 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 259991310059124</t>
   </si>
   <si>
-    <t>13-06-2025</t>
-  </si>
-  <si>
-    <t>16-06-2025</t>
-  </si>
-  <si>
     <t>00275T/403829/2025</t>
   </si>
   <si>
     <t>Pembayaran tunjangan kinerja  bulan Mei tahun 2025 untuk 137 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 259991310059125</t>
-  </si>
-  <si>
-    <t>00277T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran tunjangan kinerja bulan Mei tahun 2025 untuk 50 Pegawai</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 259991310059126</t>
-  </si>
-  <si>
-    <t>00280T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran tunjangan kinerja bulan Mei tahun 2025 untuk 35 Pegawai</t>
+    <t xml:space="preserve"> 259991330013161</t>
+  </si>
+  <si>
+    <t>00278T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran tunjangan kinerja bulan Mei tahun 2025 untuk 63 Pegawai</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 259991330013162</t>
+  </si>
+  <si>
+    <t>00279T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran tunjangan kinerja bulan Mei tahun 2025 untuk 23 Pegawai</t>
   </si>
   <si>
     <t xml:space="preserve"> 259991330013160</t>
@@ -1640,24 +1658,6 @@
     <t>Pembayaran tunjangan kinerja bulan Mei tahun 2025 untuk 173 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 259991330013162</t>
-  </si>
-  <si>
-    <t>00279T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran tunjangan kinerja bulan Mei tahun 2025 untuk 23 Pegawai</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 259991330013161</t>
-  </si>
-  <si>
-    <t>00278T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran tunjangan kinerja bulan Mei tahun 2025 untuk 63 Pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 259991320016562</t>
   </si>
   <si>
@@ -1670,18 +1670,18 @@
     <t>Pembayaran Belanja Barang berupa Tagihan Internet Bulan Mei 2025 idpel No.GO18A106 An Balai Riset Perikanan Budidaya Air Tawar dan Penyuluhan Perikanan</t>
   </si>
   <si>
+    <t xml:space="preserve"> 259991310050295</t>
+  </si>
+  <si>
+    <t>00274T/403829/2025</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 259991310050294</t>
   </si>
   <si>
     <t>00273T/403829/2025</t>
   </si>
   <si>
-    <t xml:space="preserve"> 259991310050295</t>
-  </si>
-  <si>
-    <t>00274T/403829/2025</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 259991310039873</t>
   </si>
   <si>
@@ -1721,15 +1721,24 @@
     <t>Pembayaran Belanja Pegawai berupa Kekurangan Gaji Bulan April 2025 sd Mei 2025 untuk 11 Pegawai/41 Jiwa</t>
   </si>
   <si>
+    <t xml:space="preserve"> 259991310036823</t>
+  </si>
+  <si>
+    <t>00252T/403829/2025</t>
+  </si>
+  <si>
+    <t>05-06-2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Kekurangan Gaji Bulan April 2025 sd Mei 2025 untuk 2 Pegawai/5 Jiwa</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 259991310036822</t>
   </si>
   <si>
     <t>00256T/403829/2025</t>
   </si>
   <si>
-    <t>05-06-2025</t>
-  </si>
-  <si>
     <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Mei 2025 untuk 38 Jiwa</t>
   </si>
   <si>
@@ -1751,13 +1760,13 @@
     <t>Pembayaran Belanja Pegawai berupa Kekurangan Gaji bulan Mei 2025 untuk 2 pegawai/ 4 Jiwa</t>
   </si>
   <si>
-    <t xml:space="preserve"> 259991310036823</t>
-  </si>
-  <si>
-    <t>00252T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Kekurangan Gaji Bulan April 2025 sd Mei 2025 untuk 2 Pegawai/5 Jiwa</t>
+    <t xml:space="preserve"> 259991330008175</t>
+  </si>
+  <si>
+    <t>00253T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Kekurangan Gaji Bulan Juni 2025 untuk 1 Pegawai/1 Jiwa</t>
   </si>
   <si>
     <t xml:space="preserve"> 259991330008176</t>
@@ -1769,15 +1778,6 @@
     <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Mei 2025 untuk 171 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 259991330008175</t>
-  </si>
-  <si>
-    <t>00253T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Kekurangan Gaji Bulan Juni 2025 untuk 1 Pegawai/1 Jiwa</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 259991330008177</t>
   </si>
   <si>
@@ -1796,6 +1796,15 @@
     <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Mei 2025 untuk 2 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 259991310033060</t>
+  </si>
+  <si>
+    <t>00248T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Uang Makan PPPK Bulan Mei 2025 untuk 50 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 259991310033061</t>
   </si>
   <si>
@@ -1805,15 +1814,6 @@
     <t>Pembayaran Belanja Pegawai berupa Uang Makan PPPK Bulan Mei 2025 untuk 34 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 259991310033060</t>
-  </si>
-  <si>
-    <t>00248T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Uang Makan PPPK Bulan Mei 2025 untuk 50 Pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 259991330007277</t>
   </si>
   <si>
@@ -1913,6 +1913,15 @@
     <t>Pembayaran Tukin ke-13 Tahun 2025 Untuk 35 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231303002008</t>
+  </si>
+  <si>
+    <t>00242T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Tukin ke-13 Tahun 2025 Untuk 23 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231303002007</t>
   </si>
   <si>
@@ -1931,15 +1940,6 @@
     <t>Pembayaran Tukin ke-13 Tahun 2025 Untuk 173 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231303002008</t>
-  </si>
-  <si>
-    <t>00242T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Tukin ke-13 Tahun 2025 Untuk 23 Pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231305000975</t>
   </si>
   <si>
@@ -1952,39 +1952,39 @@
     <t>Pembayaran Tukin ke-13 Tahun 2025 Untuk 2 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231501001439</t>
+  </si>
+  <si>
+    <t>26-05-2025</t>
+  </si>
+  <si>
+    <t>00228T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Gaji ke-13 Tahun 2025 Untuk 137 Pegawai</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 250231501001414</t>
+  </si>
+  <si>
+    <t>00234T/403829/2025</t>
+  </si>
+  <si>
+    <t>SPM Gaji 13 PPPK</t>
+  </si>
+  <si>
+    <t>Pembayaran Gaji ke-13 Tahun 2025 Untuk 35 PPPK.</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231501001413</t>
   </si>
   <si>
-    <t>26-05-2025</t>
-  </si>
-  <si>
     <t>00232T/403829/2025</t>
   </si>
   <si>
-    <t>SPM Gaji 13 PPPK</t>
-  </si>
-  <si>
     <t>Pembayaran Gaji ke-13 Tahun 2025 Untuk 50 PPPK.</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231501001439</t>
-  </si>
-  <si>
-    <t>00228T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Gaji ke-13 Tahun 2025 Untuk 137 Pegawai</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 250231501001414</t>
-  </si>
-  <si>
-    <t>00234T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Gaji ke-13 Tahun 2025 Untuk 35 PPPK.</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231507000406</t>
   </si>
   <si>
@@ -1994,6 +1994,24 @@
     <t>Pembayaran Gaji ke-13 Tahun 2025 Untuk 2 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231503000384</t>
+  </si>
+  <si>
+    <t>00235T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Gaji ke-13 Tahun 2025 Untuk 23 PPPK.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 250231503000382</t>
+  </si>
+  <si>
+    <t>00229T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Gaji ke-13 Tahun 2025 Untuk 173 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231503000383</t>
   </si>
   <si>
@@ -2003,24 +2021,6 @@
     <t>Pembayaran Gaji ke-13 Tahun 2025 Untuk 63 PPPK.</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231503000382</t>
-  </si>
-  <si>
-    <t>00229T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Gaji ke-13 Tahun 2025 Untuk 173 Pegawai</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 250231503000384</t>
-  </si>
-  <si>
-    <t>00235T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Gaji ke-13 Tahun 2025 Untuk 23 PPPK.</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231305000959</t>
   </si>
   <si>
@@ -2072,30 +2072,30 @@
     <t>Pembayaran Belanja Barang Berupa Honor PPNPN Bulan Mei Tahun 2025 untuk 91 Pegawai.sesuai Sk No.9 Tahun 2025 Tanggal 6 Januari 2025</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231503000352</t>
+  </si>
+  <si>
+    <t>21-05-2025</t>
+  </si>
+  <si>
+    <t>00204T/403829/2025</t>
+  </si>
+  <si>
+    <t>08-05-2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan Juni 2025 untuk 23 Pegawai/52 Jiwa</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231503000351</t>
   </si>
   <si>
-    <t>21-05-2025</t>
-  </si>
-  <si>
     <t>00202T/403829/2025</t>
   </si>
   <si>
-    <t>08-05-2025</t>
-  </si>
-  <si>
     <t>Pembayaran Belanja Pegawai berupa Gaji induk PPPK Bulan Juni 2025 untuk 63 Pegawai/181 Jiwa</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231503000352</t>
-  </si>
-  <si>
-    <t>00204T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan Juni 2025 untuk 23 Pegawai/52 Jiwa</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231503000350</t>
   </si>
   <si>
@@ -2117,6 +2117,33 @@
     <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan Juni 2025 untuk 2 Pegawai/8 jiwa</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231501001209</t>
+  </si>
+  <si>
+    <t>00203T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan Juni 2025 untuk 35 Pegawai/101 Jiwa</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 250231501001201</t>
+  </si>
+  <si>
+    <t>00205T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa  Gaji Induk Bulan Juni 2025 untuk 39 Pegawai/111 Jiwa</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 250231501001208</t>
+  </si>
+  <si>
+    <t>00201T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan Juni 2025 untuk 50 Pegawai/124 Jiwa</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231501001202</t>
   </si>
   <si>
@@ -2126,54 +2153,27 @@
     <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan Juni 2025 untuk 135 Pegawai/ 396 Jiwa</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231501001208</t>
-  </si>
-  <si>
-    <t>00201T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan Juni 2025 untuk 50 Pegawai/124 Jiwa</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 250231501001201</t>
-  </si>
-  <si>
-    <t>00205T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa  Gaji Induk Bulan Juni 2025 untuk 39 Pegawai/111 Jiwa</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 250231501001209</t>
-  </si>
-  <si>
-    <t>00203T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan Juni 2025 untuk 35 Pegawai/101 Jiwa</t>
+    <t xml:space="preserve"> 250231303001770</t>
+  </si>
+  <si>
+    <t>20-05-2025</t>
+  </si>
+  <si>
+    <t>00219T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai Berupa Uang Makan PPPK Bulan April 2025 untuk 63 Pegawai</t>
   </si>
   <si>
     <t xml:space="preserve"> 250231303001771</t>
   </si>
   <si>
-    <t>20-05-2025</t>
-  </si>
-  <si>
     <t>00222T/403829/2025</t>
   </si>
   <si>
     <t>Pembayaran tunjangan kinerja bulan April tahun 2025 untuk 63 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231303001770</t>
-  </si>
-  <si>
-    <t>00219T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai Berupa Uang Makan PPPK Bulan April 2025 untuk 63 Pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231303001766</t>
   </si>
   <si>
@@ -2246,6 +2246,15 @@
     <t>Pembayaran tunjangan kinerja bulan April tahun 2025 untuk 173 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231301005717</t>
+  </si>
+  <si>
+    <t>00212T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran tunjangan kinerja bulan April tahun 2025 untuk 50 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231301005718</t>
   </si>
   <si>
@@ -2264,30 +2273,21 @@
     <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan April 2025  untuk 135 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231301005717</t>
-  </si>
-  <si>
-    <t>00212T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran tunjangan kinerja bulan April tahun 2025 untuk 50 Pegawai</t>
+    <t xml:space="preserve"> 250231301005583</t>
+  </si>
+  <si>
+    <t>14-05-2025</t>
+  </si>
+  <si>
+    <t>00209T/403829/2025</t>
   </si>
   <si>
     <t xml:space="preserve"> 250231301005582</t>
   </si>
   <si>
-    <t>14-05-2025</t>
-  </si>
-  <si>
     <t>00210T/403829/2025</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231301005583</t>
-  </si>
-  <si>
-    <t>00209T/403829/2025</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231302005378</t>
   </si>
   <si>
@@ -2345,27 +2345,27 @@
     <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan April 2025 untuk 38 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231302005131</t>
+  </si>
+  <si>
+    <t>06-05-2025</t>
+  </si>
+  <si>
+    <t>00194T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Barang sesuai Kwitansi No.02/SAj/KW/IV/2025 Tanggal 8 April 2025 berupa pemeliharaan CCTV Instalasi depok</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231302005132</t>
   </si>
   <si>
-    <t>06-05-2025</t>
-  </si>
-  <si>
     <t>00189T/403829/2025</t>
   </si>
   <si>
     <t>Pembayaran Belanja Barang berupa Tagihan PDAM Bulan April 2025 Idpel No. 1249-1046 An. Lemb Perikanan Darat</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231302005131</t>
-  </si>
-  <si>
-    <t>00194T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Barang sesuai Kwitansi No.02/SAj/KW/IV/2025 Tanggal 8 April 2025 berupa pemeliharaan CCTV Instalasi depok</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231301005196</t>
   </si>
   <si>
@@ -2498,45 +2498,45 @@
     <t>Pembayaran Belanja Barang Berupa Honor PPNPN Bulan April Tahun 2025 untuk 91 Pegawai.sesuai Sk No.9 Tahun 2025 tanggal 6 januari 2025</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231501001057</t>
+  </si>
+  <si>
+    <t>00156T/403829/2025</t>
+  </si>
+  <si>
+    <t>10-04-2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan Mei 2025 untuk 50 Pegawai/124 Jiwa</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 250231501001059</t>
+  </si>
+  <si>
+    <t>00153T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan Mei 2025 untuk 36 Pegawai/105 Jiwa</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 250231501001058</t>
+  </si>
+  <si>
+    <t>00159T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan Mei 2025 untuk 137 Pegawai/401 Jiwa</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231501001051</t>
   </si>
   <si>
     <t>00158T/403829/2025</t>
   </si>
   <si>
-    <t>10-04-2025</t>
-  </si>
-  <si>
     <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan Mei 2025 untuk 39 Pegawai/111 Jiwa</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231501001059</t>
-  </si>
-  <si>
-    <t>00153T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan Mei 2025 untuk 36 Pegawai/105 Jiwa</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 250231501001057</t>
-  </si>
-  <si>
-    <t>00156T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan Mei 2025 untuk 50 Pegawai/124 Jiwa</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 250231501001058</t>
-  </si>
-  <si>
-    <t>00159T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan Mei 2025 untuk 137 Pegawai/401 Jiwa</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231507000303</t>
   </si>
   <si>
@@ -2585,6 +2585,15 @@
     <t>Pembayaran tunjangan kinerja bulan Maret tahun 2025 untuk 63 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231301004026</t>
+  </si>
+  <si>
+    <t>00175T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran tunjangan kinerja bulan Maret tahun 2025 untuk 36 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231301004024</t>
   </si>
   <si>
@@ -2594,15 +2603,6 @@
     <t>Pembayaran tunjangan kinerja bulan Maret tahun 2025 untuk 138 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231301004026</t>
-  </si>
-  <si>
-    <t>00175T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran tunjangan kinerja bulan Maret tahun 2025 untuk 36 Pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231301004025</t>
   </si>
   <si>
@@ -2612,6 +2612,15 @@
     <t>Pembayaran tunjangan kinerja bulan Maret tahun 2025 untuk 50 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231303001236</t>
+  </si>
+  <si>
+    <t>00179T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran tunjangan kinerja bulan Maret tahun 2025 untuk 23 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231303001235</t>
   </si>
   <si>
@@ -2621,15 +2630,6 @@
     <t>Pembayaran tunjangan kinerja bulan Maret tahun 2025 untuk 175 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231303001236</t>
-  </si>
-  <si>
-    <t>00179T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran tunjangan kinerja bulan Maret tahun 2025 untuk 23 Pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231302003921</t>
   </si>
   <si>
@@ -2699,6 +2699,33 @@
     <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Maret 2025 untuk 2 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231301003743</t>
+  </si>
+  <si>
+    <t>00167T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Maret 2025 untuk 38 Pegawai</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 250231301003744</t>
+  </si>
+  <si>
+    <t>00163T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Uang Makan PPPK Bulan Maret 2025 untuk 49 Pegawai</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 250231301003746</t>
+  </si>
+  <si>
+    <t>00162T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Uang Makan PPPK Bulan Maret 2025 untuk 36 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231301003745</t>
   </si>
   <si>
@@ -2708,33 +2735,6 @@
     <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Maret 2025 untuk 136 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231301003744</t>
-  </si>
-  <si>
-    <t>00163T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Uang Makan PPPK Bulan Maret 2025 untuk 49 Pegawai</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 250231301003746</t>
-  </si>
-  <si>
-    <t>00162T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Uang Makan PPPK Bulan Maret 2025 untuk 36 Pegawai</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 250231301003743</t>
-  </si>
-  <si>
-    <t>00167T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Maret 2025 untuk 38 Pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231303001158</t>
   </si>
   <si>
@@ -2846,6 +2846,24 @@
     <t>Pembayaran tunjangan kinerja bulan April tahun 2025 untuk 39 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231501000907</t>
+  </si>
+  <si>
+    <t>00145T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Barang Berupa Honor PPNPN Bulan Maret Tahun 2025 untuk 102 Pegawai.Sesuai SK No. 9 Tahun 2025 Tanggal 6 Januari 2025</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 250231501000908</t>
+  </si>
+  <si>
+    <t>00135T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Barang Berupa Honor PPNPN Bulan Maret Tahun 2025 untuk 16 Pegawai.sesuai Sk No.B.4/BRPBATPP/KP.340/I/2025 Tanggal 2 Januari 2025</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231501000906</t>
   </si>
   <si>
@@ -2855,24 +2873,6 @@
     <t>Pembayaran Belanja Barang Berupa Honor PPNPN Bulan Maret Tahun 2025 untuk 1 Pegawai.sesuai SK No. 9 Tahun 2025 tanggal 6 Januari 2025</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231501000908</t>
-  </si>
-  <si>
-    <t>00135T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Barang Berupa Honor PPNPN Bulan Maret Tahun 2025 untuk 16 Pegawai.sesuai Sk No.B.4/BRPBATPP/KP.340/I/2025 Tanggal 2 Januari 2025</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 250231501000907</t>
-  </si>
-  <si>
-    <t>00145T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Barang Berupa Honor PPNPN Bulan Maret Tahun 2025 untuk 102 Pegawai.Sesuai SK No. 9 Tahun 2025 Tanggal 6 Januari 2025</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231503000261</t>
   </si>
   <si>
@@ -2882,15 +2882,33 @@
     <t>Pembayaran Belanja Barang Berupa Honor PPNPN Bulan Maret Tahun 2025 untuk 91 Pegawai.Sesuai Sk No.9 tahun 2025 Tanggal 6 Januari 2025</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231501000765</t>
+  </si>
+  <si>
+    <t>00090T/403829/2025</t>
+  </si>
+  <si>
+    <t>11-03-2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan April 2025 untuk 39 Pegawai/ 111 Jiwa</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 250231501000766</t>
+  </si>
+  <si>
+    <t>00089T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan April 2025 untuk 137 Pegawai/403 Jiwa</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231501000781</t>
   </si>
   <si>
     <t>00092T/403829/2025</t>
   </si>
   <si>
-    <t>11-03-2025</t>
-  </si>
-  <si>
     <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan April 2025 untuk 50 Pegawai/124 Jiwa</t>
   </si>
   <si>
@@ -2903,24 +2921,6 @@
     <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan April 2025 untuk 36 Pegawai/106 Jiwa</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231501000766</t>
-  </si>
-  <si>
-    <t>00089T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan April 2025 untuk 137 Pegawai/403 Jiwa</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 250231501000765</t>
-  </si>
-  <si>
-    <t>00090T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan April 2025 untuk 39 Pegawai/ 111 Jiwa</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231507000254</t>
   </si>
   <si>
@@ -3086,6 +3086,24 @@
     <t>Pembayaran THR Tunkin Tahun 2025 Untuk 2 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231303000888</t>
+  </si>
+  <si>
+    <t>00130T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Januari 2025 untuk 1 Pegawai</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 250231303000887</t>
+  </si>
+  <si>
+    <t>00126T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran THR Tunkin Tahun 2025 Untuk 63 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231303000889</t>
   </si>
   <si>
@@ -3095,24 +3113,6 @@
     <t>Pembayaran Belanja Pegawai berupa Uang Makan februari 2025 untuk 1 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231303000888</t>
-  </si>
-  <si>
-    <t>00130T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Januari 2025 untuk 1 Pegawai</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 250231303000887</t>
-  </si>
-  <si>
-    <t>00126T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran THR Tunkin Tahun 2025 Untuk 63 Pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231301002724</t>
   </si>
   <si>
@@ -3158,6 +3158,15 @@
     <t>Pembayaran THR Tahun 2025 Untuk 2 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231503000157</t>
+  </si>
+  <si>
+    <t>00119T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran THR Tahun 2025 Untuk 63 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231503000156</t>
   </si>
   <si>
@@ -3167,13 +3176,13 @@
     <t>Pembayaran THR Tahun 2025 Untuk 177 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231503000157</t>
-  </si>
-  <si>
-    <t>00119T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran THR Tahun 2025 Untuk 63 Pegawai</t>
+    <t xml:space="preserve"> 250231501000528</t>
+  </si>
+  <si>
+    <t>00116T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran THR Tahun 2025 Untuk 139 Pegawai</t>
   </si>
   <si>
     <t xml:space="preserve"> 250231501000527</t>
@@ -3185,6 +3194,24 @@
     <t>Pembayaran THR Tahun 2025 Untuk 1 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231501000545</t>
+  </si>
+  <si>
+    <t>00121T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran THR Keagamaan Tahun 2025 Untuk 16 Pegawai.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 250231501000530</t>
+  </si>
+  <si>
+    <t>00120T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran THR Tahun 2025 Untuk 36 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231501000526</t>
   </si>
   <si>
@@ -3194,24 +3221,6 @@
     <t>Pembayaran THR Tahun 2025 Untuk 39 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231501000528</t>
-  </si>
-  <si>
-    <t>00116T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran THR Tahun 2025 Untuk 139 Pegawai</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 250231501000545</t>
-  </si>
-  <si>
-    <t>00121T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran THR Keagamaan Tahun 2025 Untuk 16 Pegawai.</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231501000529</t>
   </si>
   <si>
@@ -3221,15 +3230,6 @@
     <t>Pembayaran THR Tahun 2025 Untuk 50 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231501000530</t>
-  </si>
-  <si>
-    <t>00120T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran THR Tahun 2025 Untuk 36 Pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231302002452</t>
   </si>
   <si>
@@ -3278,6 +3278,18 @@
     <t>Pembayaran tunjangan kinerja bulan Januari tahun 2025 untuk 1 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231303000777</t>
+  </si>
+  <si>
+    <t>00096T/403829/2025</t>
+  </si>
+  <si>
+    <t>GAJI SUSULAN</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji Susulan Bulan Maret 2025 untuk 1 Pegawai/4 jiwa</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231303000778</t>
   </si>
   <si>
@@ -3287,16 +3299,22 @@
     <t>Pembayaran tunjangan kinerja bulan Februari tahun 2025 untuk 177 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231303000777</t>
-  </si>
-  <si>
-    <t>00096T/403829/2025</t>
-  </si>
-  <si>
-    <t>GAJI SUSULAN</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji Susulan Bulan Maret 2025 untuk 1 Pegawai/4 jiwa</t>
+    <t xml:space="preserve"> 250231301002369</t>
+  </si>
+  <si>
+    <t>00103T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan februari 2025 untuk 136 Pegawai</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 250231301002372</t>
+  </si>
+  <si>
+    <t>00106T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran tunjangan kinerja bulan Februari tahun 2025 untuk 36 Pegawai</t>
   </si>
   <si>
     <t xml:space="preserve"> 250231301002370</t>
@@ -3308,24 +3326,6 @@
     <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Februari 2025 untuk 37 pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231301002372</t>
-  </si>
-  <si>
-    <t>00106T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran tunjangan kinerja bulan Februari tahun 2025 untuk 36 Pegawai</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 250231301002369</t>
-  </si>
-  <si>
-    <t>00103T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan februari 2025 untuk 136 Pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231301002371</t>
   </si>
   <si>
@@ -3344,6 +3344,15 @@
     <t>Pembayaran Belanja Pegawai berupa Uang Makan bulan Februari 2025 untuk 36 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231303000773</t>
+  </si>
+  <si>
+    <t>00099T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan februari 2025 untuk 63 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231303000774</t>
   </si>
   <si>
@@ -3353,15 +3362,6 @@
     <t>Pembayaran tunjangan kinerja bulan Februari tahun 2025 untuk 63 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231303000773</t>
-  </si>
-  <si>
-    <t>00099T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan februari 2025 untuk 63 Pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231303000772</t>
   </si>
   <si>
@@ -3473,30 +3473,39 @@
     <t>Pembayaran Belanja Barang Berupa Honor PPNPN Bulan Januari Tahun 2025 untuk 90 Pegawai.sesuai Sk no.9 tahun 2025 tanggal 6 januari 2025</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231303000473</t>
+  </si>
+  <si>
+    <t>25-02-2025</t>
+  </si>
+  <si>
+    <t>26-02-2025</t>
+  </si>
+  <si>
+    <t>00073T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Januari 2025 untuk 175 pegawai</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 250231303000476</t>
+  </si>
+  <si>
+    <t>00075T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran tunjangan kinerja bulan Januari tahun 2025 untuk 177 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231303000475</t>
   </si>
   <si>
-    <t>25-02-2025</t>
-  </si>
-  <si>
-    <t>26-02-2025</t>
-  </si>
-  <si>
     <t>00076T/403829/2025</t>
   </si>
   <si>
     <t>Pembayaran tunjangan kinerja bulan Januari tahun 2025 untuk 63 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231303000476</t>
-  </si>
-  <si>
-    <t>00075T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran tunjangan kinerja bulan Januari tahun 2025 untuk 177 Pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231303000474</t>
   </si>
   <si>
@@ -3506,15 +3515,6 @@
     <t>Pembayaran Belanja Pegawai berupa Uang Makan PPPK bulan Januari 2025 untuk 63 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231303000473</t>
-  </si>
-  <si>
-    <t>00073T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Januari 2025 untuk 175 pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231305000180</t>
   </si>
   <si>
@@ -3563,6 +3563,15 @@
     <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan Maret 2025 untuk 2 Pegawai /8 Jiwa</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231501000431</t>
+  </si>
+  <si>
+    <t>00062T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan Maret 2025 untuk 39 Pegawai/112 Jiwa</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231501000434</t>
   </si>
   <si>
@@ -3575,6 +3584,27 @@
     <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan Maret 2025 untuk 36 Pegawai/106 Jiwa</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231501000433</t>
+  </si>
+  <si>
+    <t>00065T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai Berupa Gaji Induk Maret 2025 untuk 50 Pegawai/123 Jiwa</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 250231501000339</t>
+  </si>
+  <si>
+    <t>00069T/403829/2025</t>
+  </si>
+  <si>
+    <t>20-02-2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Barang Berupa Honor PPNPN Bulan Februari Tahun 2025 untuk 16 Pegawai.sesuai SK No.04/BRPBATPP/KP.340/I/2025 Tanggal 2 Januari 2025</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231501000432</t>
   </si>
   <si>
@@ -3584,36 +3614,6 @@
     <t>Pembayaran Belanja Pegawai Berupa Gaji Induk bulan Maret 2025 untuk 137 Pegawai/403 Jiwa</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231501000433</t>
-  </si>
-  <si>
-    <t>00065T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai Berupa Gaji Induk Maret 2025 untuk 50 Pegawai/123 Jiwa</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 250231501000431</t>
-  </si>
-  <si>
-    <t>00062T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan Maret 2025 untuk 39 Pegawai/112 Jiwa</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 250231501000339</t>
-  </si>
-  <si>
-    <t>00069T/403829/2025</t>
-  </si>
-  <si>
-    <t>20-02-2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Barang Berupa Honor PPNPN Bulan Februari Tahun 2025 untuk 16 Pegawai.sesuai SK No.04/BRPBATPP/KP.340/I/2025 Tanggal 2 Januari 2025</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231503000118</t>
   </si>
   <si>
@@ -3644,6 +3644,15 @@
     <t>Pembayaran tunjangan kinerja bulan Januari tahun 2025 untuk 138 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231301001112</t>
+  </si>
+  <si>
+    <t>00060T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran tunjangan kinerja  bulan Januari tahun 2025 untuk 50 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231301001113</t>
   </si>
   <si>
@@ -3653,39 +3662,30 @@
     <t>Pembayaran tunjangan kinerja bulan Januari tahun 2025 untuk 36 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231301001112</t>
-  </si>
-  <si>
-    <t>00060T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran tunjangan kinerja  bulan Januari tahun 2025 untuk 50 Pegawai</t>
+    <t xml:space="preserve"> 250231301001061</t>
+  </si>
+  <si>
+    <t>16-02-2025</t>
+  </si>
+  <si>
+    <t>00052T/403829/2025</t>
+  </si>
+  <si>
+    <t>13-02-2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Januari 2025 untuk 37 Pegawai</t>
   </si>
   <si>
     <t xml:space="preserve"> 250231301001062</t>
   </si>
   <si>
-    <t>16-02-2025</t>
-  </si>
-  <si>
     <t>00051T/403829/2025</t>
   </si>
   <si>
-    <t>13-02-2025</t>
-  </si>
-  <si>
     <t>Pembayaran Belanja Pegawai berupa Uang Makan bulan Januari 2025 untuk 36 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231301001061</t>
-  </si>
-  <si>
-    <t>00052T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Januari 2025 untuk 37 Pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231305000122</t>
   </si>
   <si>
@@ -3698,6 +3698,15 @@
     <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Januari 2025 untuk 2 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231301000960</t>
+  </si>
+  <si>
+    <t>00058T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Januari 2025 untuk 136 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231301000961</t>
   </si>
   <si>
@@ -3707,15 +3716,6 @@
     <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Januari 2025 untuk 50 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231301000960</t>
-  </si>
-  <si>
-    <t>00058T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Uang Makan Bulan Januari 2025 untuk 136 Pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231305000116</t>
   </si>
   <si>
@@ -3764,6 +3764,15 @@
     <t>Pembayaran belanja barang berupa tagihan telepon bulan Februari 2025 untuk 12 invoice</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231302000795</t>
+  </si>
+  <si>
+    <t>00049T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Barang sesuai Kwitansi No.001/KW-PNA/II/2025 Tanggal 6 Februari 2025 berupa Pemelliharaan Talud Cijeruk</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231302000796</t>
   </si>
   <si>
@@ -3773,15 +3782,6 @@
     <t>Pembayaran Belanja Barang sesuai Kwitansi No. 02/SAJ/KW/II/2025 Tanggal 3 Februari 2025 berupa Pemeliharaan Halaman Kantor Instalasi Riset Pengendalian Penyakit Ikan Depok</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231302000795</t>
-  </si>
-  <si>
-    <t>00049T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Barang sesuai Kwitansi No.001/KW-PNA/II/2025 Tanggal 6 Februari 2025 berupa Pemelliharaan Talud Cijeruk</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231301000882</t>
   </si>
   <si>
@@ -3893,6 +3893,15 @@
     <t>Pembayaran tunjangan kinerja bulan Februari tahun 2025 untuk 2 Pegawai</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231301000433</t>
+  </si>
+  <si>
+    <t>00031T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran tunjangan kinerja bulan Februari tahun 2025 untuk 1 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231301000432</t>
   </si>
   <si>
@@ -3902,15 +3911,6 @@
     <t>Pembayaran tunjangan kinerja bulan Februari tahun 2025 untuk 38 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231301000433</t>
-  </si>
-  <si>
-    <t>00031T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran tunjangan kinerja bulan Februari tahun 2025 untuk 1 Pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231303000130</t>
   </si>
   <si>
@@ -3920,6 +3920,15 @@
     <t>Pembayaran Belanja Barang sesuai Kwitansi No. 02/MSP/KW/I/2025 Tanggal 20 Januari 2025 berupa Perbaikan Kamar Mandi dan Sanitasi</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231301000417</t>
+  </si>
+  <si>
+    <t>00032T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran kekurangan tunjangan kinerja bulan Desember tahun 2024 untuk 1 Pegawai</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231301000416</t>
   </si>
   <si>
@@ -3929,15 +3938,6 @@
     <t>Pembayaran tunjangan kinerja susulan bulan Desember tahun 2024 untuk 1 Pegawai</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231301000417</t>
-  </si>
-  <si>
-    <t>00032T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran kekurangan tunjangan kinerja bulan Desember tahun 2024 untuk 1 Pegawai</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231501000261</t>
   </si>
   <si>
@@ -3950,27 +3950,27 @@
     <t>Pembayaran Belanja Barang Berupa Honor PPNPN Bulan Januari Tahun 2025 untuk 17 Pegawai.sesuai SK No.B.4/BRPBATPP/KP.340/I/2025 tanggal 2 Januari 2025</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231301000386</t>
+  </si>
+  <si>
+    <t>23-01-2025</t>
+  </si>
+  <si>
+    <t>00026T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Kekurangan Gaji Bulan Desember 2024 untuk 1 Pegawai/4 Jiwa</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231301000385</t>
   </si>
   <si>
-    <t>23-01-2025</t>
-  </si>
-  <si>
     <t>00025T/403829/2025</t>
   </si>
   <si>
     <t>Pembayaran Belanja Pegawai berupa Gaji Susulan Bulan Desember 2024 untuk 1 Pegawai/4 Jiwa</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231301000386</t>
-  </si>
-  <si>
-    <t>00026T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Kekurangan Gaji Bulan Desember 2024 untuk 1 Pegawai/4 Jiwa</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231302000370</t>
   </si>
   <si>
@@ -3995,36 +3995,36 @@
     <t>Pembayaran Belanja Pegawai berupa Gaji Induk PPPK Bulan Februari 2025 untuk 36 Pegawai/105 Jiwa</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231501000229</t>
+  </si>
+  <si>
+    <t>00010T/403829/2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai Berupa Gaji Induk PPPK Bulan Februari 2025 untuk 50 Pegawai/123 Jiwa</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 250231501000227</t>
+  </si>
+  <si>
+    <t>00019T/403829/2025</t>
+  </si>
+  <si>
+    <t>14-01-2025</t>
+  </si>
+  <si>
+    <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan februari 2025 untuk 39 Pegawai/112 jiwa</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231501000228</t>
   </si>
   <si>
     <t>00021T/403829/2025</t>
   </si>
   <si>
-    <t>14-01-2025</t>
-  </si>
-  <si>
     <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan februari 2025 untuk 138 Pegawai/406 Jiwa</t>
   </si>
   <si>
-    <t xml:space="preserve"> 250231501000227</t>
-  </si>
-  <si>
-    <t>00019T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai berupa Gaji Induk Bulan februari 2025 untuk 39 Pegawai/112 jiwa</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 250231501000229</t>
-  </si>
-  <si>
-    <t>00010T/403829/2025</t>
-  </si>
-  <si>
-    <t>Pembayaran Belanja Pegawai Berupa Gaji Induk PPPK Bulan Februari 2025 untuk 50 Pegawai/123 Jiwa</t>
-  </si>
-  <si>
     <t xml:space="preserve"> 250231507000048</t>
   </si>
   <si>
@@ -4067,31 +4067,31 @@
     <t>Pembayaran Belanja Barang berupa Tagihan Internet Bulan Januari 2025 Idpel No.GO18A106 An Balai Riset Perikanan Budidaya Air Tawar dan Penyuluhan Perikanan</t>
   </si>
   <si>
+    <t xml:space="preserve"> 250231301000153</t>
+  </si>
+  <si>
+    <t>10-01-2025</t>
+  </si>
+  <si>
+    <t>13-01-2025</t>
+  </si>
+  <si>
+    <t>00017T/403829/2025</t>
+  </si>
+  <si>
+    <t>UP</t>
+  </si>
+  <si>
+    <t>Penyediaan Uang Persediaan BALAI RISET PERIKANAN BUDIDAYA AIR TAWAR DAN PENYULUHAN PERIKANAN Tahun Anggaran 2025</t>
+  </si>
+  <si>
     <t xml:space="preserve"> 250231301000152</t>
   </si>
   <si>
-    <t>10-01-2025</t>
-  </si>
-  <si>
-    <t>13-01-2025</t>
-  </si>
-  <si>
     <t>00016T/403829/2025</t>
   </si>
   <si>
     <t>Pembayaran Belanja Pegawai berupa Gai Susulan Bulan Desember 2024 sd Januari 2025 untuk 1 Pegawai/4 Jiwa</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> 250231301000153</t>
-  </si>
-  <si>
-    <t>00017T/403829/2025</t>
-  </si>
-  <si>
-    <t>UP</t>
-  </si>
-  <si>
-    <t>Penyediaan Uang Persediaan BALAI RISET PERIKANAN BUDIDAYA AIR TAWAR DAN PENYULUHAN PERIKANAN Tahun Anggaran 2025</t>
   </si>
   <si>
     <t xml:space="preserve"> 250231303000044</t>
@@ -6830,7 +6830,7 @@
         <v>211</v>
       </c>
       <c r="E65" s="1">
-        <v>200500400</v>
+        <v>655816000</v>
       </c>
       <c r="F65" s="1" t="s">
         <v>238</v>
@@ -6839,7 +6839,7 @@
         <v>239</v>
       </c>
       <c r="H65" s="1" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="I65" s="1" t="s">
         <v>78</v>
@@ -6866,7 +6866,7 @@
         <v>211</v>
       </c>
       <c r="E66" s="1">
-        <v>655816000</v>
+        <v>200500400</v>
       </c>
       <c r="F66" s="1" t="s">
         <v>242</v>
@@ -6875,7 +6875,7 @@
         <v>239</v>
       </c>
       <c r="H66" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I66" s="1" t="s">
         <v>78</v>
@@ -6902,22 +6902,22 @@
         <v>211</v>
       </c>
       <c r="E67" s="1">
-        <v>144846400</v>
+        <v>168310100</v>
       </c>
       <c r="F67" s="1" t="s">
         <v>245</v>
       </c>
       <c r="G67" s="1" t="s">
-        <v>239</v>
+        <v>246</v>
       </c>
       <c r="H67" s="1" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="I67" s="1" t="s">
         <v>78</v>
       </c>
       <c r="J67" s="1" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="K67" s="1" t="s">
         <v>19</v>
@@ -6929,7 +6929,7 @@
         <v>65</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="C68" s="1" t="s">
         <v>237</v>
@@ -6938,16 +6938,16 @@
         <v>211</v>
       </c>
       <c r="E68" s="1">
-        <v>168310100</v>
+        <v>144846400</v>
       </c>
       <c r="F68" s="1" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="G68" s="1" t="s">
-        <v>249</v>
+        <v>239</v>
       </c>
       <c r="H68" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I68" s="1" t="s">
         <v>78</v>
@@ -7010,7 +7010,7 @@
         <v>211</v>
       </c>
       <c r="E70" s="1">
-        <v>844985400</v>
+        <v>268443100</v>
       </c>
       <c r="F70" s="1" t="s">
         <v>255</v>
@@ -7019,7 +7019,7 @@
         <v>239</v>
       </c>
       <c r="H70" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I70" s="1" t="s">
         <v>78</v>
@@ -7046,7 +7046,7 @@
         <v>211</v>
       </c>
       <c r="E71" s="1">
-        <v>91372600</v>
+        <v>844985400</v>
       </c>
       <c r="F71" s="1" t="s">
         <v>258</v>
@@ -7055,7 +7055,7 @@
         <v>239</v>
       </c>
       <c r="H71" s="1" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="I71" s="1" t="s">
         <v>78</v>
@@ -7082,7 +7082,7 @@
         <v>211</v>
       </c>
       <c r="E72" s="1">
-        <v>268443100</v>
+        <v>91372600</v>
       </c>
       <c r="F72" s="1" t="s">
         <v>261</v>
@@ -7112,19 +7112,19 @@
         <v>263</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D73" s="1" t="s">
         <v>237</v>
       </c>
       <c r="E73" s="1">
-        <v>213199358</v>
+        <v>153763873</v>
       </c>
       <c r="F73" s="1" t="s">
         <v>264</v>
       </c>
       <c r="G73" s="1" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="H73" s="1" t="s">
         <v>135</v>
@@ -7148,19 +7148,19 @@
         <v>266</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D74" s="1" t="s">
         <v>237</v>
       </c>
       <c r="E74" s="1">
-        <v>153763873</v>
+        <v>823139642</v>
       </c>
       <c r="F74" s="1" t="s">
         <v>267</v>
       </c>
       <c r="G74" s="1" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="H74" s="1" t="s">
         <v>135</v>
@@ -7184,19 +7184,19 @@
         <v>269</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D75" s="1" t="s">
         <v>237</v>
       </c>
       <c r="E75" s="1">
-        <v>823139642</v>
+        <v>213199358</v>
       </c>
       <c r="F75" s="1" t="s">
         <v>270</v>
       </c>
       <c r="G75" s="1" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="H75" s="1" t="s">
         <v>135</v>
@@ -7220,7 +7220,7 @@
         <v>272</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D76" s="1" t="s">
         <v>237</v>
@@ -7232,7 +7232,7 @@
         <v>273</v>
       </c>
       <c r="G76" s="1" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="H76" s="1" t="s">
         <v>135</v>
@@ -7256,7 +7256,7 @@
         <v>275</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D77" s="1" t="s">
         <v>237</v>
@@ -7268,7 +7268,7 @@
         <v>276</v>
       </c>
       <c r="G77" s="1" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="H77" s="1" t="s">
         <v>135</v>
@@ -7292,10 +7292,10 @@
         <v>278</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D78" s="1" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="E78" s="1">
         <v>455600</v>
@@ -7304,7 +7304,7 @@
         <v>279</v>
       </c>
       <c r="G78" s="1" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="H78" s="1" t="s">
         <v>42</v>
@@ -7328,10 +7328,10 @@
         <v>281</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D79" s="1" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="E79" s="1">
         <v>698200</v>
@@ -7340,7 +7340,7 @@
         <v>282</v>
       </c>
       <c r="G79" s="1" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="H79" s="1" t="s">
         <v>42</v>
@@ -7727,7 +7727,7 @@
         <v>239</v>
       </c>
       <c r="D90" s="1" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="E90" s="1">
         <v>41758847</v>
@@ -7763,7 +7763,7 @@
         <v>239</v>
       </c>
       <c r="D91" s="1" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="E91" s="1">
         <v>2844264</v>
@@ -8270,7 +8270,7 @@
         <v>336</v>
       </c>
       <c r="E105" s="1">
-        <v>661725600</v>
+        <v>200371400</v>
       </c>
       <c r="F105" s="1" t="s">
         <v>370</v>
@@ -8279,7 +8279,7 @@
         <v>371</v>
       </c>
       <c r="H105" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I105" s="1" t="s">
         <v>78</v>
@@ -8306,7 +8306,7 @@
         <v>336</v>
       </c>
       <c r="E106" s="1">
-        <v>171835300</v>
+        <v>661725600</v>
       </c>
       <c r="F106" s="1" t="s">
         <v>374</v>
@@ -8378,7 +8378,7 @@
         <v>336</v>
       </c>
       <c r="E108" s="1">
-        <v>200371400</v>
+        <v>171835300</v>
       </c>
       <c r="F108" s="1" t="s">
         <v>380</v>
@@ -8387,7 +8387,7 @@
         <v>371</v>
       </c>
       <c r="H108" s="1" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="I108" s="1" t="s">
         <v>78</v>
@@ -8558,7 +8558,7 @@
         <v>397</v>
       </c>
       <c r="E113" s="1">
-        <v>154096751</v>
+        <v>822658451</v>
       </c>
       <c r="F113" s="1" t="s">
         <v>398</v>
@@ -8594,7 +8594,7 @@
         <v>397</v>
       </c>
       <c r="E114" s="1">
-        <v>822658451</v>
+        <v>154096751</v>
       </c>
       <c r="F114" s="1" t="s">
         <v>401</v>
@@ -8630,7 +8630,7 @@
         <v>397</v>
       </c>
       <c r="E115" s="1">
-        <v>99668220</v>
+        <v>1040244280</v>
       </c>
       <c r="F115" s="1" t="s">
         <v>404</v>
@@ -8702,7 +8702,7 @@
         <v>397</v>
       </c>
       <c r="E117" s="1">
-        <v>1040244280</v>
+        <v>99668220</v>
       </c>
       <c r="F117" s="1" t="s">
         <v>410</v>
@@ -8774,7 +8774,7 @@
         <v>416</v>
       </c>
       <c r="E119" s="1">
-        <v>21398250</v>
+        <v>22399900</v>
       </c>
       <c r="F119" s="1" t="s">
         <v>417</v>
@@ -8783,7 +8783,7 @@
         <v>371</v>
       </c>
       <c r="H119" s="1" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="I119" s="1" t="s">
         <v>17</v>
@@ -8810,7 +8810,7 @@
         <v>416</v>
       </c>
       <c r="E120" s="1">
-        <v>22399900</v>
+        <v>82033000</v>
       </c>
       <c r="F120" s="1" t="s">
         <v>420</v>
@@ -8882,7 +8882,7 @@
         <v>416</v>
       </c>
       <c r="E122" s="1">
-        <v>82033000</v>
+        <v>21398250</v>
       </c>
       <c r="F122" s="1" t="s">
         <v>426</v>
@@ -8891,7 +8891,7 @@
         <v>371</v>
       </c>
       <c r="H122" s="1" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="I122" s="1" t="s">
         <v>17</v>
@@ -8954,7 +8954,7 @@
         <v>416</v>
       </c>
       <c r="E124" s="1">
-        <v>13597650</v>
+        <v>106926550</v>
       </c>
       <c r="F124" s="1" t="s">
         <v>432</v>
@@ -8963,7 +8963,7 @@
         <v>371</v>
       </c>
       <c r="H124" s="1" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="I124" s="1" t="s">
         <v>17</v>
@@ -8990,7 +8990,7 @@
         <v>416</v>
       </c>
       <c r="E125" s="1">
-        <v>106926550</v>
+        <v>38519000</v>
       </c>
       <c r="F125" s="1" t="s">
         <v>435</v>
@@ -8999,7 +8999,7 @@
         <v>371</v>
       </c>
       <c r="H125" s="1" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="I125" s="1" t="s">
         <v>17</v>
@@ -9026,7 +9026,7 @@
         <v>416</v>
       </c>
       <c r="E126" s="1">
-        <v>38519000</v>
+        <v>13597650</v>
       </c>
       <c r="F126" s="1" t="s">
         <v>438</v>
@@ -9242,7 +9242,7 @@
         <v>456</v>
       </c>
       <c r="E132" s="1">
-        <v>597550</v>
+        <v>4595150</v>
       </c>
       <c r="F132" s="1" t="s">
         <v>463</v>
@@ -9251,7 +9251,7 @@
         <v>464</v>
       </c>
       <c r="H132" s="1" t="s">
-        <v>16</v>
+        <v>135</v>
       </c>
       <c r="I132" s="1" t="s">
         <v>17</v>
@@ -9278,7 +9278,7 @@
         <v>456</v>
       </c>
       <c r="E133" s="1">
-        <v>4595150</v>
+        <v>597550</v>
       </c>
       <c r="F133" s="1" t="s">
         <v>467</v>
@@ -9287,7 +9287,7 @@
         <v>464</v>
       </c>
       <c r="H133" s="1" t="s">
-        <v>135</v>
+        <v>16</v>
       </c>
       <c r="I133" s="1" t="s">
         <v>17</v>
@@ -9422,7 +9422,7 @@
         <v>464</v>
       </c>
       <c r="E137" s="1">
-        <v>177279700</v>
+        <v>679180900</v>
       </c>
       <c r="F137" s="1" t="s">
         <v>481</v>
@@ -9458,7 +9458,7 @@
         <v>464</v>
       </c>
       <c r="E138" s="1">
-        <v>679180900</v>
+        <v>200371400</v>
       </c>
       <c r="F138" s="1" t="s">
         <v>485</v>
@@ -9467,7 +9467,7 @@
         <v>482</v>
       </c>
       <c r="H138" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I138" s="1" t="s">
         <v>78</v>
@@ -9530,7 +9530,7 @@
         <v>464</v>
       </c>
       <c r="E140" s="1">
-        <v>200371400</v>
+        <v>177279700</v>
       </c>
       <c r="F140" s="1" t="s">
         <v>491</v>
@@ -9539,7 +9539,7 @@
         <v>482</v>
       </c>
       <c r="H140" s="1" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="I140" s="1" t="s">
         <v>78</v>
@@ -9638,7 +9638,7 @@
         <v>464</v>
       </c>
       <c r="E143" s="1">
-        <v>261119293</v>
+        <v>62679696</v>
       </c>
       <c r="F143" s="1" t="s">
         <v>502</v>
@@ -9674,7 +9674,7 @@
         <v>464</v>
       </c>
       <c r="E144" s="1">
-        <v>62679696</v>
+        <v>261119293</v>
       </c>
       <c r="F144" s="1" t="s">
         <v>505</v>
@@ -9710,16 +9710,16 @@
         <v>464</v>
       </c>
       <c r="E145" s="1">
-        <v>261772500</v>
+        <v>230734521</v>
       </c>
       <c r="F145" s="1" t="s">
         <v>508</v>
       </c>
       <c r="G145" s="1" t="s">
-        <v>482</v>
+        <v>496</v>
       </c>
       <c r="H145" s="1" t="s">
-        <v>101</v>
+        <v>77</v>
       </c>
       <c r="I145" s="1" t="s">
         <v>78</v>
@@ -9746,22 +9746,22 @@
         <v>464</v>
       </c>
       <c r="E146" s="1">
-        <v>865011300</v>
+        <v>91372600</v>
       </c>
       <c r="F146" s="1" t="s">
         <v>511</v>
       </c>
       <c r="G146" s="1" t="s">
-        <v>512</v>
+        <v>482</v>
       </c>
       <c r="H146" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I146" s="1" t="s">
         <v>78</v>
       </c>
       <c r="J146" s="1" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="K146" s="1" t="s">
         <v>19</v>
@@ -9773,7 +9773,7 @@
         <v>144</v>
       </c>
       <c r="B147" s="1" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="C147" s="1" t="s">
         <v>494</v>
@@ -9782,16 +9782,16 @@
         <v>464</v>
       </c>
       <c r="E147" s="1">
-        <v>91372600</v>
+        <v>865011300</v>
       </c>
       <c r="F147" s="1" t="s">
+        <v>514</v>
+      </c>
+      <c r="G147" s="1" t="s">
         <v>515</v>
       </c>
-      <c r="G147" s="1" t="s">
-        <v>482</v>
-      </c>
       <c r="H147" s="1" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="I147" s="1" t="s">
         <v>78</v>
@@ -9818,16 +9818,16 @@
         <v>464</v>
       </c>
       <c r="E148" s="1">
-        <v>230734521</v>
+        <v>261772500</v>
       </c>
       <c r="F148" s="1" t="s">
         <v>518</v>
       </c>
       <c r="G148" s="1" t="s">
-        <v>496</v>
+        <v>482</v>
       </c>
       <c r="H148" s="1" t="s">
-        <v>77</v>
+        <v>101</v>
       </c>
       <c r="I148" s="1" t="s">
         <v>78</v>
@@ -9884,10 +9884,10 @@
         <v>523</v>
       </c>
       <c r="C150" s="1" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
       <c r="D150" s="1" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
       <c r="E150" s="1">
         <v>150900</v>
@@ -9926,7 +9926,7 @@
         <v>529</v>
       </c>
       <c r="E151" s="1">
-        <v>846201196</v>
+        <v>213272917</v>
       </c>
       <c r="F151" s="1" t="s">
         <v>530</v>
@@ -9962,7 +9962,7 @@
         <v>529</v>
       </c>
       <c r="E152" s="1">
-        <v>213272917</v>
+        <v>153824056</v>
       </c>
       <c r="F152" s="1" t="s">
         <v>533</v>
@@ -9998,7 +9998,7 @@
         <v>529</v>
       </c>
       <c r="E153" s="1">
-        <v>153824056</v>
+        <v>846201196</v>
       </c>
       <c r="F153" s="1" t="s">
         <v>536</v>
@@ -10034,7 +10034,7 @@
         <v>529</v>
       </c>
       <c r="E154" s="1">
-        <v>1035489776</v>
+        <v>279620735</v>
       </c>
       <c r="F154" s="1" t="s">
         <v>539</v>
@@ -10106,7 +10106,7 @@
         <v>529</v>
       </c>
       <c r="E156" s="1">
-        <v>279620735</v>
+        <v>1035489776</v>
       </c>
       <c r="F156" s="1" t="s">
         <v>545</v>
@@ -10178,7 +10178,7 @@
         <v>548</v>
       </c>
       <c r="E158" s="1">
-        <v>119845265</v>
+        <v>15407872</v>
       </c>
       <c r="F158" s="1" t="s">
         <v>552</v>
@@ -10187,13 +10187,13 @@
         <v>548</v>
       </c>
       <c r="H158" s="1" t="s">
-        <v>53</v>
+        <v>129</v>
       </c>
       <c r="I158" s="1" t="s">
         <v>17</v>
       </c>
       <c r="J158" s="1" t="s">
-        <v>54</v>
+        <v>130</v>
       </c>
       <c r="K158" s="1" t="s">
         <v>19</v>
@@ -10214,7 +10214,7 @@
         <v>548</v>
       </c>
       <c r="E159" s="1">
-        <v>15407872</v>
+        <v>119845265</v>
       </c>
       <c r="F159" s="1" t="s">
         <v>554</v>
@@ -10223,13 +10223,13 @@
         <v>548</v>
       </c>
       <c r="H159" s="1" t="s">
-        <v>129</v>
+        <v>53</v>
       </c>
       <c r="I159" s="1" t="s">
         <v>17</v>
       </c>
       <c r="J159" s="1" t="s">
-        <v>130</v>
+        <v>54</v>
       </c>
       <c r="K159" s="1" t="s">
         <v>19</v>
@@ -10394,7 +10394,7 @@
         <v>556</v>
       </c>
       <c r="E164" s="1">
-        <v>22220250</v>
+        <v>933200</v>
       </c>
       <c r="F164" s="1" t="s">
         <v>569</v>
@@ -10403,7 +10403,7 @@
         <v>570</v>
       </c>
       <c r="H164" s="1" t="s">
-        <v>16</v>
+        <v>42</v>
       </c>
       <c r="I164" s="1" t="s">
         <v>17</v>
@@ -10430,7 +10430,7 @@
         <v>556</v>
       </c>
       <c r="E165" s="1">
-        <v>79464800</v>
+        <v>22220250</v>
       </c>
       <c r="F165" s="1" t="s">
         <v>573</v>
@@ -10466,7 +10466,7 @@
         <v>556</v>
       </c>
       <c r="E166" s="1">
-        <v>441700</v>
+        <v>79464800</v>
       </c>
       <c r="F166" s="1" t="s">
         <v>576</v>
@@ -10475,7 +10475,7 @@
         <v>570</v>
       </c>
       <c r="H166" s="1" t="s">
-        <v>42</v>
+        <v>16</v>
       </c>
       <c r="I166" s="1" t="s">
         <v>17</v>
@@ -10502,7 +10502,7 @@
         <v>556</v>
       </c>
       <c r="E167" s="1">
-        <v>933200</v>
+        <v>441700</v>
       </c>
       <c r="F167" s="1" t="s">
         <v>579</v>
@@ -10538,7 +10538,7 @@
         <v>556</v>
       </c>
       <c r="E168" s="1">
-        <v>100681700</v>
+        <v>219100</v>
       </c>
       <c r="F168" s="1" t="s">
         <v>582</v>
@@ -10547,7 +10547,7 @@
         <v>570</v>
       </c>
       <c r="H168" s="1" t="s">
-        <v>16</v>
+        <v>42</v>
       </c>
       <c r="I168" s="1" t="s">
         <v>17</v>
@@ -10574,7 +10574,7 @@
         <v>556</v>
       </c>
       <c r="E169" s="1">
-        <v>219100</v>
+        <v>100681700</v>
       </c>
       <c r="F169" s="1" t="s">
         <v>585</v>
@@ -10583,7 +10583,7 @@
         <v>570</v>
       </c>
       <c r="H169" s="1" t="s">
-        <v>42</v>
+        <v>16</v>
       </c>
       <c r="I169" s="1" t="s">
         <v>17</v>
@@ -10682,7 +10682,7 @@
         <v>570</v>
       </c>
       <c r="E172" s="1">
-        <v>20168600</v>
+        <v>29781850</v>
       </c>
       <c r="F172" s="1" t="s">
         <v>594</v>
@@ -10718,7 +10718,7 @@
         <v>570</v>
       </c>
       <c r="E173" s="1">
-        <v>29781850</v>
+        <v>20168600</v>
       </c>
       <c r="F173" s="1" t="s">
         <v>597</v>
@@ -11114,7 +11114,7 @@
         <v>613</v>
       </c>
       <c r="E184" s="1">
-        <v>287324950</v>
+        <v>102434200</v>
       </c>
       <c r="F184" s="1" t="s">
         <v>633</v>
@@ -11150,7 +11150,7 @@
         <v>613</v>
       </c>
       <c r="E185" s="1">
-        <v>1037129350</v>
+        <v>287324950</v>
       </c>
       <c r="F185" s="1" t="s">
         <v>636</v>
@@ -11186,7 +11186,7 @@
         <v>613</v>
       </c>
       <c r="E186" s="1">
-        <v>102434200</v>
+        <v>1037129350</v>
       </c>
       <c r="F186" s="1" t="s">
         <v>639</v>
@@ -11258,7 +11258,7 @@
         <v>613</v>
       </c>
       <c r="E188" s="1">
-        <v>204525900</v>
+        <v>751528800</v>
       </c>
       <c r="F188" s="1" t="s">
         <v>647</v>
@@ -11267,13 +11267,13 @@
         <v>646</v>
       </c>
       <c r="H188" s="1" t="s">
-        <v>648</v>
+        <v>474</v>
       </c>
       <c r="I188" s="1" t="s">
         <v>78</v>
       </c>
       <c r="J188" s="1" t="s">
-        <v>649</v>
+        <v>648</v>
       </c>
       <c r="K188" s="1" t="s">
         <v>19</v>
@@ -11285,7 +11285,7 @@
         <v>186</v>
       </c>
       <c r="B189" s="1" t="s">
-        <v>650</v>
+        <v>649</v>
       </c>
       <c r="C189" s="1" t="s">
         <v>646</v>
@@ -11294,16 +11294,16 @@
         <v>613</v>
       </c>
       <c r="E189" s="1">
-        <v>751528800</v>
+        <v>147826000</v>
       </c>
       <c r="F189" s="1" t="s">
-        <v>651</v>
+        <v>650</v>
       </c>
       <c r="G189" s="1" t="s">
         <v>646</v>
       </c>
       <c r="H189" s="1" t="s">
-        <v>474</v>
+        <v>651</v>
       </c>
       <c r="I189" s="1" t="s">
         <v>78</v>
@@ -11330,7 +11330,7 @@
         <v>613</v>
       </c>
       <c r="E190" s="1">
-        <v>147826000</v>
+        <v>204525900</v>
       </c>
       <c r="F190" s="1" t="s">
         <v>654</v>
@@ -11339,7 +11339,7 @@
         <v>646</v>
       </c>
       <c r="H190" s="1" t="s">
-        <v>648</v>
+        <v>651</v>
       </c>
       <c r="I190" s="1" t="s">
         <v>78</v>
@@ -11402,7 +11402,7 @@
         <v>613</v>
       </c>
       <c r="E192" s="1">
-        <v>267194900</v>
+        <v>93291700</v>
       </c>
       <c r="F192" s="1" t="s">
         <v>660</v>
@@ -11411,7 +11411,7 @@
         <v>646</v>
       </c>
       <c r="H192" s="1" t="s">
-        <v>648</v>
+        <v>651</v>
       </c>
       <c r="I192" s="1" t="s">
         <v>78</v>
@@ -11474,7 +11474,7 @@
         <v>613</v>
       </c>
       <c r="E194" s="1">
-        <v>93291700</v>
+        <v>267194900</v>
       </c>
       <c r="F194" s="1" t="s">
         <v>666</v>
@@ -11483,7 +11483,7 @@
         <v>646</v>
       </c>
       <c r="H194" s="1" t="s">
-        <v>648</v>
+        <v>651</v>
       </c>
       <c r="I194" s="1" t="s">
         <v>78</v>
@@ -11690,7 +11690,7 @@
         <v>669</v>
       </c>
       <c r="E200" s="1">
-        <v>261772500</v>
+        <v>91372600</v>
       </c>
       <c r="F200" s="1" t="s">
         <v>687</v>
@@ -11726,7 +11726,7 @@
         <v>669</v>
       </c>
       <c r="E201" s="1">
-        <v>91372600</v>
+        <v>261772500</v>
       </c>
       <c r="F201" s="1" t="s">
         <v>691</v>
@@ -11834,16 +11834,16 @@
         <v>669</v>
       </c>
       <c r="E204" s="1">
-        <v>679180900</v>
+        <v>144846400</v>
       </c>
       <c r="F204" s="1" t="s">
         <v>701</v>
       </c>
       <c r="G204" s="1" t="s">
-        <v>695</v>
+        <v>688</v>
       </c>
       <c r="H204" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I204" s="1" t="s">
         <v>78</v>
@@ -11870,16 +11870,16 @@
         <v>669</v>
       </c>
       <c r="E205" s="1">
-        <v>200371400</v>
+        <v>177279700</v>
       </c>
       <c r="F205" s="1" t="s">
         <v>704</v>
       </c>
       <c r="G205" s="1" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
       <c r="H205" s="1" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="I205" s="1" t="s">
         <v>78</v>
@@ -11906,16 +11906,16 @@
         <v>669</v>
       </c>
       <c r="E206" s="1">
-        <v>177279700</v>
+        <v>200371400</v>
       </c>
       <c r="F206" s="1" t="s">
         <v>707</v>
       </c>
       <c r="G206" s="1" t="s">
-        <v>695</v>
+        <v>688</v>
       </c>
       <c r="H206" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I206" s="1" t="s">
         <v>78</v>
@@ -11942,16 +11942,16 @@
         <v>669</v>
       </c>
       <c r="E207" s="1">
-        <v>144846400</v>
+        <v>679180900</v>
       </c>
       <c r="F207" s="1" t="s">
         <v>710</v>
       </c>
       <c r="G207" s="1" t="s">
-        <v>688</v>
+        <v>695</v>
       </c>
       <c r="H207" s="1" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="I207" s="1" t="s">
         <v>78</v>
@@ -11978,7 +11978,7 @@
         <v>713</v>
       </c>
       <c r="E208" s="1">
-        <v>279581387</v>
+        <v>34899150</v>
       </c>
       <c r="F208" s="1" t="s">
         <v>714</v>
@@ -11987,7 +11987,7 @@
         <v>713</v>
       </c>
       <c r="H208" s="1" t="s">
-        <v>135</v>
+        <v>25</v>
       </c>
       <c r="I208" s="1" t="s">
         <v>17</v>
@@ -12014,7 +12014,7 @@
         <v>713</v>
       </c>
       <c r="E209" s="1">
-        <v>34899150</v>
+        <v>279581387</v>
       </c>
       <c r="F209" s="1" t="s">
         <v>717</v>
@@ -12023,7 +12023,7 @@
         <v>713</v>
       </c>
       <c r="H209" s="1" t="s">
-        <v>25</v>
+        <v>135</v>
       </c>
       <c r="I209" s="1" t="s">
         <v>17</v>
@@ -12302,7 +12302,7 @@
         <v>730</v>
       </c>
       <c r="E217" s="1">
-        <v>158091056</v>
+        <v>212914412</v>
       </c>
       <c r="F217" s="1" t="s">
         <v>744</v>
@@ -12338,7 +12338,7 @@
         <v>730</v>
       </c>
       <c r="E218" s="1">
-        <v>74276700</v>
+        <v>158091056</v>
       </c>
       <c r="F218" s="1" t="s">
         <v>747</v>
@@ -12347,7 +12347,7 @@
         <v>730</v>
       </c>
       <c r="H218" s="1" t="s">
-        <v>16</v>
+        <v>135</v>
       </c>
       <c r="I218" s="1" t="s">
         <v>17</v>
@@ -12374,7 +12374,7 @@
         <v>730</v>
       </c>
       <c r="E219" s="1">
-        <v>212914412</v>
+        <v>74276700</v>
       </c>
       <c r="F219" s="1" t="s">
         <v>750</v>
@@ -12383,7 +12383,7 @@
         <v>730</v>
       </c>
       <c r="H219" s="1" t="s">
-        <v>135</v>
+        <v>16</v>
       </c>
       <c r="I219" s="1" t="s">
         <v>17</v>
@@ -12410,7 +12410,7 @@
         <v>730</v>
       </c>
       <c r="E220" s="1">
-        <v>1912000</v>
+        <v>100933077</v>
       </c>
       <c r="F220" s="1" t="s">
         <v>754</v>
@@ -12419,13 +12419,13 @@
         <v>753</v>
       </c>
       <c r="H220" s="1" t="s">
-        <v>129</v>
+        <v>53</v>
       </c>
       <c r="I220" s="1" t="s">
         <v>17</v>
       </c>
       <c r="J220" s="1" t="s">
-        <v>130</v>
+        <v>54</v>
       </c>
       <c r="K220" s="1" t="s">
         <v>19</v>
@@ -12446,7 +12446,7 @@
         <v>730</v>
       </c>
       <c r="E221" s="1">
-        <v>100933077</v>
+        <v>1912000</v>
       </c>
       <c r="F221" s="1" t="s">
         <v>756</v>
@@ -12455,13 +12455,13 @@
         <v>753</v>
       </c>
       <c r="H221" s="1" t="s">
-        <v>53</v>
+        <v>129</v>
       </c>
       <c r="I221" s="1" t="s">
         <v>17</v>
       </c>
       <c r="J221" s="1" t="s">
-        <v>54</v>
+        <v>130</v>
       </c>
       <c r="K221" s="1" t="s">
         <v>19</v>
@@ -12698,7 +12698,7 @@
         <v>688</v>
       </c>
       <c r="E228" s="1">
-        <v>337800</v>
+        <v>3160500</v>
       </c>
       <c r="F228" s="1" t="s">
         <v>778</v>
@@ -12734,7 +12734,7 @@
         <v>688</v>
       </c>
       <c r="E229" s="1">
-        <v>3160500</v>
+        <v>337800</v>
       </c>
       <c r="F229" s="1" t="s">
         <v>781</v>
@@ -13202,7 +13202,7 @@
         <v>811</v>
       </c>
       <c r="E242" s="1">
-        <v>177618600</v>
+        <v>200371400</v>
       </c>
       <c r="F242" s="1" t="s">
         <v>828</v>
@@ -13211,7 +13211,7 @@
         <v>829</v>
       </c>
       <c r="H242" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I242" s="1" t="s">
         <v>78</v>
@@ -13274,7 +13274,7 @@
         <v>811</v>
       </c>
       <c r="E244" s="1">
-        <v>200371400</v>
+        <v>688714100</v>
       </c>
       <c r="F244" s="1" t="s">
         <v>835</v>
@@ -13283,7 +13283,7 @@
         <v>829</v>
       </c>
       <c r="H244" s="1" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="I244" s="1" t="s">
         <v>78</v>
@@ -13310,7 +13310,7 @@
         <v>811</v>
       </c>
       <c r="E245" s="1">
-        <v>688714100</v>
+        <v>177618600</v>
       </c>
       <c r="F245" s="1" t="s">
         <v>838</v>
@@ -13526,7 +13526,7 @@
         <v>853</v>
       </c>
       <c r="E251" s="1">
-        <v>845082696</v>
+        <v>158436845</v>
       </c>
       <c r="F251" s="1" t="s">
         <v>857</v>
@@ -13562,7 +13562,7 @@
         <v>853</v>
       </c>
       <c r="E252" s="1">
-        <v>158436845</v>
+        <v>845082696</v>
       </c>
       <c r="F252" s="1" t="s">
         <v>860</v>
@@ -13634,7 +13634,7 @@
         <v>853</v>
       </c>
       <c r="E254" s="1">
-        <v>1055833082</v>
+        <v>99929015</v>
       </c>
       <c r="F254" s="1" t="s">
         <v>866</v>
@@ -13670,7 +13670,7 @@
         <v>853</v>
       </c>
       <c r="E255" s="1">
-        <v>99929015</v>
+        <v>1055833082</v>
       </c>
       <c r="F255" s="1" t="s">
         <v>869</v>
@@ -13958,7 +13958,7 @@
         <v>885</v>
       </c>
       <c r="E263" s="1">
-        <v>90092300</v>
+        <v>24294250</v>
       </c>
       <c r="F263" s="1" t="s">
         <v>895</v>
@@ -14066,7 +14066,7 @@
         <v>885</v>
       </c>
       <c r="E266" s="1">
-        <v>24294250</v>
+        <v>90092300</v>
       </c>
       <c r="F266" s="1" t="s">
         <v>904</v>
@@ -14462,7 +14462,7 @@
         <v>937</v>
       </c>
       <c r="E277" s="1">
-        <v>2548731</v>
+        <v>258570562</v>
       </c>
       <c r="F277" s="1" t="s">
         <v>944</v>
@@ -14534,7 +14534,7 @@
         <v>937</v>
       </c>
       <c r="E279" s="1">
-        <v>258570562</v>
+        <v>2548731</v>
       </c>
       <c r="F279" s="1" t="s">
         <v>950</v>
@@ -14606,7 +14606,7 @@
         <v>937</v>
       </c>
       <c r="E281" s="1">
-        <v>200371400</v>
+        <v>177359200</v>
       </c>
       <c r="F281" s="1" t="s">
         <v>956</v>
@@ -14615,7 +14615,7 @@
         <v>957</v>
       </c>
       <c r="H281" s="1" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="I281" s="1" t="s">
         <v>78</v>
@@ -14642,7 +14642,7 @@
         <v>937</v>
       </c>
       <c r="E282" s="1">
-        <v>149250700</v>
+        <v>689018800</v>
       </c>
       <c r="F282" s="1" t="s">
         <v>960</v>
@@ -14651,7 +14651,7 @@
         <v>957</v>
       </c>
       <c r="H282" s="1" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="I282" s="1" t="s">
         <v>78</v>
@@ -14678,7 +14678,7 @@
         <v>937</v>
       </c>
       <c r="E283" s="1">
-        <v>689018800</v>
+        <v>200371400</v>
       </c>
       <c r="F283" s="1" t="s">
         <v>963</v>
@@ -14687,7 +14687,7 @@
         <v>957</v>
       </c>
       <c r="H283" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I283" s="1" t="s">
         <v>78</v>
@@ -14714,7 +14714,7 @@
         <v>937</v>
       </c>
       <c r="E284" s="1">
-        <v>177359200</v>
+        <v>149250700</v>
       </c>
       <c r="F284" s="1" t="s">
         <v>966</v>
@@ -14723,7 +14723,7 @@
         <v>957</v>
       </c>
       <c r="H284" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I284" s="1" t="s">
         <v>78</v>
@@ -15326,7 +15326,7 @@
         <v>1010</v>
       </c>
       <c r="E301" s="1">
-        <v>703000</v>
+        <v>667850</v>
       </c>
       <c r="F301" s="1" t="s">
         <v>1024</v>
@@ -15362,7 +15362,7 @@
         <v>1010</v>
       </c>
       <c r="E302" s="1">
-        <v>667850</v>
+        <v>287324950</v>
       </c>
       <c r="F302" s="1" t="s">
         <v>1027</v>
@@ -15371,7 +15371,7 @@
         <v>1015</v>
       </c>
       <c r="H302" s="1" t="s">
-        <v>16</v>
+        <v>929</v>
       </c>
       <c r="I302" s="1" t="s">
         <v>17</v>
@@ -15398,7 +15398,7 @@
         <v>1010</v>
       </c>
       <c r="E303" s="1">
-        <v>287324950</v>
+        <v>703000</v>
       </c>
       <c r="F303" s="1" t="s">
         <v>1030</v>
@@ -15407,7 +15407,7 @@
         <v>1015</v>
       </c>
       <c r="H303" s="1" t="s">
-        <v>929</v>
+        <v>16</v>
       </c>
       <c r="I303" s="1" t="s">
         <v>17</v>
@@ -15578,7 +15578,7 @@
         <v>1015</v>
       </c>
       <c r="E308" s="1">
-        <v>960197300</v>
+        <v>267194900</v>
       </c>
       <c r="F308" s="1" t="s">
         <v>1048</v>
@@ -15587,7 +15587,7 @@
         <v>1044</v>
       </c>
       <c r="H308" s="1" t="s">
-        <v>1045</v>
+        <v>933</v>
       </c>
       <c r="I308" s="1" t="s">
         <v>78</v>
@@ -15614,7 +15614,7 @@
         <v>1015</v>
       </c>
       <c r="E309" s="1">
-        <v>267194900</v>
+        <v>960197300</v>
       </c>
       <c r="F309" s="1" t="s">
         <v>1051</v>
@@ -15623,7 +15623,7 @@
         <v>1044</v>
       </c>
       <c r="H309" s="1" t="s">
-        <v>933</v>
+        <v>1045</v>
       </c>
       <c r="I309" s="1" t="s">
         <v>78</v>
@@ -15650,7 +15650,7 @@
         <v>1015</v>
       </c>
       <c r="E310" s="1">
-        <v>4313300</v>
+        <v>762330900</v>
       </c>
       <c r="F310" s="1" t="s">
         <v>1054</v>
@@ -15686,7 +15686,7 @@
         <v>1015</v>
       </c>
       <c r="E311" s="1">
-        <v>193894600</v>
+        <v>4313300</v>
       </c>
       <c r="F311" s="1" t="s">
         <v>1057</v>
@@ -15722,7 +15722,7 @@
         <v>1015</v>
       </c>
       <c r="E312" s="1">
-        <v>762330900</v>
+        <v>63500000</v>
       </c>
       <c r="F312" s="1" t="s">
         <v>1060</v>
@@ -15731,7 +15731,7 @@
         <v>1044</v>
       </c>
       <c r="H312" s="1" t="s">
-        <v>1045</v>
+        <v>995</v>
       </c>
       <c r="I312" s="1" t="s">
         <v>78</v>
@@ -15758,7 +15758,7 @@
         <v>1015</v>
       </c>
       <c r="E313" s="1">
-        <v>63500000</v>
+        <v>151924700</v>
       </c>
       <c r="F313" s="1" t="s">
         <v>1063</v>
@@ -15767,7 +15767,7 @@
         <v>1044</v>
       </c>
       <c r="H313" s="1" t="s">
-        <v>995</v>
+        <v>933</v>
       </c>
       <c r="I313" s="1" t="s">
         <v>78</v>
@@ -15794,7 +15794,7 @@
         <v>1015</v>
       </c>
       <c r="E314" s="1">
-        <v>204133200</v>
+        <v>193894600</v>
       </c>
       <c r="F314" s="1" t="s">
         <v>1066</v>
@@ -15803,7 +15803,7 @@
         <v>1044</v>
       </c>
       <c r="H314" s="1" t="s">
-        <v>933</v>
+        <v>1045</v>
       </c>
       <c r="I314" s="1" t="s">
         <v>78</v>
@@ -15830,7 +15830,7 @@
         <v>1015</v>
       </c>
       <c r="E315" s="1">
-        <v>151924700</v>
+        <v>204133200</v>
       </c>
       <c r="F315" s="1" t="s">
         <v>1069</v>
@@ -16046,7 +16046,7 @@
         <v>1072</v>
       </c>
       <c r="E321" s="1">
-        <v>1067934069</v>
+        <v>5246000</v>
       </c>
       <c r="F321" s="1" t="s">
         <v>1088</v>
@@ -16055,13 +16055,13 @@
         <v>957</v>
       </c>
       <c r="H321" s="1" t="s">
-        <v>135</v>
+        <v>1089</v>
       </c>
       <c r="I321" s="1" t="s">
         <v>17</v>
       </c>
       <c r="J321" s="1" t="s">
-        <v>1089</v>
+        <v>1090</v>
       </c>
       <c r="K321" s="1" t="s">
         <v>19</v>
@@ -16073,7 +16073,7 @@
         <v>319</v>
       </c>
       <c r="B322" s="1" t="s">
-        <v>1090</v>
+        <v>1091</v>
       </c>
       <c r="C322" s="1" t="s">
         <v>1072</v>
@@ -16082,16 +16082,16 @@
         <v>1072</v>
       </c>
       <c r="E322" s="1">
-        <v>5246000</v>
+        <v>1067934069</v>
       </c>
       <c r="F322" s="1" t="s">
-        <v>1091</v>
+        <v>1092</v>
       </c>
       <c r="G322" s="1" t="s">
         <v>957</v>
       </c>
       <c r="H322" s="1" t="s">
-        <v>1092</v>
+        <v>135</v>
       </c>
       <c r="I322" s="1" t="s">
         <v>17</v>
@@ -16118,7 +16118,7 @@
         <v>1072</v>
       </c>
       <c r="E323" s="1">
-        <v>25170300</v>
+        <v>94750900</v>
       </c>
       <c r="F323" s="1" t="s">
         <v>1095</v>
@@ -16190,7 +16190,7 @@
         <v>1072</v>
       </c>
       <c r="E325" s="1">
-        <v>94750900</v>
+        <v>25170300</v>
       </c>
       <c r="F325" s="1" t="s">
         <v>1101</v>
@@ -16298,7 +16298,7 @@
         <v>1072</v>
       </c>
       <c r="E328" s="1">
-        <v>279548291</v>
+        <v>44072100</v>
       </c>
       <c r="F328" s="1" t="s">
         <v>1110</v>
@@ -16307,7 +16307,7 @@
         <v>957</v>
       </c>
       <c r="H328" s="1" t="s">
-        <v>135</v>
+        <v>25</v>
       </c>
       <c r="I328" s="1" t="s">
         <v>17</v>
@@ -16334,7 +16334,7 @@
         <v>1072</v>
       </c>
       <c r="E329" s="1">
-        <v>44072100</v>
+        <v>279548291</v>
       </c>
       <c r="F329" s="1" t="s">
         <v>1113</v>
@@ -16343,7 +16343,7 @@
         <v>957</v>
       </c>
       <c r="H329" s="1" t="s">
-        <v>25</v>
+        <v>135</v>
       </c>
       <c r="I329" s="1" t="s">
         <v>17</v>
@@ -16523,7 +16523,7 @@
         <v>1121</v>
       </c>
       <c r="H334" s="1" t="s">
-        <v>1092</v>
+        <v>1089</v>
       </c>
       <c r="I334" s="1" t="s">
         <v>17</v>
@@ -16766,7 +16766,7 @@
         <v>1154</v>
       </c>
       <c r="E341" s="1">
-        <v>279584469</v>
+        <v>116066650</v>
       </c>
       <c r="F341" s="1" t="s">
         <v>1155</v>
@@ -16775,7 +16775,7 @@
         <v>1153</v>
       </c>
       <c r="H341" s="1" t="s">
-        <v>135</v>
+        <v>16</v>
       </c>
       <c r="I341" s="1" t="s">
         <v>17</v>
@@ -16838,7 +16838,7 @@
         <v>1154</v>
       </c>
       <c r="E343" s="1">
-        <v>41365850</v>
+        <v>279584469</v>
       </c>
       <c r="F343" s="1" t="s">
         <v>1161</v>
@@ -16847,7 +16847,7 @@
         <v>1153</v>
       </c>
       <c r="H343" s="1" t="s">
-        <v>25</v>
+        <v>135</v>
       </c>
       <c r="I343" s="1" t="s">
         <v>17</v>
@@ -16874,7 +16874,7 @@
         <v>1154</v>
       </c>
       <c r="E344" s="1">
-        <v>116066650</v>
+        <v>41365850</v>
       </c>
       <c r="F344" s="1" t="s">
         <v>1164</v>
@@ -16883,7 +16883,7 @@
         <v>1153</v>
       </c>
       <c r="H344" s="1" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="I344" s="1" t="s">
         <v>17</v>
@@ -17054,22 +17054,22 @@
         <v>1168</v>
       </c>
       <c r="E349" s="1">
-        <v>149250700</v>
+        <v>177151200</v>
       </c>
       <c r="F349" s="1" t="s">
         <v>1183</v>
       </c>
       <c r="G349" s="1" t="s">
-        <v>1184</v>
+        <v>1180</v>
       </c>
       <c r="H349" s="1" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="I349" s="1" t="s">
         <v>78</v>
       </c>
       <c r="J349" s="1" t="s">
-        <v>1185</v>
+        <v>1184</v>
       </c>
       <c r="K349" s="1" t="s">
         <v>19</v>
@@ -17081,7 +17081,7 @@
         <v>347</v>
       </c>
       <c r="B350" s="1" t="s">
-        <v>1186</v>
+        <v>1185</v>
       </c>
       <c r="C350" s="1" t="s">
         <v>1170</v>
@@ -17090,16 +17090,16 @@
         <v>1168</v>
       </c>
       <c r="E350" s="1">
-        <v>689692300</v>
+        <v>149250700</v>
       </c>
       <c r="F350" s="1" t="s">
+        <v>1186</v>
+      </c>
+      <c r="G350" s="1" t="s">
         <v>1187</v>
       </c>
-      <c r="G350" s="1" t="s">
-        <v>1180</v>
-      </c>
       <c r="H350" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I350" s="1" t="s">
         <v>78</v>
@@ -17162,22 +17162,22 @@
         <v>1168</v>
       </c>
       <c r="E352" s="1">
-        <v>177151200</v>
+        <v>62679696</v>
       </c>
       <c r="F352" s="1" t="s">
         <v>1193</v>
       </c>
       <c r="G352" s="1" t="s">
-        <v>1180</v>
+        <v>1194</v>
       </c>
       <c r="H352" s="1" t="s">
-        <v>97</v>
+        <v>77</v>
       </c>
       <c r="I352" s="1" t="s">
         <v>78</v>
       </c>
       <c r="J352" s="1" t="s">
-        <v>1194</v>
+        <v>1195</v>
       </c>
       <c r="K352" s="1" t="s">
         <v>19</v>
@@ -17189,7 +17189,7 @@
         <v>350</v>
       </c>
       <c r="B353" s="1" t="s">
-        <v>1195</v>
+        <v>1196</v>
       </c>
       <c r="C353" s="1" t="s">
         <v>1170</v>
@@ -17198,16 +17198,16 @@
         <v>1168</v>
       </c>
       <c r="E353" s="1">
-        <v>62679696</v>
+        <v>689692300</v>
       </c>
       <c r="F353" s="1" t="s">
-        <v>1196</v>
+        <v>1197</v>
       </c>
       <c r="G353" s="1" t="s">
-        <v>1197</v>
+        <v>1180</v>
       </c>
       <c r="H353" s="1" t="s">
-        <v>77</v>
+        <v>97</v>
       </c>
       <c r="I353" s="1" t="s">
         <v>78</v>
@@ -17240,7 +17240,7 @@
         <v>1200</v>
       </c>
       <c r="G354" s="1" t="s">
-        <v>1184</v>
+        <v>1187</v>
       </c>
       <c r="H354" s="1" t="s">
         <v>101</v>
@@ -17267,7 +17267,7 @@
         <v>1203</v>
       </c>
       <c r="D355" s="1" t="s">
-        <v>1197</v>
+        <v>1194</v>
       </c>
       <c r="E355" s="1">
         <v>258570562</v>
@@ -17303,7 +17303,7 @@
         <v>1180</v>
       </c>
       <c r="D356" s="1" t="s">
-        <v>1184</v>
+        <v>1187</v>
       </c>
       <c r="E356" s="1">
         <v>837896759</v>
@@ -17339,10 +17339,10 @@
         <v>1180</v>
       </c>
       <c r="D357" s="1" t="s">
-        <v>1184</v>
+        <v>1187</v>
       </c>
       <c r="E357" s="1">
-        <v>158575478</v>
+        <v>213243288</v>
       </c>
       <c r="F357" s="1" t="s">
         <v>1210</v>
@@ -17375,10 +17375,10 @@
         <v>1180</v>
       </c>
       <c r="D358" s="1" t="s">
-        <v>1184</v>
+        <v>1187</v>
       </c>
       <c r="E358" s="1">
-        <v>213243288</v>
+        <v>158575478</v>
       </c>
       <c r="F358" s="1" t="s">
         <v>1213</v>
@@ -17414,7 +17414,7 @@
         <v>1180</v>
       </c>
       <c r="E359" s="1">
-        <v>24034050</v>
+        <v>22608400</v>
       </c>
       <c r="F359" s="1" t="s">
         <v>1217</v>
@@ -17423,7 +17423,7 @@
         <v>1218</v>
       </c>
       <c r="H359" s="1" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="I359" s="1" t="s">
         <v>17</v>
@@ -17450,7 +17450,7 @@
         <v>1180</v>
       </c>
       <c r="E360" s="1">
-        <v>22608400</v>
+        <v>24034050</v>
       </c>
       <c r="F360" s="1" t="s">
         <v>1221</v>
@@ -17459,7 +17459,7 @@
         <v>1218</v>
       </c>
       <c r="H360" s="1" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="I360" s="1" t="s">
         <v>17</v>
@@ -17522,16 +17522,16 @@
         <v>1180</v>
       </c>
       <c r="E362" s="1">
-        <v>33188550</v>
+        <v>89459600</v>
       </c>
       <c r="F362" s="1" t="s">
         <v>1228</v>
       </c>
       <c r="G362" s="1" t="s">
-        <v>1218</v>
+        <v>1224</v>
       </c>
       <c r="H362" s="1" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="I362" s="1" t="s">
         <v>17</v>
@@ -17558,16 +17558,16 @@
         <v>1180</v>
       </c>
       <c r="E363" s="1">
-        <v>89459600</v>
+        <v>33188550</v>
       </c>
       <c r="F363" s="1" t="s">
         <v>1231</v>
       </c>
       <c r="G363" s="1" t="s">
-        <v>1224</v>
+        <v>1218</v>
       </c>
       <c r="H363" s="1" t="s">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="I363" s="1" t="s">
         <v>17</v>
@@ -17699,7 +17699,7 @@
         <v>1242</v>
       </c>
       <c r="D367" s="1" t="s">
-        <v>1184</v>
+        <v>1187</v>
       </c>
       <c r="E367" s="1">
         <v>60825925</v>
@@ -17735,7 +17735,7 @@
         <v>1242</v>
       </c>
       <c r="D368" s="1" t="s">
-        <v>1184</v>
+        <v>1187</v>
       </c>
       <c r="E368" s="1">
         <v>2844264</v>
@@ -17774,7 +17774,7 @@
         <v>1242</v>
       </c>
       <c r="E369" s="1">
-        <v>12740000</v>
+        <v>34511892</v>
       </c>
       <c r="F369" s="1" t="s">
         <v>1250</v>
@@ -17810,7 +17810,7 @@
         <v>1242</v>
       </c>
       <c r="E370" s="1">
-        <v>34511892</v>
+        <v>12740000</v>
       </c>
       <c r="F370" s="1" t="s">
         <v>1253</v>
@@ -18206,7 +18206,7 @@
         <v>1289</v>
       </c>
       <c r="E381" s="1">
-        <v>161741108</v>
+        <v>3915950</v>
       </c>
       <c r="F381" s="1" t="s">
         <v>1293</v>
@@ -18242,7 +18242,7 @@
         <v>1289</v>
       </c>
       <c r="E382" s="1">
-        <v>3915950</v>
+        <v>161741108</v>
       </c>
       <c r="F382" s="1" t="s">
         <v>1296</v>
@@ -18314,7 +18314,7 @@
         <v>1284</v>
       </c>
       <c r="E384" s="1">
-        <v>3915950</v>
+        <v>679200</v>
       </c>
       <c r="F384" s="1" t="s">
         <v>1302</v>
@@ -18323,7 +18323,7 @@
         <v>1288</v>
       </c>
       <c r="H384" s="1" t="s">
-        <v>135</v>
+        <v>803</v>
       </c>
       <c r="I384" s="1" t="s">
         <v>17</v>
@@ -18350,7 +18350,7 @@
         <v>1284</v>
       </c>
       <c r="E385" s="1">
-        <v>679200</v>
+        <v>3915950</v>
       </c>
       <c r="F385" s="1" t="s">
         <v>1305</v>
@@ -18359,7 +18359,7 @@
         <v>1288</v>
       </c>
       <c r="H385" s="1" t="s">
-        <v>803</v>
+        <v>135</v>
       </c>
       <c r="I385" s="1" t="s">
         <v>17</v>
@@ -18422,7 +18422,7 @@
         <v>1312</v>
       </c>
       <c r="E387" s="1">
-        <v>4759600</v>
+        <v>346500</v>
       </c>
       <c r="F387" s="1" t="s">
         <v>1313</v>
@@ -18431,7 +18431,7 @@
         <v>1308</v>
       </c>
       <c r="H387" s="1" t="s">
-        <v>1092</v>
+        <v>42</v>
       </c>
       <c r="I387" s="1" t="s">
         <v>17</v>
@@ -18458,7 +18458,7 @@
         <v>1312</v>
       </c>
       <c r="E388" s="1">
-        <v>346500</v>
+        <v>4759600</v>
       </c>
       <c r="F388" s="1" t="s">
         <v>1316</v>
@@ -18467,7 +18467,7 @@
         <v>1308</v>
       </c>
       <c r="H388" s="1" t="s">
-        <v>42</v>
+        <v>1089</v>
       </c>
       <c r="I388" s="1" t="s">
         <v>17</v>
@@ -18566,22 +18566,22 @@
         <v>1289</v>
       </c>
       <c r="E391" s="1">
-        <v>694524200</v>
+        <v>199981800</v>
       </c>
       <c r="F391" s="1" t="s">
         <v>1327</v>
       </c>
       <c r="G391" s="1" t="s">
-        <v>1328</v>
+        <v>1324</v>
       </c>
       <c r="H391" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="I391" s="1" t="s">
         <v>78</v>
       </c>
       <c r="J391" s="1" t="s">
-        <v>1329</v>
+        <v>1328</v>
       </c>
       <c r="K391" s="1" t="s">
         <v>19</v>
@@ -18593,7 +18593,7 @@
         <v>389</v>
       </c>
       <c r="B392" s="1" t="s">
-        <v>1330</v>
+        <v>1329</v>
       </c>
       <c r="C392" s="1" t="s">
         <v>1322</v>
@@ -18605,10 +18605,10 @@
         <v>176866300</v>
       </c>
       <c r="F392" s="1" t="s">
+        <v>1330</v>
+      </c>
+      <c r="G392" s="1" t="s">
         <v>1331</v>
-      </c>
-      <c r="G392" s="1" t="s">
-        <v>1328</v>
       </c>
       <c r="H392" s="1" t="s">
         <v>97</v>
@@ -18638,16 +18638,16 @@
         <v>1289</v>
       </c>
       <c r="E393" s="1">
-        <v>199981800</v>
+        <v>694524200</v>
       </c>
       <c r="F393" s="1" t="s">
         <v>1334</v>
       </c>
       <c r="G393" s="1" t="s">
-        <v>1324</v>
+        <v>1331</v>
       </c>
       <c r="H393" s="1" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="I393" s="1" t="s">
         <v>78</v>
@@ -18680,7 +18680,7 @@
         <v>1337</v>
       </c>
       <c r="G394" s="1" t="s">
-        <v>1328</v>
+        <v>1331</v>
       </c>
       <c r="H394" s="1" t="s">
         <v>97</v>
@@ -18752,7 +18752,7 @@
         <v>1343</v>
       </c>
       <c r="G396" s="1" t="s">
-        <v>1328</v>
+        <v>1331</v>
       </c>
       <c r="H396" s="1" t="s">
         <v>97</v>
@@ -18788,7 +18788,7 @@
         <v>1348</v>
       </c>
       <c r="G397" s="1" t="s">
-        <v>1328</v>
+        <v>1331</v>
       </c>
       <c r="H397" s="1" t="s">
         <v>17</v>
@@ -18818,7 +18818,7 @@
         <v>1352</v>
       </c>
       <c r="E398" s="1">
-        <v>4759600</v>
+        <v>120000000</v>
       </c>
       <c r="F398" s="1" t="s">
         <v>1353</v>
@@ -18827,13 +18827,13 @@
         <v>1351</v>
       </c>
       <c r="H398" s="1" t="s">
-        <v>1092</v>
+        <v>1354</v>
       </c>
       <c r="I398" s="1" t="s">
         <v>17</v>
       </c>
       <c r="J398" s="1" t="s">
-        <v>1354</v>
+        <v>1355</v>
       </c>
       <c r="K398" s="1" t="s">
         <v>19</v>
@@ -18845,7 +18845,7 @@
         <v>396</v>
       </c>
       <c r="B399" s="1" t="s">
-        <v>1355</v>
+        <v>1356</v>
       </c>
       <c r="C399" s="1" t="s">
         <v>1351</v>
@@ -18854,16 +18854,16 @@
         <v>1352</v>
       </c>
       <c r="E399" s="1">
-        <v>120000000</v>
+        <v>4759600</v>
       </c>
       <c r="F399" s="1" t="s">
-        <v>1356</v>
+        <v>1357</v>
       </c>
       <c r="G399" s="1" t="s">
         <v>1351</v>
       </c>
       <c r="H399" s="1" t="s">
-        <v>1357</v>
+        <v>1089</v>
       </c>
       <c r="I399" s="1" t="s">
         <v>17</v>

</xml_diff>